<commit_message>
Phase 1-4 Complete: Removed KM meter, fixed mobile UI, added Target Management, and fixed Excel formulas & totals
</commit_message>
<xml_diff>
--- a/templates/template_Aurangabad.xlsx
+++ b/templates/template_Aurangabad.xlsx
@@ -108,12 +108,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -965,7 +966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1167,6 +1168,37 @@
       </c>
       <c r="I5" s="2">
         <f>'CONSOLIDATED SHEET'!H5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="D6" s="3">
+        <f>SUM(D2:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="3">
+        <f>SUM(E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="3">
+        <f>SUM(F2:F5)</f>
+        <v/>
+      </c>
+      <c r="G6" s="3">
+        <f>SUM(G2:G5)</f>
+        <v/>
+      </c>
+      <c r="H6" s="3">
+        <f>SUM(H2:H5)</f>
+        <v/>
+      </c>
+      <c r="I6" s="3">
+        <f>SUM(I2:I5)</f>
         <v/>
       </c>
     </row>
@@ -3259,22 +3291,22 @@
           <t>Consent with ID</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>Prince Kumar</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>Rahul Kumar</t>
         </is>
       </c>
-      <c r="AG1" s="3" t="inlineStr">
+      <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>Ram Ji Singh</t>
         </is>
       </c>
-      <c r="AL1" s="3" t="inlineStr">
+      <c r="AL1" s="4" t="inlineStr">
         <is>
           <t>Rishu Kumar</t>
         </is>
@@ -3292,157 +3324,157 @@
         </is>
       </c>
       <c r="C2" s="2">
-        <f>COUNTA('1ST'!C2:C41)+COUNTA('2nd'!C2:C41)+COUNTA('3rd'!C2:C41)+COUNTA('4th'!C2:C41)+COUNTA('5th'!C2:C41)+COUNTA('6th'!C2:C41)+COUNTA('7th'!C2:C41)+COUNTA('8th'!C2:C41)+COUNTA('9th'!C2:C41)+COUNTA('10th'!C2:C41)+COUNTA('11th'!C2:C41)+COUNTA('12th'!C2:C41)+COUNTA('13th'!C2:C41)+COUNTA('14th'!C2:C41)+COUNTA('15th'!C2:C41)+COUNTA('16th'!C2:C41)+COUNTA('17th'!C2:C41)+COUNTA('18th'!C2:C41)+COUNTA('19th'!C2:C41)+COUNTA('20th'!C2:C41)+COUNTA('21st'!C2:C41)+COUNTA('22nd'!C2:C41)+COUNTA('23rd'!C2:C41)+COUNTA('24th'!C2:C41)+COUNTA('25th'!C2:C41)+COUNTA('26th'!C2:C41)+COUNTA('27th'!C2:C41)+COUNTA('28th'!C2:C41)+COUNTA('29th'!C2:C41)+COUNTA('30th'!C2:C41)+COUNTA('31st'!C2:C41)</f>
+        <f>(COUNTA('1ST'!C2:C41)+COUNTA('2nd'!C2:C41)+COUNTA('3rd'!C2:C41)+COUNTA('4th'!C2:C41)+COUNTA('5th'!C2:C41)+COUNTA('6th'!C2:C41)+COUNTA('7th'!C2:C41)+COUNTA('8th'!C2:C41)+COUNTA('9th'!C2:C41)+COUNTA('10th'!C2:C41)+COUNTA('11th'!C2:C41)+COUNTA('12th'!C2:C41)+COUNTA('13th'!C2:C41)+COUNTA('14th'!C2:C41)+COUNTA('15th'!C2:C41)+COUNTA('16th'!C2:C41)+COUNTA('17th'!C2:C41)+COUNTA('18th'!C2:C41)+COUNTA('19th'!C2:C41)+COUNTA('20th'!C2:C41)+COUNTA('21st'!C2:C41)+COUNTA('22nd'!C2:C41)+COUNTA('23rd'!C2:C41)+COUNTA('24th'!C2:C41)+COUNTA('25th'!C2:C41)+COUNTA('26th'!C2:C41)+COUNTA('27th'!C2:C41)+COUNTA('28th'!C2:C41)+COUNTA('29th'!C2:C41)+COUNTA('30th'!C2:C41)+COUNTA('31st'!C2:C41))+0</f>
         <v/>
       </c>
       <c r="D2" s="2">
-        <f>COUNTA('1ST'!D2:D41)+COUNTA('2nd'!D2:D41)+COUNTA('3rd'!D2:D41)+COUNTA('4th'!D2:D41)+COUNTA('5th'!D2:D41)+COUNTA('6th'!D2:D41)+COUNTA('7th'!D2:D41)+COUNTA('8th'!D2:D41)+COUNTA('9th'!D2:D41)+COUNTA('10th'!D2:D41)+COUNTA('11th'!D2:D41)+COUNTA('12th'!D2:D41)+COUNTA('13th'!D2:D41)+COUNTA('14th'!D2:D41)+COUNTA('15th'!D2:D41)+COUNTA('16th'!D2:D41)+COUNTA('17th'!D2:D41)+COUNTA('18th'!D2:D41)+COUNTA('19th'!D2:D41)+COUNTA('20th'!D2:D41)+COUNTA('21st'!D2:D41)+COUNTA('22nd'!D2:D41)+COUNTA('23rd'!D2:D41)+COUNTA('24th'!D2:D41)+COUNTA('25th'!D2:D41)+COUNTA('26th'!D2:D41)+COUNTA('27th'!D2:D41)+COUNTA('28th'!D2:D41)+COUNTA('29th'!D2:D41)+COUNTA('30th'!D2:D41)+COUNTA('31st'!D2:D41)</f>
+        <f>(COUNTA('1ST'!D2:D41)+COUNTA('2nd'!D2:D41)+COUNTA('3rd'!D2:D41)+COUNTA('4th'!D2:D41)+COUNTA('5th'!D2:D41)+COUNTA('6th'!D2:D41)+COUNTA('7th'!D2:D41)+COUNTA('8th'!D2:D41)+COUNTA('9th'!D2:D41)+COUNTA('10th'!D2:D41)+COUNTA('11th'!D2:D41)+COUNTA('12th'!D2:D41)+COUNTA('13th'!D2:D41)+COUNTA('14th'!D2:D41)+COUNTA('15th'!D2:D41)+COUNTA('16th'!D2:D41)+COUNTA('17th'!D2:D41)+COUNTA('18th'!D2:D41)+COUNTA('19th'!D2:D41)+COUNTA('20th'!D2:D41)+COUNTA('21st'!D2:D41)+COUNTA('22nd'!D2:D41)+COUNTA('23rd'!D2:D41)+COUNTA('24th'!D2:D41)+COUNTA('25th'!D2:D41)+COUNTA('26th'!D2:D41)+COUNTA('27th'!D2:D41)+COUNTA('28th'!D2:D41)+COUNTA('29th'!D2:D41)+COUNTA('30th'!D2:D41)+COUNTA('31st'!D2:D41))+0</f>
         <v/>
       </c>
       <c r="E2" s="2">
-        <f>COUNTA('1ST'!E2:E41)+COUNTA('2nd'!E2:E41)+COUNTA('3rd'!E2:E41)+COUNTA('4th'!E2:E41)+COUNTA('5th'!E2:E41)+COUNTA('6th'!E2:E41)+COUNTA('7th'!E2:E41)+COUNTA('8th'!E2:E41)+COUNTA('9th'!E2:E41)+COUNTA('10th'!E2:E41)+COUNTA('11th'!E2:E41)+COUNTA('12th'!E2:E41)+COUNTA('13th'!E2:E41)+COUNTA('14th'!E2:E41)+COUNTA('15th'!E2:E41)+COUNTA('16th'!E2:E41)+COUNTA('17th'!E2:E41)+COUNTA('18th'!E2:E41)+COUNTA('19th'!E2:E41)+COUNTA('20th'!E2:E41)+COUNTA('21st'!E2:E41)+COUNTA('22nd'!E2:E41)+COUNTA('23rd'!E2:E41)+COUNTA('24th'!E2:E41)+COUNTA('25th'!E2:E41)+COUNTA('26th'!E2:E41)+COUNTA('27th'!E2:E41)+COUNTA('28th'!E2:E41)+COUNTA('29th'!E2:E41)+COUNTA('30th'!E2:E41)+COUNTA('31st'!E2:E41)</f>
+        <f>(COUNTA('1ST'!E2:E41)+COUNTA('2nd'!E2:E41)+COUNTA('3rd'!E2:E41)+COUNTA('4th'!E2:E41)+COUNTA('5th'!E2:E41)+COUNTA('6th'!E2:E41)+COUNTA('7th'!E2:E41)+COUNTA('8th'!E2:E41)+COUNTA('9th'!E2:E41)+COUNTA('10th'!E2:E41)+COUNTA('11th'!E2:E41)+COUNTA('12th'!E2:E41)+COUNTA('13th'!E2:E41)+COUNTA('14th'!E2:E41)+COUNTA('15th'!E2:E41)+COUNTA('16th'!E2:E41)+COUNTA('17th'!E2:E41)+COUNTA('18th'!E2:E41)+COUNTA('19th'!E2:E41)+COUNTA('20th'!E2:E41)+COUNTA('21st'!E2:E41)+COUNTA('22nd'!E2:E41)+COUNTA('23rd'!E2:E41)+COUNTA('24th'!E2:E41)+COUNTA('25th'!E2:E41)+COUNTA('26th'!E2:E41)+COUNTA('27th'!E2:E41)+COUNTA('28th'!E2:E41)+COUNTA('29th'!E2:E41)+COUNTA('30th'!E2:E41)+COUNTA('31st'!E2:E41))+0</f>
         <v/>
       </c>
       <c r="F2" s="2">
-        <f>COUNTA('1ST'!F2:F41)+COUNTA('2nd'!F2:F41)+COUNTA('3rd'!F2:F41)+COUNTA('4th'!F2:F41)+COUNTA('5th'!F2:F41)+COUNTA('6th'!F2:F41)+COUNTA('7th'!F2:F41)+COUNTA('8th'!F2:F41)+COUNTA('9th'!F2:F41)+COUNTA('10th'!F2:F41)+COUNTA('11th'!F2:F41)+COUNTA('12th'!F2:F41)+COUNTA('13th'!F2:F41)+COUNTA('14th'!F2:F41)+COUNTA('15th'!F2:F41)+COUNTA('16th'!F2:F41)+COUNTA('17th'!F2:F41)+COUNTA('18th'!F2:F41)+COUNTA('19th'!F2:F41)+COUNTA('20th'!F2:F41)+COUNTA('21st'!F2:F41)+COUNTA('22nd'!F2:F41)+COUNTA('23rd'!F2:F41)+COUNTA('24th'!F2:F41)+COUNTA('25th'!F2:F41)+COUNTA('26th'!F2:F41)+COUNTA('27th'!F2:F41)+COUNTA('28th'!F2:F41)+COUNTA('29th'!F2:F41)+COUNTA('30th'!F2:F41)+COUNTA('31st'!F2:F41)</f>
+        <f>(COUNTA('1ST'!F2:F41)+COUNTA('2nd'!F2:F41)+COUNTA('3rd'!F2:F41)+COUNTA('4th'!F2:F41)+COUNTA('5th'!F2:F41)+COUNTA('6th'!F2:F41)+COUNTA('7th'!F2:F41)+COUNTA('8th'!F2:F41)+COUNTA('9th'!F2:F41)+COUNTA('10th'!F2:F41)+COUNTA('11th'!F2:F41)+COUNTA('12th'!F2:F41)+COUNTA('13th'!F2:F41)+COUNTA('14th'!F2:F41)+COUNTA('15th'!F2:F41)+COUNTA('16th'!F2:F41)+COUNTA('17th'!F2:F41)+COUNTA('18th'!F2:F41)+COUNTA('19th'!F2:F41)+COUNTA('20th'!F2:F41)+COUNTA('21st'!F2:F41)+COUNTA('22nd'!F2:F41)+COUNTA('23rd'!F2:F41)+COUNTA('24th'!F2:F41)+COUNTA('25th'!F2:F41)+COUNTA('26th'!F2:F41)+COUNTA('27th'!F2:F41)+COUNTA('28th'!F2:F41)+COUNTA('29th'!F2:F41)+COUNTA('30th'!F2:F41)+COUNTA('31st'!F2:F41))+0</f>
         <v/>
       </c>
       <c r="G2" s="2">
-        <f>COUNTA('1ST'!G2:G41)+COUNTA('2nd'!G2:G41)+COUNTA('3rd'!G2:G41)+COUNTA('4th'!G2:G41)+COUNTA('5th'!G2:G41)+COUNTA('6th'!G2:G41)+COUNTA('7th'!G2:G41)+COUNTA('8th'!G2:G41)+COUNTA('9th'!G2:G41)+COUNTA('10th'!G2:G41)+COUNTA('11th'!G2:G41)+COUNTA('12th'!G2:G41)+COUNTA('13th'!G2:G41)+COUNTA('14th'!G2:G41)+COUNTA('15th'!G2:G41)+COUNTA('16th'!G2:G41)+COUNTA('17th'!G2:G41)+COUNTA('18th'!G2:G41)+COUNTA('19th'!G2:G41)+COUNTA('20th'!G2:G41)+COUNTA('21st'!G2:G41)+COUNTA('22nd'!G2:G41)+COUNTA('23rd'!G2:G41)+COUNTA('24th'!G2:G41)+COUNTA('25th'!G2:G41)+COUNTA('26th'!G2:G41)+COUNTA('27th'!G2:G41)+COUNTA('28th'!G2:G41)+COUNTA('29th'!G2:G41)+COUNTA('30th'!G2:G41)+COUNTA('31st'!G2:G41)</f>
+        <f>(COUNTA('1ST'!G2:G41)+COUNTA('2nd'!G2:G41)+COUNTA('3rd'!G2:G41)+COUNTA('4th'!G2:G41)+COUNTA('5th'!G2:G41)+COUNTA('6th'!G2:G41)+COUNTA('7th'!G2:G41)+COUNTA('8th'!G2:G41)+COUNTA('9th'!G2:G41)+COUNTA('10th'!G2:G41)+COUNTA('11th'!G2:G41)+COUNTA('12th'!G2:G41)+COUNTA('13th'!G2:G41)+COUNTA('14th'!G2:G41)+COUNTA('15th'!G2:G41)+COUNTA('16th'!G2:G41)+COUNTA('17th'!G2:G41)+COUNTA('18th'!G2:G41)+COUNTA('19th'!G2:G41)+COUNTA('20th'!G2:G41)+COUNTA('21st'!G2:G41)+COUNTA('22nd'!G2:G41)+COUNTA('23rd'!G2:G41)+COUNTA('24th'!G2:G41)+COUNTA('25th'!G2:G41)+COUNTA('26th'!G2:G41)+COUNTA('27th'!G2:G41)+COUNTA('28th'!G2:G41)+COUNTA('29th'!G2:G41)+COUNTA('30th'!G2:G41)+COUNTA('31st'!G2:G41))+0</f>
         <v/>
       </c>
       <c r="H2" s="2">
-        <f>COUNTA('1ST'!H2:H41)+COUNTA('2nd'!H2:H41)+COUNTA('3rd'!H2:H41)+COUNTA('4th'!H2:H41)+COUNTA('5th'!H2:H41)+COUNTA('6th'!H2:H41)+COUNTA('7th'!H2:H41)+COUNTA('8th'!H2:H41)+COUNTA('9th'!H2:H41)+COUNTA('10th'!H2:H41)+COUNTA('11th'!H2:H41)+COUNTA('12th'!H2:H41)+COUNTA('13th'!H2:H41)+COUNTA('14th'!H2:H41)+COUNTA('15th'!H2:H41)+COUNTA('16th'!H2:H41)+COUNTA('17th'!H2:H41)+COUNTA('18th'!H2:H41)+COUNTA('19th'!H2:H41)+COUNTA('20th'!H2:H41)+COUNTA('21st'!H2:H41)+COUNTA('22nd'!H2:H41)+COUNTA('23rd'!H2:H41)+COUNTA('24th'!H2:H41)+COUNTA('25th'!H2:H41)+COUNTA('26th'!H2:H41)+COUNTA('27th'!H2:H41)+COUNTA('28th'!H2:H41)+COUNTA('29th'!H2:H41)+COUNTA('30th'!H2:H41)+COUNTA('31st'!H2:H41)</f>
+        <f>(COUNTA('1ST'!H2:H41)+COUNTA('2nd'!H2:H41)+COUNTA('3rd'!H2:H41)+COUNTA('4th'!H2:H41)+COUNTA('5th'!H2:H41)+COUNTA('6th'!H2:H41)+COUNTA('7th'!H2:H41)+COUNTA('8th'!H2:H41)+COUNTA('9th'!H2:H41)+COUNTA('10th'!H2:H41)+COUNTA('11th'!H2:H41)+COUNTA('12th'!H2:H41)+COUNTA('13th'!H2:H41)+COUNTA('14th'!H2:H41)+COUNTA('15th'!H2:H41)+COUNTA('16th'!H2:H41)+COUNTA('17th'!H2:H41)+COUNTA('18th'!H2:H41)+COUNTA('19th'!H2:H41)+COUNTA('20th'!H2:H41)+COUNTA('21st'!H2:H41)+COUNTA('22nd'!H2:H41)+COUNTA('23rd'!H2:H41)+COUNTA('24th'!H2:H41)+COUNTA('25th'!H2:H41)+COUNTA('26th'!H2:H41)+COUNTA('27th'!H2:H41)+COUNTA('28th'!H2:H41)+COUNTA('29th'!H2:H41)+COUNTA('30th'!H2:H41)+COUNTA('31st'!H2:H41))+0</f>
         <v/>
       </c>
       <c r="I2" s="2">
-        <f>COUNTA('1ST'!I2:I41)+COUNTA('2nd'!I2:I41)+COUNTA('3rd'!I2:I41)+COUNTA('4th'!I2:I41)+COUNTA('5th'!I2:I41)+COUNTA('6th'!I2:I41)+COUNTA('7th'!I2:I41)+COUNTA('8th'!I2:I41)+COUNTA('9th'!I2:I41)+COUNTA('10th'!I2:I41)+COUNTA('11th'!I2:I41)+COUNTA('12th'!I2:I41)+COUNTA('13th'!I2:I41)+COUNTA('14th'!I2:I41)+COUNTA('15th'!I2:I41)+COUNTA('16th'!I2:I41)+COUNTA('17th'!I2:I41)+COUNTA('18th'!I2:I41)+COUNTA('19th'!I2:I41)+COUNTA('20th'!I2:I41)+COUNTA('21st'!I2:I41)+COUNTA('22nd'!I2:I41)+COUNTA('23rd'!I2:I41)+COUNTA('24th'!I2:I41)+COUNTA('25th'!I2:I41)+COUNTA('26th'!I2:I41)+COUNTA('27th'!I2:I41)+COUNTA('28th'!I2:I41)+COUNTA('29th'!I2:I41)+COUNTA('30th'!I2:I41)+COUNTA('31st'!I2:I41)</f>
+        <f>(COUNTA('1ST'!I2:I41)+COUNTA('2nd'!I2:I41)+COUNTA('3rd'!I2:I41)+COUNTA('4th'!I2:I41)+COUNTA('5th'!I2:I41)+COUNTA('6th'!I2:I41)+COUNTA('7th'!I2:I41)+COUNTA('8th'!I2:I41)+COUNTA('9th'!I2:I41)+COUNTA('10th'!I2:I41)+COUNTA('11th'!I2:I41)+COUNTA('12th'!I2:I41)+COUNTA('13th'!I2:I41)+COUNTA('14th'!I2:I41)+COUNTA('15th'!I2:I41)+COUNTA('16th'!I2:I41)+COUNTA('17th'!I2:I41)+COUNTA('18th'!I2:I41)+COUNTA('19th'!I2:I41)+COUNTA('20th'!I2:I41)+COUNTA('21st'!I2:I41)+COUNTA('22nd'!I2:I41)+COUNTA('23rd'!I2:I41)+COUNTA('24th'!I2:I41)+COUNTA('25th'!I2:I41)+COUNTA('26th'!I2:I41)+COUNTA('27th'!I2:I41)+COUNTA('28th'!I2:I41)+COUNTA('29th'!I2:I41)+COUNTA('30th'!I2:I41)+COUNTA('31st'!I2:I41))+0</f>
         <v/>
       </c>
       <c r="J2" s="2">
-        <f>COUNTA('1ST'!J2:J41)+COUNTA('2nd'!J2:J41)+COUNTA('3rd'!J2:J41)+COUNTA('4th'!J2:J41)+COUNTA('5th'!J2:J41)+COUNTA('6th'!J2:J41)+COUNTA('7th'!J2:J41)+COUNTA('8th'!J2:J41)+COUNTA('9th'!J2:J41)+COUNTA('10th'!J2:J41)+COUNTA('11th'!J2:J41)+COUNTA('12th'!J2:J41)+COUNTA('13th'!J2:J41)+COUNTA('14th'!J2:J41)+COUNTA('15th'!J2:J41)+COUNTA('16th'!J2:J41)+COUNTA('17th'!J2:J41)+COUNTA('18th'!J2:J41)+COUNTA('19th'!J2:J41)+COUNTA('20th'!J2:J41)+COUNTA('21st'!J2:J41)+COUNTA('22nd'!J2:J41)+COUNTA('23rd'!J2:J41)+COUNTA('24th'!J2:J41)+COUNTA('25th'!J2:J41)+COUNTA('26th'!J2:J41)+COUNTA('27th'!J2:J41)+COUNTA('28th'!J2:J41)+COUNTA('29th'!J2:J41)+COUNTA('30th'!J2:J41)+COUNTA('31st'!J2:J41)</f>
+        <f>(COUNTA('1ST'!J2:J41)+COUNTA('2nd'!J2:J41)+COUNTA('3rd'!J2:J41)+COUNTA('4th'!J2:J41)+COUNTA('5th'!J2:J41)+COUNTA('6th'!J2:J41)+COUNTA('7th'!J2:J41)+COUNTA('8th'!J2:J41)+COUNTA('9th'!J2:J41)+COUNTA('10th'!J2:J41)+COUNTA('11th'!J2:J41)+COUNTA('12th'!J2:J41)+COUNTA('13th'!J2:J41)+COUNTA('14th'!J2:J41)+COUNTA('15th'!J2:J41)+COUNTA('16th'!J2:J41)+COUNTA('17th'!J2:J41)+COUNTA('18th'!J2:J41)+COUNTA('19th'!J2:J41)+COUNTA('20th'!J2:J41)+COUNTA('21st'!J2:J41)+COUNTA('22nd'!J2:J41)+COUNTA('23rd'!J2:J41)+COUNTA('24th'!J2:J41)+COUNTA('25th'!J2:J41)+COUNTA('26th'!J2:J41)+COUNTA('27th'!J2:J41)+COUNTA('28th'!J2:J41)+COUNTA('29th'!J2:J41)+COUNTA('30th'!J2:J41)+COUNTA('31st'!J2:J41))+0</f>
         <v/>
       </c>
       <c r="K2" s="2">
-        <f>COUNTA('1ST'!K2:K41)+COUNTA('2nd'!K2:K41)+COUNTA('3rd'!K2:K41)+COUNTA('4th'!K2:K41)+COUNTA('5th'!K2:K41)+COUNTA('6th'!K2:K41)+COUNTA('7th'!K2:K41)+COUNTA('8th'!K2:K41)+COUNTA('9th'!K2:K41)+COUNTA('10th'!K2:K41)+COUNTA('11th'!K2:K41)+COUNTA('12th'!K2:K41)+COUNTA('13th'!K2:K41)+COUNTA('14th'!K2:K41)+COUNTA('15th'!K2:K41)+COUNTA('16th'!K2:K41)+COUNTA('17th'!K2:K41)+COUNTA('18th'!K2:K41)+COUNTA('19th'!K2:K41)+COUNTA('20th'!K2:K41)+COUNTA('21st'!K2:K41)+COUNTA('22nd'!K2:K41)+COUNTA('23rd'!K2:K41)+COUNTA('24th'!K2:K41)+COUNTA('25th'!K2:K41)+COUNTA('26th'!K2:K41)+COUNTA('27th'!K2:K41)+COUNTA('28th'!K2:K41)+COUNTA('29th'!K2:K41)+COUNTA('30th'!K2:K41)+COUNTA('31st'!K2:K41)</f>
+        <f>(COUNTA('1ST'!K2:K41)+COUNTA('2nd'!K2:K41)+COUNTA('3rd'!K2:K41)+COUNTA('4th'!K2:K41)+COUNTA('5th'!K2:K41)+COUNTA('6th'!K2:K41)+COUNTA('7th'!K2:K41)+COUNTA('8th'!K2:K41)+COUNTA('9th'!K2:K41)+COUNTA('10th'!K2:K41)+COUNTA('11th'!K2:K41)+COUNTA('12th'!K2:K41)+COUNTA('13th'!K2:K41)+COUNTA('14th'!K2:K41)+COUNTA('15th'!K2:K41)+COUNTA('16th'!K2:K41)+COUNTA('17th'!K2:K41)+COUNTA('18th'!K2:K41)+COUNTA('19th'!K2:K41)+COUNTA('20th'!K2:K41)+COUNTA('21st'!K2:K41)+COUNTA('22nd'!K2:K41)+COUNTA('23rd'!K2:K41)+COUNTA('24th'!K2:K41)+COUNTA('25th'!K2:K41)+COUNTA('26th'!K2:K41)+COUNTA('27th'!K2:K41)+COUNTA('28th'!K2:K41)+COUNTA('29th'!K2:K41)+COUNTA('30th'!K2:K41)+COUNTA('31st'!K2:K41))+0</f>
         <v/>
       </c>
       <c r="L2" s="2">
-        <f>COUNTA('1ST'!L2:L41)+COUNTA('2nd'!L2:L41)+COUNTA('3rd'!L2:L41)+COUNTA('4th'!L2:L41)+COUNTA('5th'!L2:L41)+COUNTA('6th'!L2:L41)+COUNTA('7th'!L2:L41)+COUNTA('8th'!L2:L41)+COUNTA('9th'!L2:L41)+COUNTA('10th'!L2:L41)+COUNTA('11th'!L2:L41)+COUNTA('12th'!L2:L41)+COUNTA('13th'!L2:L41)+COUNTA('14th'!L2:L41)+COUNTA('15th'!L2:L41)+COUNTA('16th'!L2:L41)+COUNTA('17th'!L2:L41)+COUNTA('18th'!L2:L41)+COUNTA('19th'!L2:L41)+COUNTA('20th'!L2:L41)+COUNTA('21st'!L2:L41)+COUNTA('22nd'!L2:L41)+COUNTA('23rd'!L2:L41)+COUNTA('24th'!L2:L41)+COUNTA('25th'!L2:L41)+COUNTA('26th'!L2:L41)+COUNTA('27th'!L2:L41)+COUNTA('28th'!L2:L41)+COUNTA('29th'!L2:L41)+COUNTA('30th'!L2:L41)+COUNTA('31st'!L2:L41)</f>
+        <f>(COUNTA('1ST'!L2:L41)+COUNTA('2nd'!L2:L41)+COUNTA('3rd'!L2:L41)+COUNTA('4th'!L2:L41)+COUNTA('5th'!L2:L41)+COUNTA('6th'!L2:L41)+COUNTA('7th'!L2:L41)+COUNTA('8th'!L2:L41)+COUNTA('9th'!L2:L41)+COUNTA('10th'!L2:L41)+COUNTA('11th'!L2:L41)+COUNTA('12th'!L2:L41)+COUNTA('13th'!L2:L41)+COUNTA('14th'!L2:L41)+COUNTA('15th'!L2:L41)+COUNTA('16th'!L2:L41)+COUNTA('17th'!L2:L41)+COUNTA('18th'!L2:L41)+COUNTA('19th'!L2:L41)+COUNTA('20th'!L2:L41)+COUNTA('21st'!L2:L41)+COUNTA('22nd'!L2:L41)+COUNTA('23rd'!L2:L41)+COUNTA('24th'!L2:L41)+COUNTA('25th'!L2:L41)+COUNTA('26th'!L2:L41)+COUNTA('27th'!L2:L41)+COUNTA('28th'!L2:L41)+COUNTA('29th'!L2:L41)+COUNTA('30th'!L2:L41)+COUNTA('31st'!L2:L41))+0</f>
         <v/>
       </c>
       <c r="M2" s="2">
-        <f>COUNTA('1ST'!M2:M41)+COUNTA('2nd'!M2:M41)+COUNTA('3rd'!M2:M41)+COUNTA('4th'!M2:M41)+COUNTA('5th'!M2:M41)+COUNTA('6th'!M2:M41)+COUNTA('7th'!M2:M41)+COUNTA('8th'!M2:M41)+COUNTA('9th'!M2:M41)+COUNTA('10th'!M2:M41)+COUNTA('11th'!M2:M41)+COUNTA('12th'!M2:M41)+COUNTA('13th'!M2:M41)+COUNTA('14th'!M2:M41)+COUNTA('15th'!M2:M41)+COUNTA('16th'!M2:M41)+COUNTA('17th'!M2:M41)+COUNTA('18th'!M2:M41)+COUNTA('19th'!M2:M41)+COUNTA('20th'!M2:M41)+COUNTA('21st'!M2:M41)+COUNTA('22nd'!M2:M41)+COUNTA('23rd'!M2:M41)+COUNTA('24th'!M2:M41)+COUNTA('25th'!M2:M41)+COUNTA('26th'!M2:M41)+COUNTA('27th'!M2:M41)+COUNTA('28th'!M2:M41)+COUNTA('29th'!M2:M41)+COUNTA('30th'!M2:M41)+COUNTA('31st'!M2:M41)</f>
+        <f>(COUNTA('1ST'!M2:M41)+COUNTA('2nd'!M2:M41)+COUNTA('3rd'!M2:M41)+COUNTA('4th'!M2:M41)+COUNTA('5th'!M2:M41)+COUNTA('6th'!M2:M41)+COUNTA('7th'!M2:M41)+COUNTA('8th'!M2:M41)+COUNTA('9th'!M2:M41)+COUNTA('10th'!M2:M41)+COUNTA('11th'!M2:M41)+COUNTA('12th'!M2:M41)+COUNTA('13th'!M2:M41)+COUNTA('14th'!M2:M41)+COUNTA('15th'!M2:M41)+COUNTA('16th'!M2:M41)+COUNTA('17th'!M2:M41)+COUNTA('18th'!M2:M41)+COUNTA('19th'!M2:M41)+COUNTA('20th'!M2:M41)+COUNTA('21st'!M2:M41)+COUNTA('22nd'!M2:M41)+COUNTA('23rd'!M2:M41)+COUNTA('24th'!M2:M41)+COUNTA('25th'!M2:M41)+COUNTA('26th'!M2:M41)+COUNTA('27th'!M2:M41)+COUNTA('28th'!M2:M41)+COUNTA('29th'!M2:M41)+COUNTA('30th'!M2:M41)+COUNTA('31st'!M2:M41))+0</f>
         <v/>
       </c>
       <c r="N2" s="2">
-        <f>COUNTA('1ST'!N2:N41)+COUNTA('2nd'!N2:N41)+COUNTA('3rd'!N2:N41)+COUNTA('4th'!N2:N41)+COUNTA('5th'!N2:N41)+COUNTA('6th'!N2:N41)+COUNTA('7th'!N2:N41)+COUNTA('8th'!N2:N41)+COUNTA('9th'!N2:N41)+COUNTA('10th'!N2:N41)+COUNTA('11th'!N2:N41)+COUNTA('12th'!N2:N41)+COUNTA('13th'!N2:N41)+COUNTA('14th'!N2:N41)+COUNTA('15th'!N2:N41)+COUNTA('16th'!N2:N41)+COUNTA('17th'!N2:N41)+COUNTA('18th'!N2:N41)+COUNTA('19th'!N2:N41)+COUNTA('20th'!N2:N41)+COUNTA('21st'!N2:N41)+COUNTA('22nd'!N2:N41)+COUNTA('23rd'!N2:N41)+COUNTA('24th'!N2:N41)+COUNTA('25th'!N2:N41)+COUNTA('26th'!N2:N41)+COUNTA('27th'!N2:N41)+COUNTA('28th'!N2:N41)+COUNTA('29th'!N2:N41)+COUNTA('30th'!N2:N41)+COUNTA('31st'!N2:N41)</f>
+        <f>(COUNTA('1ST'!N2:N41)+COUNTA('2nd'!N2:N41)+COUNTA('3rd'!N2:N41)+COUNTA('4th'!N2:N41)+COUNTA('5th'!N2:N41)+COUNTA('6th'!N2:N41)+COUNTA('7th'!N2:N41)+COUNTA('8th'!N2:N41)+COUNTA('9th'!N2:N41)+COUNTA('10th'!N2:N41)+COUNTA('11th'!N2:N41)+COUNTA('12th'!N2:N41)+COUNTA('13th'!N2:N41)+COUNTA('14th'!N2:N41)+COUNTA('15th'!N2:N41)+COUNTA('16th'!N2:N41)+COUNTA('17th'!N2:N41)+COUNTA('18th'!N2:N41)+COUNTA('19th'!N2:N41)+COUNTA('20th'!N2:N41)+COUNTA('21st'!N2:N41)+COUNTA('22nd'!N2:N41)+COUNTA('23rd'!N2:N41)+COUNTA('24th'!N2:N41)+COUNTA('25th'!N2:N41)+COUNTA('26th'!N2:N41)+COUNTA('27th'!N2:N41)+COUNTA('28th'!N2:N41)+COUNTA('29th'!N2:N41)+COUNTA('30th'!N2:N41)+COUNTA('31st'!N2:N41))+0</f>
         <v/>
       </c>
       <c r="O2" s="2">
-        <f>COUNTA('1ST'!O2:O41)+COUNTA('2nd'!O2:O41)+COUNTA('3rd'!O2:O41)+COUNTA('4th'!O2:O41)+COUNTA('5th'!O2:O41)+COUNTA('6th'!O2:O41)+COUNTA('7th'!O2:O41)+COUNTA('8th'!O2:O41)+COUNTA('9th'!O2:O41)+COUNTA('10th'!O2:O41)+COUNTA('11th'!O2:O41)+COUNTA('12th'!O2:O41)+COUNTA('13th'!O2:O41)+COUNTA('14th'!O2:O41)+COUNTA('15th'!O2:O41)+COUNTA('16th'!O2:O41)+COUNTA('17th'!O2:O41)+COUNTA('18th'!O2:O41)+COUNTA('19th'!O2:O41)+COUNTA('20th'!O2:O41)+COUNTA('21st'!O2:O41)+COUNTA('22nd'!O2:O41)+COUNTA('23rd'!O2:O41)+COUNTA('24th'!O2:O41)+COUNTA('25th'!O2:O41)+COUNTA('26th'!O2:O41)+COUNTA('27th'!O2:O41)+COUNTA('28th'!O2:O41)+COUNTA('29th'!O2:O41)+COUNTA('30th'!O2:O41)+COUNTA('31st'!O2:O41)</f>
+        <f>(COUNTA('1ST'!O2:O41)+COUNTA('2nd'!O2:O41)+COUNTA('3rd'!O2:O41)+COUNTA('4th'!O2:O41)+COUNTA('5th'!O2:O41)+COUNTA('6th'!O2:O41)+COUNTA('7th'!O2:O41)+COUNTA('8th'!O2:O41)+COUNTA('9th'!O2:O41)+COUNTA('10th'!O2:O41)+COUNTA('11th'!O2:O41)+COUNTA('12th'!O2:O41)+COUNTA('13th'!O2:O41)+COUNTA('14th'!O2:O41)+COUNTA('15th'!O2:O41)+COUNTA('16th'!O2:O41)+COUNTA('17th'!O2:O41)+COUNTA('18th'!O2:O41)+COUNTA('19th'!O2:O41)+COUNTA('20th'!O2:O41)+COUNTA('21st'!O2:O41)+COUNTA('22nd'!O2:O41)+COUNTA('23rd'!O2:O41)+COUNTA('24th'!O2:O41)+COUNTA('25th'!O2:O41)+COUNTA('26th'!O2:O41)+COUNTA('27th'!O2:O41)+COUNTA('28th'!O2:O41)+COUNTA('29th'!O2:O41)+COUNTA('30th'!O2:O41)+COUNTA('31st'!O2:O41))+0</f>
         <v/>
       </c>
       <c r="P2" s="2">
-        <f>COUNTA('1ST'!P2:P41)+COUNTA('2nd'!P2:P41)+COUNTA('3rd'!P2:P41)+COUNTA('4th'!P2:P41)+COUNTA('5th'!P2:P41)+COUNTA('6th'!P2:P41)+COUNTA('7th'!P2:P41)+COUNTA('8th'!P2:P41)+COUNTA('9th'!P2:P41)+COUNTA('10th'!P2:P41)+COUNTA('11th'!P2:P41)+COUNTA('12th'!P2:P41)+COUNTA('13th'!P2:P41)+COUNTA('14th'!P2:P41)+COUNTA('15th'!P2:P41)+COUNTA('16th'!P2:P41)+COUNTA('17th'!P2:P41)+COUNTA('18th'!P2:P41)+COUNTA('19th'!P2:P41)+COUNTA('20th'!P2:P41)+COUNTA('21st'!P2:P41)+COUNTA('22nd'!P2:P41)+COUNTA('23rd'!P2:P41)+COUNTA('24th'!P2:P41)+COUNTA('25th'!P2:P41)+COUNTA('26th'!P2:P41)+COUNTA('27th'!P2:P41)+COUNTA('28th'!P2:P41)+COUNTA('29th'!P2:P41)+COUNTA('30th'!P2:P41)+COUNTA('31st'!P2:P41)</f>
+        <f>(COUNTA('1ST'!P2:P41)+COUNTA('2nd'!P2:P41)+COUNTA('3rd'!P2:P41)+COUNTA('4th'!P2:P41)+COUNTA('5th'!P2:P41)+COUNTA('6th'!P2:P41)+COUNTA('7th'!P2:P41)+COUNTA('8th'!P2:P41)+COUNTA('9th'!P2:P41)+COUNTA('10th'!P2:P41)+COUNTA('11th'!P2:P41)+COUNTA('12th'!P2:P41)+COUNTA('13th'!P2:P41)+COUNTA('14th'!P2:P41)+COUNTA('15th'!P2:P41)+COUNTA('16th'!P2:P41)+COUNTA('17th'!P2:P41)+COUNTA('18th'!P2:P41)+COUNTA('19th'!P2:P41)+COUNTA('20th'!P2:P41)+COUNTA('21st'!P2:P41)+COUNTA('22nd'!P2:P41)+COUNTA('23rd'!P2:P41)+COUNTA('24th'!P2:P41)+COUNTA('25th'!P2:P41)+COUNTA('26th'!P2:P41)+COUNTA('27th'!P2:P41)+COUNTA('28th'!P2:P41)+COUNTA('29th'!P2:P41)+COUNTA('30th'!P2:P41)+COUNTA('31st'!P2:P41))+0</f>
         <v/>
       </c>
       <c r="Q2" s="2">
-        <f>COUNTA('1ST'!Q2:Q41)+COUNTA('2nd'!Q2:Q41)+COUNTA('3rd'!Q2:Q41)+COUNTA('4th'!Q2:Q41)+COUNTA('5th'!Q2:Q41)+COUNTA('6th'!Q2:Q41)+COUNTA('7th'!Q2:Q41)+COUNTA('8th'!Q2:Q41)+COUNTA('9th'!Q2:Q41)+COUNTA('10th'!Q2:Q41)+COUNTA('11th'!Q2:Q41)+COUNTA('12th'!Q2:Q41)+COUNTA('13th'!Q2:Q41)+COUNTA('14th'!Q2:Q41)+COUNTA('15th'!Q2:Q41)+COUNTA('16th'!Q2:Q41)+COUNTA('17th'!Q2:Q41)+COUNTA('18th'!Q2:Q41)+COUNTA('19th'!Q2:Q41)+COUNTA('20th'!Q2:Q41)+COUNTA('21st'!Q2:Q41)+COUNTA('22nd'!Q2:Q41)+COUNTA('23rd'!Q2:Q41)+COUNTA('24th'!Q2:Q41)+COUNTA('25th'!Q2:Q41)+COUNTA('26th'!Q2:Q41)+COUNTA('27th'!Q2:Q41)+COUNTA('28th'!Q2:Q41)+COUNTA('29th'!Q2:Q41)+COUNTA('30th'!Q2:Q41)+COUNTA('31st'!Q2:Q41)</f>
+        <f>(COUNTA('1ST'!Q2:Q41)+COUNTA('2nd'!Q2:Q41)+COUNTA('3rd'!Q2:Q41)+COUNTA('4th'!Q2:Q41)+COUNTA('5th'!Q2:Q41)+COUNTA('6th'!Q2:Q41)+COUNTA('7th'!Q2:Q41)+COUNTA('8th'!Q2:Q41)+COUNTA('9th'!Q2:Q41)+COUNTA('10th'!Q2:Q41)+COUNTA('11th'!Q2:Q41)+COUNTA('12th'!Q2:Q41)+COUNTA('13th'!Q2:Q41)+COUNTA('14th'!Q2:Q41)+COUNTA('15th'!Q2:Q41)+COUNTA('16th'!Q2:Q41)+COUNTA('17th'!Q2:Q41)+COUNTA('18th'!Q2:Q41)+COUNTA('19th'!Q2:Q41)+COUNTA('20th'!Q2:Q41)+COUNTA('21st'!Q2:Q41)+COUNTA('22nd'!Q2:Q41)+COUNTA('23rd'!Q2:Q41)+COUNTA('24th'!Q2:Q41)+COUNTA('25th'!Q2:Q41)+COUNTA('26th'!Q2:Q41)+COUNTA('27th'!Q2:Q41)+COUNTA('28th'!Q2:Q41)+COUNTA('29th'!Q2:Q41)+COUNTA('30th'!Q2:Q41)+COUNTA('31st'!Q2:Q41))+0</f>
         <v/>
       </c>
       <c r="R2" s="2">
-        <f>COUNTA('1ST'!R2:R41)+COUNTA('2nd'!R2:R41)+COUNTA('3rd'!R2:R41)+COUNTA('4th'!R2:R41)+COUNTA('5th'!R2:R41)+COUNTA('6th'!R2:R41)+COUNTA('7th'!R2:R41)+COUNTA('8th'!R2:R41)+COUNTA('9th'!R2:R41)+COUNTA('10th'!R2:R41)+COUNTA('11th'!R2:R41)+COUNTA('12th'!R2:R41)+COUNTA('13th'!R2:R41)+COUNTA('14th'!R2:R41)+COUNTA('15th'!R2:R41)+COUNTA('16th'!R2:R41)+COUNTA('17th'!R2:R41)+COUNTA('18th'!R2:R41)+COUNTA('19th'!R2:R41)+COUNTA('20th'!R2:R41)+COUNTA('21st'!R2:R41)+COUNTA('22nd'!R2:R41)+COUNTA('23rd'!R2:R41)+COUNTA('24th'!R2:R41)+COUNTA('25th'!R2:R41)+COUNTA('26th'!R2:R41)+COUNTA('27th'!R2:R41)+COUNTA('28th'!R2:R41)+COUNTA('29th'!R2:R41)+COUNTA('30th'!R2:R41)+COUNTA('31st'!R2:R41)</f>
+        <f>(COUNTA('1ST'!R2:R41)+COUNTA('2nd'!R2:R41)+COUNTA('3rd'!R2:R41)+COUNTA('4th'!R2:R41)+COUNTA('5th'!R2:R41)+COUNTA('6th'!R2:R41)+COUNTA('7th'!R2:R41)+COUNTA('8th'!R2:R41)+COUNTA('9th'!R2:R41)+COUNTA('10th'!R2:R41)+COUNTA('11th'!R2:R41)+COUNTA('12th'!R2:R41)+COUNTA('13th'!R2:R41)+COUNTA('14th'!R2:R41)+COUNTA('15th'!R2:R41)+COUNTA('16th'!R2:R41)+COUNTA('17th'!R2:R41)+COUNTA('18th'!R2:R41)+COUNTA('19th'!R2:R41)+COUNTA('20th'!R2:R41)+COUNTA('21st'!R2:R41)+COUNTA('22nd'!R2:R41)+COUNTA('23rd'!R2:R41)+COUNTA('24th'!R2:R41)+COUNTA('25th'!R2:R41)+COUNTA('26th'!R2:R41)+COUNTA('27th'!R2:R41)+COUNTA('28th'!R2:R41)+COUNTA('29th'!R2:R41)+COUNTA('30th'!R2:R41)+COUNTA('31st'!R2:R41))+0</f>
         <v/>
       </c>
       <c r="S2" s="2">
-        <f>COUNTA('1ST'!S2:S41)+COUNTA('2nd'!S2:S41)+COUNTA('3rd'!S2:S41)+COUNTA('4th'!S2:S41)+COUNTA('5th'!S2:S41)+COUNTA('6th'!S2:S41)+COUNTA('7th'!S2:S41)+COUNTA('8th'!S2:S41)+COUNTA('9th'!S2:S41)+COUNTA('10th'!S2:S41)+COUNTA('11th'!S2:S41)+COUNTA('12th'!S2:S41)+COUNTA('13th'!S2:S41)+COUNTA('14th'!S2:S41)+COUNTA('15th'!S2:S41)+COUNTA('16th'!S2:S41)+COUNTA('17th'!S2:S41)+COUNTA('18th'!S2:S41)+COUNTA('19th'!S2:S41)+COUNTA('20th'!S2:S41)+COUNTA('21st'!S2:S41)+COUNTA('22nd'!S2:S41)+COUNTA('23rd'!S2:S41)+COUNTA('24th'!S2:S41)+COUNTA('25th'!S2:S41)+COUNTA('26th'!S2:S41)+COUNTA('27th'!S2:S41)+COUNTA('28th'!S2:S41)+COUNTA('29th'!S2:S41)+COUNTA('30th'!S2:S41)+COUNTA('31st'!S2:S41)</f>
+        <f>(COUNTA('1ST'!S2:S41)+COUNTA('2nd'!S2:S41)+COUNTA('3rd'!S2:S41)+COUNTA('4th'!S2:S41)+COUNTA('5th'!S2:S41)+COUNTA('6th'!S2:S41)+COUNTA('7th'!S2:S41)+COUNTA('8th'!S2:S41)+COUNTA('9th'!S2:S41)+COUNTA('10th'!S2:S41)+COUNTA('11th'!S2:S41)+COUNTA('12th'!S2:S41)+COUNTA('13th'!S2:S41)+COUNTA('14th'!S2:S41)+COUNTA('15th'!S2:S41)+COUNTA('16th'!S2:S41)+COUNTA('17th'!S2:S41)+COUNTA('18th'!S2:S41)+COUNTA('19th'!S2:S41)+COUNTA('20th'!S2:S41)+COUNTA('21st'!S2:S41)+COUNTA('22nd'!S2:S41)+COUNTA('23rd'!S2:S41)+COUNTA('24th'!S2:S41)+COUNTA('25th'!S2:S41)+COUNTA('26th'!S2:S41)+COUNTA('27th'!S2:S41)+COUNTA('28th'!S2:S41)+COUNTA('29th'!S2:S41)+COUNTA('30th'!S2:S41)+COUNTA('31st'!S2:S41))+0</f>
         <v/>
       </c>
       <c r="T2" s="2">
-        <f>COUNTA('1ST'!T2:T41)+COUNTA('2nd'!T2:T41)+COUNTA('3rd'!T2:T41)+COUNTA('4th'!T2:T41)+COUNTA('5th'!T2:T41)+COUNTA('6th'!T2:T41)+COUNTA('7th'!T2:T41)+COUNTA('8th'!T2:T41)+COUNTA('9th'!T2:T41)+COUNTA('10th'!T2:T41)+COUNTA('11th'!T2:T41)+COUNTA('12th'!T2:T41)+COUNTA('13th'!T2:T41)+COUNTA('14th'!T2:T41)+COUNTA('15th'!T2:T41)+COUNTA('16th'!T2:T41)+COUNTA('17th'!T2:T41)+COUNTA('18th'!T2:T41)+COUNTA('19th'!T2:T41)+COUNTA('20th'!T2:T41)+COUNTA('21st'!T2:T41)+COUNTA('22nd'!T2:T41)+COUNTA('23rd'!T2:T41)+COUNTA('24th'!T2:T41)+COUNTA('25th'!T2:T41)+COUNTA('26th'!T2:T41)+COUNTA('27th'!T2:T41)+COUNTA('28th'!T2:T41)+COUNTA('29th'!T2:T41)+COUNTA('30th'!T2:T41)+COUNTA('31st'!T2:T41)</f>
+        <f>(COUNTA('1ST'!T2:T41)+COUNTA('2nd'!T2:T41)+COUNTA('3rd'!T2:T41)+COUNTA('4th'!T2:T41)+COUNTA('5th'!T2:T41)+COUNTA('6th'!T2:T41)+COUNTA('7th'!T2:T41)+COUNTA('8th'!T2:T41)+COUNTA('9th'!T2:T41)+COUNTA('10th'!T2:T41)+COUNTA('11th'!T2:T41)+COUNTA('12th'!T2:T41)+COUNTA('13th'!T2:T41)+COUNTA('14th'!T2:T41)+COUNTA('15th'!T2:T41)+COUNTA('16th'!T2:T41)+COUNTA('17th'!T2:T41)+COUNTA('18th'!T2:T41)+COUNTA('19th'!T2:T41)+COUNTA('20th'!T2:T41)+COUNTA('21st'!T2:T41)+COUNTA('22nd'!T2:T41)+COUNTA('23rd'!T2:T41)+COUNTA('24th'!T2:T41)+COUNTA('25th'!T2:T41)+COUNTA('26th'!T2:T41)+COUNTA('27th'!T2:T41)+COUNTA('28th'!T2:T41)+COUNTA('29th'!T2:T41)+COUNTA('30th'!T2:T41)+COUNTA('31st'!T2:T41))+0</f>
         <v/>
       </c>
       <c r="U2" s="2">
-        <f>COUNTA('1ST'!U2:U41)+COUNTA('2nd'!U2:U41)+COUNTA('3rd'!U2:U41)+COUNTA('4th'!U2:U41)+COUNTA('5th'!U2:U41)+COUNTA('6th'!U2:U41)+COUNTA('7th'!U2:U41)+COUNTA('8th'!U2:U41)+COUNTA('9th'!U2:U41)+COUNTA('10th'!U2:U41)+COUNTA('11th'!U2:U41)+COUNTA('12th'!U2:U41)+COUNTA('13th'!U2:U41)+COUNTA('14th'!U2:U41)+COUNTA('15th'!U2:U41)+COUNTA('16th'!U2:U41)+COUNTA('17th'!U2:U41)+COUNTA('18th'!U2:U41)+COUNTA('19th'!U2:U41)+COUNTA('20th'!U2:U41)+COUNTA('21st'!U2:U41)+COUNTA('22nd'!U2:U41)+COUNTA('23rd'!U2:U41)+COUNTA('24th'!U2:U41)+COUNTA('25th'!U2:U41)+COUNTA('26th'!U2:U41)+COUNTA('27th'!U2:U41)+COUNTA('28th'!U2:U41)+COUNTA('29th'!U2:U41)+COUNTA('30th'!U2:U41)+COUNTA('31st'!U2:U41)</f>
-        <v/>
-      </c>
-      <c r="W2" s="3" t="inlineStr">
+        <f>(COUNTA('1ST'!U2:U41)+COUNTA('2nd'!U2:U41)+COUNTA('3rd'!U2:U41)+COUNTA('4th'!U2:U41)+COUNTA('5th'!U2:U41)+COUNTA('6th'!U2:U41)+COUNTA('7th'!U2:U41)+COUNTA('8th'!U2:U41)+COUNTA('9th'!U2:U41)+COUNTA('10th'!U2:U41)+COUNTA('11th'!U2:U41)+COUNTA('12th'!U2:U41)+COUNTA('13th'!U2:U41)+COUNTA('14th'!U2:U41)+COUNTA('15th'!U2:U41)+COUNTA('16th'!U2:U41)+COUNTA('17th'!U2:U41)+COUNTA('18th'!U2:U41)+COUNTA('19th'!U2:U41)+COUNTA('20th'!U2:U41)+COUNTA('21st'!U2:U41)+COUNTA('22nd'!U2:U41)+COUNTA('23rd'!U2:U41)+COUNTA('24th'!U2:U41)+COUNTA('25th'!U2:U41)+COUNTA('26th'!U2:U41)+COUNTA('27th'!U2:U41)+COUNTA('28th'!U2:U41)+COUNTA('29th'!U2:U41)+COUNTA('30th'!U2:U41)+COUNTA('31st'!U2:U41))+0</f>
+        <v/>
+      </c>
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="X2" s="3" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>Reported By</t>
         </is>
       </c>
-      <c r="Y2" s="3" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>HIV</t>
         </is>
       </c>
-      <c r="Z2" s="3" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>DBT</t>
         </is>
       </c>
-      <c r="AB2" s="3" t="inlineStr">
+      <c r="AB2" s="4" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="AC2" s="3" t="inlineStr">
+      <c r="AC2" s="4" t="inlineStr">
         <is>
           <t>Reported By</t>
         </is>
       </c>
-      <c r="AD2" s="3" t="inlineStr">
+      <c r="AD2" s="4" t="inlineStr">
         <is>
           <t>HIV</t>
         </is>
       </c>
-      <c r="AE2" s="3" t="inlineStr">
+      <c r="AE2" s="4" t="inlineStr">
         <is>
           <t>DBT</t>
         </is>
       </c>
-      <c r="AG2" s="3" t="inlineStr">
+      <c r="AG2" s="4" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="AH2" s="3" t="inlineStr">
+      <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>Reported By</t>
         </is>
       </c>
-      <c r="AI2" s="3" t="inlineStr">
+      <c r="AI2" s="4" t="inlineStr">
         <is>
           <t>HIV</t>
         </is>
       </c>
-      <c r="AJ2" s="3" t="inlineStr">
+      <c r="AJ2" s="4" t="inlineStr">
         <is>
           <t>DBT</t>
         </is>
       </c>
-      <c r="AL2" s="3" t="inlineStr">
+      <c r="AL2" s="4" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="AM2" s="3" t="inlineStr">
+      <c r="AM2" s="4" t="inlineStr">
         <is>
           <t>Reported By</t>
         </is>
       </c>
-      <c r="AN2" s="3" t="inlineStr">
+      <c r="AN2" s="4" t="inlineStr">
         <is>
           <t>HIV</t>
         </is>
       </c>
-      <c r="AO2" s="3" t="inlineStr">
+      <c r="AO2" s="4" t="inlineStr">
         <is>
           <t>DBT</t>
         </is>
@@ -3460,91 +3492,91 @@
         </is>
       </c>
       <c r="C3" s="2">
-        <f>COUNTA('1ST'!C42:C81)+COUNTA('2nd'!C42:C81)+COUNTA('3rd'!C42:C81)+COUNTA('4th'!C42:C81)+COUNTA('5th'!C42:C81)+COUNTA('6th'!C42:C81)+COUNTA('7th'!C42:C81)+COUNTA('8th'!C42:C81)+COUNTA('9th'!C42:C81)+COUNTA('10th'!C42:C81)+COUNTA('11th'!C42:C81)+COUNTA('12th'!C42:C81)+COUNTA('13th'!C42:C81)+COUNTA('14th'!C42:C81)+COUNTA('15th'!C42:C81)+COUNTA('16th'!C42:C81)+COUNTA('17th'!C42:C81)+COUNTA('18th'!C42:C81)+COUNTA('19th'!C42:C81)+COUNTA('20th'!C42:C81)+COUNTA('21st'!C42:C81)+COUNTA('22nd'!C42:C81)+COUNTA('23rd'!C42:C81)+COUNTA('24th'!C42:C81)+COUNTA('25th'!C42:C81)+COUNTA('26th'!C42:C81)+COUNTA('27th'!C42:C81)+COUNTA('28th'!C42:C81)+COUNTA('29th'!C42:C81)+COUNTA('30th'!C42:C81)+COUNTA('31st'!C42:C81)</f>
+        <f>(COUNTA('1ST'!C42:C81)+COUNTA('2nd'!C42:C81)+COUNTA('3rd'!C42:C81)+COUNTA('4th'!C42:C81)+COUNTA('5th'!C42:C81)+COUNTA('6th'!C42:C81)+COUNTA('7th'!C42:C81)+COUNTA('8th'!C42:C81)+COUNTA('9th'!C42:C81)+COUNTA('10th'!C42:C81)+COUNTA('11th'!C42:C81)+COUNTA('12th'!C42:C81)+COUNTA('13th'!C42:C81)+COUNTA('14th'!C42:C81)+COUNTA('15th'!C42:C81)+COUNTA('16th'!C42:C81)+COUNTA('17th'!C42:C81)+COUNTA('18th'!C42:C81)+COUNTA('19th'!C42:C81)+COUNTA('20th'!C42:C81)+COUNTA('21st'!C42:C81)+COUNTA('22nd'!C42:C81)+COUNTA('23rd'!C42:C81)+COUNTA('24th'!C42:C81)+COUNTA('25th'!C42:C81)+COUNTA('26th'!C42:C81)+COUNTA('27th'!C42:C81)+COUNTA('28th'!C42:C81)+COUNTA('29th'!C42:C81)+COUNTA('30th'!C42:C81)+COUNTA('31st'!C42:C81))+0</f>
         <v/>
       </c>
       <c r="D3" s="2">
-        <f>COUNTA('1ST'!D42:D81)+COUNTA('2nd'!D42:D81)+COUNTA('3rd'!D42:D81)+COUNTA('4th'!D42:D81)+COUNTA('5th'!D42:D81)+COUNTA('6th'!D42:D81)+COUNTA('7th'!D42:D81)+COUNTA('8th'!D42:D81)+COUNTA('9th'!D42:D81)+COUNTA('10th'!D42:D81)+COUNTA('11th'!D42:D81)+COUNTA('12th'!D42:D81)+COUNTA('13th'!D42:D81)+COUNTA('14th'!D42:D81)+COUNTA('15th'!D42:D81)+COUNTA('16th'!D42:D81)+COUNTA('17th'!D42:D81)+COUNTA('18th'!D42:D81)+COUNTA('19th'!D42:D81)+COUNTA('20th'!D42:D81)+COUNTA('21st'!D42:D81)+COUNTA('22nd'!D42:D81)+COUNTA('23rd'!D42:D81)+COUNTA('24th'!D42:D81)+COUNTA('25th'!D42:D81)+COUNTA('26th'!D42:D81)+COUNTA('27th'!D42:D81)+COUNTA('28th'!D42:D81)+COUNTA('29th'!D42:D81)+COUNTA('30th'!D42:D81)+COUNTA('31st'!D42:D81)</f>
+        <f>(COUNTA('1ST'!D42:D81)+COUNTA('2nd'!D42:D81)+COUNTA('3rd'!D42:D81)+COUNTA('4th'!D42:D81)+COUNTA('5th'!D42:D81)+COUNTA('6th'!D42:D81)+COUNTA('7th'!D42:D81)+COUNTA('8th'!D42:D81)+COUNTA('9th'!D42:D81)+COUNTA('10th'!D42:D81)+COUNTA('11th'!D42:D81)+COUNTA('12th'!D42:D81)+COUNTA('13th'!D42:D81)+COUNTA('14th'!D42:D81)+COUNTA('15th'!D42:D81)+COUNTA('16th'!D42:D81)+COUNTA('17th'!D42:D81)+COUNTA('18th'!D42:D81)+COUNTA('19th'!D42:D81)+COUNTA('20th'!D42:D81)+COUNTA('21st'!D42:D81)+COUNTA('22nd'!D42:D81)+COUNTA('23rd'!D42:D81)+COUNTA('24th'!D42:D81)+COUNTA('25th'!D42:D81)+COUNTA('26th'!D42:D81)+COUNTA('27th'!D42:D81)+COUNTA('28th'!D42:D81)+COUNTA('29th'!D42:D81)+COUNTA('30th'!D42:D81)+COUNTA('31st'!D42:D81))+0</f>
         <v/>
       </c>
       <c r="E3" s="2">
-        <f>COUNTA('1ST'!E42:E81)+COUNTA('2nd'!E42:E81)+COUNTA('3rd'!E42:E81)+COUNTA('4th'!E42:E81)+COUNTA('5th'!E42:E81)+COUNTA('6th'!E42:E81)+COUNTA('7th'!E42:E81)+COUNTA('8th'!E42:E81)+COUNTA('9th'!E42:E81)+COUNTA('10th'!E42:E81)+COUNTA('11th'!E42:E81)+COUNTA('12th'!E42:E81)+COUNTA('13th'!E42:E81)+COUNTA('14th'!E42:E81)+COUNTA('15th'!E42:E81)+COUNTA('16th'!E42:E81)+COUNTA('17th'!E42:E81)+COUNTA('18th'!E42:E81)+COUNTA('19th'!E42:E81)+COUNTA('20th'!E42:E81)+COUNTA('21st'!E42:E81)+COUNTA('22nd'!E42:E81)+COUNTA('23rd'!E42:E81)+COUNTA('24th'!E42:E81)+COUNTA('25th'!E42:E81)+COUNTA('26th'!E42:E81)+COUNTA('27th'!E42:E81)+COUNTA('28th'!E42:E81)+COUNTA('29th'!E42:E81)+COUNTA('30th'!E42:E81)+COUNTA('31st'!E42:E81)</f>
+        <f>(COUNTA('1ST'!E42:E81)+COUNTA('2nd'!E42:E81)+COUNTA('3rd'!E42:E81)+COUNTA('4th'!E42:E81)+COUNTA('5th'!E42:E81)+COUNTA('6th'!E42:E81)+COUNTA('7th'!E42:E81)+COUNTA('8th'!E42:E81)+COUNTA('9th'!E42:E81)+COUNTA('10th'!E42:E81)+COUNTA('11th'!E42:E81)+COUNTA('12th'!E42:E81)+COUNTA('13th'!E42:E81)+COUNTA('14th'!E42:E81)+COUNTA('15th'!E42:E81)+COUNTA('16th'!E42:E81)+COUNTA('17th'!E42:E81)+COUNTA('18th'!E42:E81)+COUNTA('19th'!E42:E81)+COUNTA('20th'!E42:E81)+COUNTA('21st'!E42:E81)+COUNTA('22nd'!E42:E81)+COUNTA('23rd'!E42:E81)+COUNTA('24th'!E42:E81)+COUNTA('25th'!E42:E81)+COUNTA('26th'!E42:E81)+COUNTA('27th'!E42:E81)+COUNTA('28th'!E42:E81)+COUNTA('29th'!E42:E81)+COUNTA('30th'!E42:E81)+COUNTA('31st'!E42:E81))+0</f>
         <v/>
       </c>
       <c r="F3" s="2">
-        <f>COUNTA('1ST'!F42:F81)+COUNTA('2nd'!F42:F81)+COUNTA('3rd'!F42:F81)+COUNTA('4th'!F42:F81)+COUNTA('5th'!F42:F81)+COUNTA('6th'!F42:F81)+COUNTA('7th'!F42:F81)+COUNTA('8th'!F42:F81)+COUNTA('9th'!F42:F81)+COUNTA('10th'!F42:F81)+COUNTA('11th'!F42:F81)+COUNTA('12th'!F42:F81)+COUNTA('13th'!F42:F81)+COUNTA('14th'!F42:F81)+COUNTA('15th'!F42:F81)+COUNTA('16th'!F42:F81)+COUNTA('17th'!F42:F81)+COUNTA('18th'!F42:F81)+COUNTA('19th'!F42:F81)+COUNTA('20th'!F42:F81)+COUNTA('21st'!F42:F81)+COUNTA('22nd'!F42:F81)+COUNTA('23rd'!F42:F81)+COUNTA('24th'!F42:F81)+COUNTA('25th'!F42:F81)+COUNTA('26th'!F42:F81)+COUNTA('27th'!F42:F81)+COUNTA('28th'!F42:F81)+COUNTA('29th'!F42:F81)+COUNTA('30th'!F42:F81)+COUNTA('31st'!F42:F81)</f>
+        <f>(COUNTA('1ST'!F42:F81)+COUNTA('2nd'!F42:F81)+COUNTA('3rd'!F42:F81)+COUNTA('4th'!F42:F81)+COUNTA('5th'!F42:F81)+COUNTA('6th'!F42:F81)+COUNTA('7th'!F42:F81)+COUNTA('8th'!F42:F81)+COUNTA('9th'!F42:F81)+COUNTA('10th'!F42:F81)+COUNTA('11th'!F42:F81)+COUNTA('12th'!F42:F81)+COUNTA('13th'!F42:F81)+COUNTA('14th'!F42:F81)+COUNTA('15th'!F42:F81)+COUNTA('16th'!F42:F81)+COUNTA('17th'!F42:F81)+COUNTA('18th'!F42:F81)+COUNTA('19th'!F42:F81)+COUNTA('20th'!F42:F81)+COUNTA('21st'!F42:F81)+COUNTA('22nd'!F42:F81)+COUNTA('23rd'!F42:F81)+COUNTA('24th'!F42:F81)+COUNTA('25th'!F42:F81)+COUNTA('26th'!F42:F81)+COUNTA('27th'!F42:F81)+COUNTA('28th'!F42:F81)+COUNTA('29th'!F42:F81)+COUNTA('30th'!F42:F81)+COUNTA('31st'!F42:F81))+0</f>
         <v/>
       </c>
       <c r="G3" s="2">
-        <f>COUNTA('1ST'!G42:G81)+COUNTA('2nd'!G42:G81)+COUNTA('3rd'!G42:G81)+COUNTA('4th'!G42:G81)+COUNTA('5th'!G42:G81)+COUNTA('6th'!G42:G81)+COUNTA('7th'!G42:G81)+COUNTA('8th'!G42:G81)+COUNTA('9th'!G42:G81)+COUNTA('10th'!G42:G81)+COUNTA('11th'!G42:G81)+COUNTA('12th'!G42:G81)+COUNTA('13th'!G42:G81)+COUNTA('14th'!G42:G81)+COUNTA('15th'!G42:G81)+COUNTA('16th'!G42:G81)+COUNTA('17th'!G42:G81)+COUNTA('18th'!G42:G81)+COUNTA('19th'!G42:G81)+COUNTA('20th'!G42:G81)+COUNTA('21st'!G42:G81)+COUNTA('22nd'!G42:G81)+COUNTA('23rd'!G42:G81)+COUNTA('24th'!G42:G81)+COUNTA('25th'!G42:G81)+COUNTA('26th'!G42:G81)+COUNTA('27th'!G42:G81)+COUNTA('28th'!G42:G81)+COUNTA('29th'!G42:G81)+COUNTA('30th'!G42:G81)+COUNTA('31st'!G42:G81)</f>
+        <f>(COUNTA('1ST'!G42:G81)+COUNTA('2nd'!G42:G81)+COUNTA('3rd'!G42:G81)+COUNTA('4th'!G42:G81)+COUNTA('5th'!G42:G81)+COUNTA('6th'!G42:G81)+COUNTA('7th'!G42:G81)+COUNTA('8th'!G42:G81)+COUNTA('9th'!G42:G81)+COUNTA('10th'!G42:G81)+COUNTA('11th'!G42:G81)+COUNTA('12th'!G42:G81)+COUNTA('13th'!G42:G81)+COUNTA('14th'!G42:G81)+COUNTA('15th'!G42:G81)+COUNTA('16th'!G42:G81)+COUNTA('17th'!G42:G81)+COUNTA('18th'!G42:G81)+COUNTA('19th'!G42:G81)+COUNTA('20th'!G42:G81)+COUNTA('21st'!G42:G81)+COUNTA('22nd'!G42:G81)+COUNTA('23rd'!G42:G81)+COUNTA('24th'!G42:G81)+COUNTA('25th'!G42:G81)+COUNTA('26th'!G42:G81)+COUNTA('27th'!G42:G81)+COUNTA('28th'!G42:G81)+COUNTA('29th'!G42:G81)+COUNTA('30th'!G42:G81)+COUNTA('31st'!G42:G81))+0</f>
         <v/>
       </c>
       <c r="H3" s="2">
-        <f>COUNTA('1ST'!H42:H81)+COUNTA('2nd'!H42:H81)+COUNTA('3rd'!H42:H81)+COUNTA('4th'!H42:H81)+COUNTA('5th'!H42:H81)+COUNTA('6th'!H42:H81)+COUNTA('7th'!H42:H81)+COUNTA('8th'!H42:H81)+COUNTA('9th'!H42:H81)+COUNTA('10th'!H42:H81)+COUNTA('11th'!H42:H81)+COUNTA('12th'!H42:H81)+COUNTA('13th'!H42:H81)+COUNTA('14th'!H42:H81)+COUNTA('15th'!H42:H81)+COUNTA('16th'!H42:H81)+COUNTA('17th'!H42:H81)+COUNTA('18th'!H42:H81)+COUNTA('19th'!H42:H81)+COUNTA('20th'!H42:H81)+COUNTA('21st'!H42:H81)+COUNTA('22nd'!H42:H81)+COUNTA('23rd'!H42:H81)+COUNTA('24th'!H42:H81)+COUNTA('25th'!H42:H81)+COUNTA('26th'!H42:H81)+COUNTA('27th'!H42:H81)+COUNTA('28th'!H42:H81)+COUNTA('29th'!H42:H81)+COUNTA('30th'!H42:H81)+COUNTA('31st'!H42:H81)</f>
+        <f>(COUNTA('1ST'!H42:H81)+COUNTA('2nd'!H42:H81)+COUNTA('3rd'!H42:H81)+COUNTA('4th'!H42:H81)+COUNTA('5th'!H42:H81)+COUNTA('6th'!H42:H81)+COUNTA('7th'!H42:H81)+COUNTA('8th'!H42:H81)+COUNTA('9th'!H42:H81)+COUNTA('10th'!H42:H81)+COUNTA('11th'!H42:H81)+COUNTA('12th'!H42:H81)+COUNTA('13th'!H42:H81)+COUNTA('14th'!H42:H81)+COUNTA('15th'!H42:H81)+COUNTA('16th'!H42:H81)+COUNTA('17th'!H42:H81)+COUNTA('18th'!H42:H81)+COUNTA('19th'!H42:H81)+COUNTA('20th'!H42:H81)+COUNTA('21st'!H42:H81)+COUNTA('22nd'!H42:H81)+COUNTA('23rd'!H42:H81)+COUNTA('24th'!H42:H81)+COUNTA('25th'!H42:H81)+COUNTA('26th'!H42:H81)+COUNTA('27th'!H42:H81)+COUNTA('28th'!H42:H81)+COUNTA('29th'!H42:H81)+COUNTA('30th'!H42:H81)+COUNTA('31st'!H42:H81))+0</f>
         <v/>
       </c>
       <c r="I3" s="2">
-        <f>COUNTA('1ST'!I42:I81)+COUNTA('2nd'!I42:I81)+COUNTA('3rd'!I42:I81)+COUNTA('4th'!I42:I81)+COUNTA('5th'!I42:I81)+COUNTA('6th'!I42:I81)+COUNTA('7th'!I42:I81)+COUNTA('8th'!I42:I81)+COUNTA('9th'!I42:I81)+COUNTA('10th'!I42:I81)+COUNTA('11th'!I42:I81)+COUNTA('12th'!I42:I81)+COUNTA('13th'!I42:I81)+COUNTA('14th'!I42:I81)+COUNTA('15th'!I42:I81)+COUNTA('16th'!I42:I81)+COUNTA('17th'!I42:I81)+COUNTA('18th'!I42:I81)+COUNTA('19th'!I42:I81)+COUNTA('20th'!I42:I81)+COUNTA('21st'!I42:I81)+COUNTA('22nd'!I42:I81)+COUNTA('23rd'!I42:I81)+COUNTA('24th'!I42:I81)+COUNTA('25th'!I42:I81)+COUNTA('26th'!I42:I81)+COUNTA('27th'!I42:I81)+COUNTA('28th'!I42:I81)+COUNTA('29th'!I42:I81)+COUNTA('30th'!I42:I81)+COUNTA('31st'!I42:I81)</f>
+        <f>(COUNTA('1ST'!I42:I81)+COUNTA('2nd'!I42:I81)+COUNTA('3rd'!I42:I81)+COUNTA('4th'!I42:I81)+COUNTA('5th'!I42:I81)+COUNTA('6th'!I42:I81)+COUNTA('7th'!I42:I81)+COUNTA('8th'!I42:I81)+COUNTA('9th'!I42:I81)+COUNTA('10th'!I42:I81)+COUNTA('11th'!I42:I81)+COUNTA('12th'!I42:I81)+COUNTA('13th'!I42:I81)+COUNTA('14th'!I42:I81)+COUNTA('15th'!I42:I81)+COUNTA('16th'!I42:I81)+COUNTA('17th'!I42:I81)+COUNTA('18th'!I42:I81)+COUNTA('19th'!I42:I81)+COUNTA('20th'!I42:I81)+COUNTA('21st'!I42:I81)+COUNTA('22nd'!I42:I81)+COUNTA('23rd'!I42:I81)+COUNTA('24th'!I42:I81)+COUNTA('25th'!I42:I81)+COUNTA('26th'!I42:I81)+COUNTA('27th'!I42:I81)+COUNTA('28th'!I42:I81)+COUNTA('29th'!I42:I81)+COUNTA('30th'!I42:I81)+COUNTA('31st'!I42:I81))+0</f>
         <v/>
       </c>
       <c r="J3" s="2">
-        <f>COUNTA('1ST'!J42:J81)+COUNTA('2nd'!J42:J81)+COUNTA('3rd'!J42:J81)+COUNTA('4th'!J42:J81)+COUNTA('5th'!J42:J81)+COUNTA('6th'!J42:J81)+COUNTA('7th'!J42:J81)+COUNTA('8th'!J42:J81)+COUNTA('9th'!J42:J81)+COUNTA('10th'!J42:J81)+COUNTA('11th'!J42:J81)+COUNTA('12th'!J42:J81)+COUNTA('13th'!J42:J81)+COUNTA('14th'!J42:J81)+COUNTA('15th'!J42:J81)+COUNTA('16th'!J42:J81)+COUNTA('17th'!J42:J81)+COUNTA('18th'!J42:J81)+COUNTA('19th'!J42:J81)+COUNTA('20th'!J42:J81)+COUNTA('21st'!J42:J81)+COUNTA('22nd'!J42:J81)+COUNTA('23rd'!J42:J81)+COUNTA('24th'!J42:J81)+COUNTA('25th'!J42:J81)+COUNTA('26th'!J42:J81)+COUNTA('27th'!J42:J81)+COUNTA('28th'!J42:J81)+COUNTA('29th'!J42:J81)+COUNTA('30th'!J42:J81)+COUNTA('31st'!J42:J81)</f>
+        <f>(COUNTA('1ST'!J42:J81)+COUNTA('2nd'!J42:J81)+COUNTA('3rd'!J42:J81)+COUNTA('4th'!J42:J81)+COUNTA('5th'!J42:J81)+COUNTA('6th'!J42:J81)+COUNTA('7th'!J42:J81)+COUNTA('8th'!J42:J81)+COUNTA('9th'!J42:J81)+COUNTA('10th'!J42:J81)+COUNTA('11th'!J42:J81)+COUNTA('12th'!J42:J81)+COUNTA('13th'!J42:J81)+COUNTA('14th'!J42:J81)+COUNTA('15th'!J42:J81)+COUNTA('16th'!J42:J81)+COUNTA('17th'!J42:J81)+COUNTA('18th'!J42:J81)+COUNTA('19th'!J42:J81)+COUNTA('20th'!J42:J81)+COUNTA('21st'!J42:J81)+COUNTA('22nd'!J42:J81)+COUNTA('23rd'!J42:J81)+COUNTA('24th'!J42:J81)+COUNTA('25th'!J42:J81)+COUNTA('26th'!J42:J81)+COUNTA('27th'!J42:J81)+COUNTA('28th'!J42:J81)+COUNTA('29th'!J42:J81)+COUNTA('30th'!J42:J81)+COUNTA('31st'!J42:J81))+0</f>
         <v/>
       </c>
       <c r="K3" s="2">
-        <f>COUNTA('1ST'!K42:K81)+COUNTA('2nd'!K42:K81)+COUNTA('3rd'!K42:K81)+COUNTA('4th'!K42:K81)+COUNTA('5th'!K42:K81)+COUNTA('6th'!K42:K81)+COUNTA('7th'!K42:K81)+COUNTA('8th'!K42:K81)+COUNTA('9th'!K42:K81)+COUNTA('10th'!K42:K81)+COUNTA('11th'!K42:K81)+COUNTA('12th'!K42:K81)+COUNTA('13th'!K42:K81)+COUNTA('14th'!K42:K81)+COUNTA('15th'!K42:K81)+COUNTA('16th'!K42:K81)+COUNTA('17th'!K42:K81)+COUNTA('18th'!K42:K81)+COUNTA('19th'!K42:K81)+COUNTA('20th'!K42:K81)+COUNTA('21st'!K42:K81)+COUNTA('22nd'!K42:K81)+COUNTA('23rd'!K42:K81)+COUNTA('24th'!K42:K81)+COUNTA('25th'!K42:K81)+COUNTA('26th'!K42:K81)+COUNTA('27th'!K42:K81)+COUNTA('28th'!K42:K81)+COUNTA('29th'!K42:K81)+COUNTA('30th'!K42:K81)+COUNTA('31st'!K42:K81)</f>
+        <f>(COUNTA('1ST'!K42:K81)+COUNTA('2nd'!K42:K81)+COUNTA('3rd'!K42:K81)+COUNTA('4th'!K42:K81)+COUNTA('5th'!K42:K81)+COUNTA('6th'!K42:K81)+COUNTA('7th'!K42:K81)+COUNTA('8th'!K42:K81)+COUNTA('9th'!K42:K81)+COUNTA('10th'!K42:K81)+COUNTA('11th'!K42:K81)+COUNTA('12th'!K42:K81)+COUNTA('13th'!K42:K81)+COUNTA('14th'!K42:K81)+COUNTA('15th'!K42:K81)+COUNTA('16th'!K42:K81)+COUNTA('17th'!K42:K81)+COUNTA('18th'!K42:K81)+COUNTA('19th'!K42:K81)+COUNTA('20th'!K42:K81)+COUNTA('21st'!K42:K81)+COUNTA('22nd'!K42:K81)+COUNTA('23rd'!K42:K81)+COUNTA('24th'!K42:K81)+COUNTA('25th'!K42:K81)+COUNTA('26th'!K42:K81)+COUNTA('27th'!K42:K81)+COUNTA('28th'!K42:K81)+COUNTA('29th'!K42:K81)+COUNTA('30th'!K42:K81)+COUNTA('31st'!K42:K81))+0</f>
         <v/>
       </c>
       <c r="L3" s="2">
-        <f>COUNTA('1ST'!L42:L81)+COUNTA('2nd'!L42:L81)+COUNTA('3rd'!L42:L81)+COUNTA('4th'!L42:L81)+COUNTA('5th'!L42:L81)+COUNTA('6th'!L42:L81)+COUNTA('7th'!L42:L81)+COUNTA('8th'!L42:L81)+COUNTA('9th'!L42:L81)+COUNTA('10th'!L42:L81)+COUNTA('11th'!L42:L81)+COUNTA('12th'!L42:L81)+COUNTA('13th'!L42:L81)+COUNTA('14th'!L42:L81)+COUNTA('15th'!L42:L81)+COUNTA('16th'!L42:L81)+COUNTA('17th'!L42:L81)+COUNTA('18th'!L42:L81)+COUNTA('19th'!L42:L81)+COUNTA('20th'!L42:L81)+COUNTA('21st'!L42:L81)+COUNTA('22nd'!L42:L81)+COUNTA('23rd'!L42:L81)+COUNTA('24th'!L42:L81)+COUNTA('25th'!L42:L81)+COUNTA('26th'!L42:L81)+COUNTA('27th'!L42:L81)+COUNTA('28th'!L42:L81)+COUNTA('29th'!L42:L81)+COUNTA('30th'!L42:L81)+COUNTA('31st'!L42:L81)</f>
+        <f>(COUNTA('1ST'!L42:L81)+COUNTA('2nd'!L42:L81)+COUNTA('3rd'!L42:L81)+COUNTA('4th'!L42:L81)+COUNTA('5th'!L42:L81)+COUNTA('6th'!L42:L81)+COUNTA('7th'!L42:L81)+COUNTA('8th'!L42:L81)+COUNTA('9th'!L42:L81)+COUNTA('10th'!L42:L81)+COUNTA('11th'!L42:L81)+COUNTA('12th'!L42:L81)+COUNTA('13th'!L42:L81)+COUNTA('14th'!L42:L81)+COUNTA('15th'!L42:L81)+COUNTA('16th'!L42:L81)+COUNTA('17th'!L42:L81)+COUNTA('18th'!L42:L81)+COUNTA('19th'!L42:L81)+COUNTA('20th'!L42:L81)+COUNTA('21st'!L42:L81)+COUNTA('22nd'!L42:L81)+COUNTA('23rd'!L42:L81)+COUNTA('24th'!L42:L81)+COUNTA('25th'!L42:L81)+COUNTA('26th'!L42:L81)+COUNTA('27th'!L42:L81)+COUNTA('28th'!L42:L81)+COUNTA('29th'!L42:L81)+COUNTA('30th'!L42:L81)+COUNTA('31st'!L42:L81))+0</f>
         <v/>
       </c>
       <c r="M3" s="2">
-        <f>COUNTA('1ST'!M42:M81)+COUNTA('2nd'!M42:M81)+COUNTA('3rd'!M42:M81)+COUNTA('4th'!M42:M81)+COUNTA('5th'!M42:M81)+COUNTA('6th'!M42:M81)+COUNTA('7th'!M42:M81)+COUNTA('8th'!M42:M81)+COUNTA('9th'!M42:M81)+COUNTA('10th'!M42:M81)+COUNTA('11th'!M42:M81)+COUNTA('12th'!M42:M81)+COUNTA('13th'!M42:M81)+COUNTA('14th'!M42:M81)+COUNTA('15th'!M42:M81)+COUNTA('16th'!M42:M81)+COUNTA('17th'!M42:M81)+COUNTA('18th'!M42:M81)+COUNTA('19th'!M42:M81)+COUNTA('20th'!M42:M81)+COUNTA('21st'!M42:M81)+COUNTA('22nd'!M42:M81)+COUNTA('23rd'!M42:M81)+COUNTA('24th'!M42:M81)+COUNTA('25th'!M42:M81)+COUNTA('26th'!M42:M81)+COUNTA('27th'!M42:M81)+COUNTA('28th'!M42:M81)+COUNTA('29th'!M42:M81)+COUNTA('30th'!M42:M81)+COUNTA('31st'!M42:M81)</f>
+        <f>(COUNTA('1ST'!M42:M81)+COUNTA('2nd'!M42:M81)+COUNTA('3rd'!M42:M81)+COUNTA('4th'!M42:M81)+COUNTA('5th'!M42:M81)+COUNTA('6th'!M42:M81)+COUNTA('7th'!M42:M81)+COUNTA('8th'!M42:M81)+COUNTA('9th'!M42:M81)+COUNTA('10th'!M42:M81)+COUNTA('11th'!M42:M81)+COUNTA('12th'!M42:M81)+COUNTA('13th'!M42:M81)+COUNTA('14th'!M42:M81)+COUNTA('15th'!M42:M81)+COUNTA('16th'!M42:M81)+COUNTA('17th'!M42:M81)+COUNTA('18th'!M42:M81)+COUNTA('19th'!M42:M81)+COUNTA('20th'!M42:M81)+COUNTA('21st'!M42:M81)+COUNTA('22nd'!M42:M81)+COUNTA('23rd'!M42:M81)+COUNTA('24th'!M42:M81)+COUNTA('25th'!M42:M81)+COUNTA('26th'!M42:M81)+COUNTA('27th'!M42:M81)+COUNTA('28th'!M42:M81)+COUNTA('29th'!M42:M81)+COUNTA('30th'!M42:M81)+COUNTA('31st'!M42:M81))+0</f>
         <v/>
       </c>
       <c r="N3" s="2">
-        <f>COUNTA('1ST'!N42:N81)+COUNTA('2nd'!N42:N81)+COUNTA('3rd'!N42:N81)+COUNTA('4th'!N42:N81)+COUNTA('5th'!N42:N81)+COUNTA('6th'!N42:N81)+COUNTA('7th'!N42:N81)+COUNTA('8th'!N42:N81)+COUNTA('9th'!N42:N81)+COUNTA('10th'!N42:N81)+COUNTA('11th'!N42:N81)+COUNTA('12th'!N42:N81)+COUNTA('13th'!N42:N81)+COUNTA('14th'!N42:N81)+COUNTA('15th'!N42:N81)+COUNTA('16th'!N42:N81)+COUNTA('17th'!N42:N81)+COUNTA('18th'!N42:N81)+COUNTA('19th'!N42:N81)+COUNTA('20th'!N42:N81)+COUNTA('21st'!N42:N81)+COUNTA('22nd'!N42:N81)+COUNTA('23rd'!N42:N81)+COUNTA('24th'!N42:N81)+COUNTA('25th'!N42:N81)+COUNTA('26th'!N42:N81)+COUNTA('27th'!N42:N81)+COUNTA('28th'!N42:N81)+COUNTA('29th'!N42:N81)+COUNTA('30th'!N42:N81)+COUNTA('31st'!N42:N81)</f>
+        <f>(COUNTA('1ST'!N42:N81)+COUNTA('2nd'!N42:N81)+COUNTA('3rd'!N42:N81)+COUNTA('4th'!N42:N81)+COUNTA('5th'!N42:N81)+COUNTA('6th'!N42:N81)+COUNTA('7th'!N42:N81)+COUNTA('8th'!N42:N81)+COUNTA('9th'!N42:N81)+COUNTA('10th'!N42:N81)+COUNTA('11th'!N42:N81)+COUNTA('12th'!N42:N81)+COUNTA('13th'!N42:N81)+COUNTA('14th'!N42:N81)+COUNTA('15th'!N42:N81)+COUNTA('16th'!N42:N81)+COUNTA('17th'!N42:N81)+COUNTA('18th'!N42:N81)+COUNTA('19th'!N42:N81)+COUNTA('20th'!N42:N81)+COUNTA('21st'!N42:N81)+COUNTA('22nd'!N42:N81)+COUNTA('23rd'!N42:N81)+COUNTA('24th'!N42:N81)+COUNTA('25th'!N42:N81)+COUNTA('26th'!N42:N81)+COUNTA('27th'!N42:N81)+COUNTA('28th'!N42:N81)+COUNTA('29th'!N42:N81)+COUNTA('30th'!N42:N81)+COUNTA('31st'!N42:N81))+0</f>
         <v/>
       </c>
       <c r="O3" s="2">
-        <f>COUNTA('1ST'!O42:O81)+COUNTA('2nd'!O42:O81)+COUNTA('3rd'!O42:O81)+COUNTA('4th'!O42:O81)+COUNTA('5th'!O42:O81)+COUNTA('6th'!O42:O81)+COUNTA('7th'!O42:O81)+COUNTA('8th'!O42:O81)+COUNTA('9th'!O42:O81)+COUNTA('10th'!O42:O81)+COUNTA('11th'!O42:O81)+COUNTA('12th'!O42:O81)+COUNTA('13th'!O42:O81)+COUNTA('14th'!O42:O81)+COUNTA('15th'!O42:O81)+COUNTA('16th'!O42:O81)+COUNTA('17th'!O42:O81)+COUNTA('18th'!O42:O81)+COUNTA('19th'!O42:O81)+COUNTA('20th'!O42:O81)+COUNTA('21st'!O42:O81)+COUNTA('22nd'!O42:O81)+COUNTA('23rd'!O42:O81)+COUNTA('24th'!O42:O81)+COUNTA('25th'!O42:O81)+COUNTA('26th'!O42:O81)+COUNTA('27th'!O42:O81)+COUNTA('28th'!O42:O81)+COUNTA('29th'!O42:O81)+COUNTA('30th'!O42:O81)+COUNTA('31st'!O42:O81)</f>
+        <f>(COUNTA('1ST'!O42:O81)+COUNTA('2nd'!O42:O81)+COUNTA('3rd'!O42:O81)+COUNTA('4th'!O42:O81)+COUNTA('5th'!O42:O81)+COUNTA('6th'!O42:O81)+COUNTA('7th'!O42:O81)+COUNTA('8th'!O42:O81)+COUNTA('9th'!O42:O81)+COUNTA('10th'!O42:O81)+COUNTA('11th'!O42:O81)+COUNTA('12th'!O42:O81)+COUNTA('13th'!O42:O81)+COUNTA('14th'!O42:O81)+COUNTA('15th'!O42:O81)+COUNTA('16th'!O42:O81)+COUNTA('17th'!O42:O81)+COUNTA('18th'!O42:O81)+COUNTA('19th'!O42:O81)+COUNTA('20th'!O42:O81)+COUNTA('21st'!O42:O81)+COUNTA('22nd'!O42:O81)+COUNTA('23rd'!O42:O81)+COUNTA('24th'!O42:O81)+COUNTA('25th'!O42:O81)+COUNTA('26th'!O42:O81)+COUNTA('27th'!O42:O81)+COUNTA('28th'!O42:O81)+COUNTA('29th'!O42:O81)+COUNTA('30th'!O42:O81)+COUNTA('31st'!O42:O81))+0</f>
         <v/>
       </c>
       <c r="P3" s="2">
-        <f>COUNTA('1ST'!P42:P81)+COUNTA('2nd'!P42:P81)+COUNTA('3rd'!P42:P81)+COUNTA('4th'!P42:P81)+COUNTA('5th'!P42:P81)+COUNTA('6th'!P42:P81)+COUNTA('7th'!P42:P81)+COUNTA('8th'!P42:P81)+COUNTA('9th'!P42:P81)+COUNTA('10th'!P42:P81)+COUNTA('11th'!P42:P81)+COUNTA('12th'!P42:P81)+COUNTA('13th'!P42:P81)+COUNTA('14th'!P42:P81)+COUNTA('15th'!P42:P81)+COUNTA('16th'!P42:P81)+COUNTA('17th'!P42:P81)+COUNTA('18th'!P42:P81)+COUNTA('19th'!P42:P81)+COUNTA('20th'!P42:P81)+COUNTA('21st'!P42:P81)+COUNTA('22nd'!P42:P81)+COUNTA('23rd'!P42:P81)+COUNTA('24th'!P42:P81)+COUNTA('25th'!P42:P81)+COUNTA('26th'!P42:P81)+COUNTA('27th'!P42:P81)+COUNTA('28th'!P42:P81)+COUNTA('29th'!P42:P81)+COUNTA('30th'!P42:P81)+COUNTA('31st'!P42:P81)</f>
+        <f>(COUNTA('1ST'!P42:P81)+COUNTA('2nd'!P42:P81)+COUNTA('3rd'!P42:P81)+COUNTA('4th'!P42:P81)+COUNTA('5th'!P42:P81)+COUNTA('6th'!P42:P81)+COUNTA('7th'!P42:P81)+COUNTA('8th'!P42:P81)+COUNTA('9th'!P42:P81)+COUNTA('10th'!P42:P81)+COUNTA('11th'!P42:P81)+COUNTA('12th'!P42:P81)+COUNTA('13th'!P42:P81)+COUNTA('14th'!P42:P81)+COUNTA('15th'!P42:P81)+COUNTA('16th'!P42:P81)+COUNTA('17th'!P42:P81)+COUNTA('18th'!P42:P81)+COUNTA('19th'!P42:P81)+COUNTA('20th'!P42:P81)+COUNTA('21st'!P42:P81)+COUNTA('22nd'!P42:P81)+COUNTA('23rd'!P42:P81)+COUNTA('24th'!P42:P81)+COUNTA('25th'!P42:P81)+COUNTA('26th'!P42:P81)+COUNTA('27th'!P42:P81)+COUNTA('28th'!P42:P81)+COUNTA('29th'!P42:P81)+COUNTA('30th'!P42:P81)+COUNTA('31st'!P42:P81))+0</f>
         <v/>
       </c>
       <c r="Q3" s="2">
-        <f>COUNTA('1ST'!Q42:Q81)+COUNTA('2nd'!Q42:Q81)+COUNTA('3rd'!Q42:Q81)+COUNTA('4th'!Q42:Q81)+COUNTA('5th'!Q42:Q81)+COUNTA('6th'!Q42:Q81)+COUNTA('7th'!Q42:Q81)+COUNTA('8th'!Q42:Q81)+COUNTA('9th'!Q42:Q81)+COUNTA('10th'!Q42:Q81)+COUNTA('11th'!Q42:Q81)+COUNTA('12th'!Q42:Q81)+COUNTA('13th'!Q42:Q81)+COUNTA('14th'!Q42:Q81)+COUNTA('15th'!Q42:Q81)+COUNTA('16th'!Q42:Q81)+COUNTA('17th'!Q42:Q81)+COUNTA('18th'!Q42:Q81)+COUNTA('19th'!Q42:Q81)+COUNTA('20th'!Q42:Q81)+COUNTA('21st'!Q42:Q81)+COUNTA('22nd'!Q42:Q81)+COUNTA('23rd'!Q42:Q81)+COUNTA('24th'!Q42:Q81)+COUNTA('25th'!Q42:Q81)+COUNTA('26th'!Q42:Q81)+COUNTA('27th'!Q42:Q81)+COUNTA('28th'!Q42:Q81)+COUNTA('29th'!Q42:Q81)+COUNTA('30th'!Q42:Q81)+COUNTA('31st'!Q42:Q81)</f>
+        <f>(COUNTA('1ST'!Q42:Q81)+COUNTA('2nd'!Q42:Q81)+COUNTA('3rd'!Q42:Q81)+COUNTA('4th'!Q42:Q81)+COUNTA('5th'!Q42:Q81)+COUNTA('6th'!Q42:Q81)+COUNTA('7th'!Q42:Q81)+COUNTA('8th'!Q42:Q81)+COUNTA('9th'!Q42:Q81)+COUNTA('10th'!Q42:Q81)+COUNTA('11th'!Q42:Q81)+COUNTA('12th'!Q42:Q81)+COUNTA('13th'!Q42:Q81)+COUNTA('14th'!Q42:Q81)+COUNTA('15th'!Q42:Q81)+COUNTA('16th'!Q42:Q81)+COUNTA('17th'!Q42:Q81)+COUNTA('18th'!Q42:Q81)+COUNTA('19th'!Q42:Q81)+COUNTA('20th'!Q42:Q81)+COUNTA('21st'!Q42:Q81)+COUNTA('22nd'!Q42:Q81)+COUNTA('23rd'!Q42:Q81)+COUNTA('24th'!Q42:Q81)+COUNTA('25th'!Q42:Q81)+COUNTA('26th'!Q42:Q81)+COUNTA('27th'!Q42:Q81)+COUNTA('28th'!Q42:Q81)+COUNTA('29th'!Q42:Q81)+COUNTA('30th'!Q42:Q81)+COUNTA('31st'!Q42:Q81))+0</f>
         <v/>
       </c>
       <c r="R3" s="2">
-        <f>COUNTA('1ST'!R42:R81)+COUNTA('2nd'!R42:R81)+COUNTA('3rd'!R42:R81)+COUNTA('4th'!R42:R81)+COUNTA('5th'!R42:R81)+COUNTA('6th'!R42:R81)+COUNTA('7th'!R42:R81)+COUNTA('8th'!R42:R81)+COUNTA('9th'!R42:R81)+COUNTA('10th'!R42:R81)+COUNTA('11th'!R42:R81)+COUNTA('12th'!R42:R81)+COUNTA('13th'!R42:R81)+COUNTA('14th'!R42:R81)+COUNTA('15th'!R42:R81)+COUNTA('16th'!R42:R81)+COUNTA('17th'!R42:R81)+COUNTA('18th'!R42:R81)+COUNTA('19th'!R42:R81)+COUNTA('20th'!R42:R81)+COUNTA('21st'!R42:R81)+COUNTA('22nd'!R42:R81)+COUNTA('23rd'!R42:R81)+COUNTA('24th'!R42:R81)+COUNTA('25th'!R42:R81)+COUNTA('26th'!R42:R81)+COUNTA('27th'!R42:R81)+COUNTA('28th'!R42:R81)+COUNTA('29th'!R42:R81)+COUNTA('30th'!R42:R81)+COUNTA('31st'!R42:R81)</f>
+        <f>(COUNTA('1ST'!R42:R81)+COUNTA('2nd'!R42:R81)+COUNTA('3rd'!R42:R81)+COUNTA('4th'!R42:R81)+COUNTA('5th'!R42:R81)+COUNTA('6th'!R42:R81)+COUNTA('7th'!R42:R81)+COUNTA('8th'!R42:R81)+COUNTA('9th'!R42:R81)+COUNTA('10th'!R42:R81)+COUNTA('11th'!R42:R81)+COUNTA('12th'!R42:R81)+COUNTA('13th'!R42:R81)+COUNTA('14th'!R42:R81)+COUNTA('15th'!R42:R81)+COUNTA('16th'!R42:R81)+COUNTA('17th'!R42:R81)+COUNTA('18th'!R42:R81)+COUNTA('19th'!R42:R81)+COUNTA('20th'!R42:R81)+COUNTA('21st'!R42:R81)+COUNTA('22nd'!R42:R81)+COUNTA('23rd'!R42:R81)+COUNTA('24th'!R42:R81)+COUNTA('25th'!R42:R81)+COUNTA('26th'!R42:R81)+COUNTA('27th'!R42:R81)+COUNTA('28th'!R42:R81)+COUNTA('29th'!R42:R81)+COUNTA('30th'!R42:R81)+COUNTA('31st'!R42:R81))+0</f>
         <v/>
       </c>
       <c r="S3" s="2">
-        <f>COUNTA('1ST'!S42:S81)+COUNTA('2nd'!S42:S81)+COUNTA('3rd'!S42:S81)+COUNTA('4th'!S42:S81)+COUNTA('5th'!S42:S81)+COUNTA('6th'!S42:S81)+COUNTA('7th'!S42:S81)+COUNTA('8th'!S42:S81)+COUNTA('9th'!S42:S81)+COUNTA('10th'!S42:S81)+COUNTA('11th'!S42:S81)+COUNTA('12th'!S42:S81)+COUNTA('13th'!S42:S81)+COUNTA('14th'!S42:S81)+COUNTA('15th'!S42:S81)+COUNTA('16th'!S42:S81)+COUNTA('17th'!S42:S81)+COUNTA('18th'!S42:S81)+COUNTA('19th'!S42:S81)+COUNTA('20th'!S42:S81)+COUNTA('21st'!S42:S81)+COUNTA('22nd'!S42:S81)+COUNTA('23rd'!S42:S81)+COUNTA('24th'!S42:S81)+COUNTA('25th'!S42:S81)+COUNTA('26th'!S42:S81)+COUNTA('27th'!S42:S81)+COUNTA('28th'!S42:S81)+COUNTA('29th'!S42:S81)+COUNTA('30th'!S42:S81)+COUNTA('31st'!S42:S81)</f>
+        <f>(COUNTA('1ST'!S42:S81)+COUNTA('2nd'!S42:S81)+COUNTA('3rd'!S42:S81)+COUNTA('4th'!S42:S81)+COUNTA('5th'!S42:S81)+COUNTA('6th'!S42:S81)+COUNTA('7th'!S42:S81)+COUNTA('8th'!S42:S81)+COUNTA('9th'!S42:S81)+COUNTA('10th'!S42:S81)+COUNTA('11th'!S42:S81)+COUNTA('12th'!S42:S81)+COUNTA('13th'!S42:S81)+COUNTA('14th'!S42:S81)+COUNTA('15th'!S42:S81)+COUNTA('16th'!S42:S81)+COUNTA('17th'!S42:S81)+COUNTA('18th'!S42:S81)+COUNTA('19th'!S42:S81)+COUNTA('20th'!S42:S81)+COUNTA('21st'!S42:S81)+COUNTA('22nd'!S42:S81)+COUNTA('23rd'!S42:S81)+COUNTA('24th'!S42:S81)+COUNTA('25th'!S42:S81)+COUNTA('26th'!S42:S81)+COUNTA('27th'!S42:S81)+COUNTA('28th'!S42:S81)+COUNTA('29th'!S42:S81)+COUNTA('30th'!S42:S81)+COUNTA('31st'!S42:S81))+0</f>
         <v/>
       </c>
       <c r="T3" s="2">
-        <f>COUNTA('1ST'!T42:T81)+COUNTA('2nd'!T42:T81)+COUNTA('3rd'!T42:T81)+COUNTA('4th'!T42:T81)+COUNTA('5th'!T42:T81)+COUNTA('6th'!T42:T81)+COUNTA('7th'!T42:T81)+COUNTA('8th'!T42:T81)+COUNTA('9th'!T42:T81)+COUNTA('10th'!T42:T81)+COUNTA('11th'!T42:T81)+COUNTA('12th'!T42:T81)+COUNTA('13th'!T42:T81)+COUNTA('14th'!T42:T81)+COUNTA('15th'!T42:T81)+COUNTA('16th'!T42:T81)+COUNTA('17th'!T42:T81)+COUNTA('18th'!T42:T81)+COUNTA('19th'!T42:T81)+COUNTA('20th'!T42:T81)+COUNTA('21st'!T42:T81)+COUNTA('22nd'!T42:T81)+COUNTA('23rd'!T42:T81)+COUNTA('24th'!T42:T81)+COUNTA('25th'!T42:T81)+COUNTA('26th'!T42:T81)+COUNTA('27th'!T42:T81)+COUNTA('28th'!T42:T81)+COUNTA('29th'!T42:T81)+COUNTA('30th'!T42:T81)+COUNTA('31st'!T42:T81)</f>
+        <f>(COUNTA('1ST'!T42:T81)+COUNTA('2nd'!T42:T81)+COUNTA('3rd'!T42:T81)+COUNTA('4th'!T42:T81)+COUNTA('5th'!T42:T81)+COUNTA('6th'!T42:T81)+COUNTA('7th'!T42:T81)+COUNTA('8th'!T42:T81)+COUNTA('9th'!T42:T81)+COUNTA('10th'!T42:T81)+COUNTA('11th'!T42:T81)+COUNTA('12th'!T42:T81)+COUNTA('13th'!T42:T81)+COUNTA('14th'!T42:T81)+COUNTA('15th'!T42:T81)+COUNTA('16th'!T42:T81)+COUNTA('17th'!T42:T81)+COUNTA('18th'!T42:T81)+COUNTA('19th'!T42:T81)+COUNTA('20th'!T42:T81)+COUNTA('21st'!T42:T81)+COUNTA('22nd'!T42:T81)+COUNTA('23rd'!T42:T81)+COUNTA('24th'!T42:T81)+COUNTA('25th'!T42:T81)+COUNTA('26th'!T42:T81)+COUNTA('27th'!T42:T81)+COUNTA('28th'!T42:T81)+COUNTA('29th'!T42:T81)+COUNTA('30th'!T42:T81)+COUNTA('31st'!T42:T81))+0</f>
         <v/>
       </c>
       <c r="U3" s="2">
-        <f>COUNTA('1ST'!U42:U81)+COUNTA('2nd'!U42:U81)+COUNTA('3rd'!U42:U81)+COUNTA('4th'!U42:U81)+COUNTA('5th'!U42:U81)+COUNTA('6th'!U42:U81)+COUNTA('7th'!U42:U81)+COUNTA('8th'!U42:U81)+COUNTA('9th'!U42:U81)+COUNTA('10th'!U42:U81)+COUNTA('11th'!U42:U81)+COUNTA('12th'!U42:U81)+COUNTA('13th'!U42:U81)+COUNTA('14th'!U42:U81)+COUNTA('15th'!U42:U81)+COUNTA('16th'!U42:U81)+COUNTA('17th'!U42:U81)+COUNTA('18th'!U42:U81)+COUNTA('19th'!U42:U81)+COUNTA('20th'!U42:U81)+COUNTA('21st'!U42:U81)+COUNTA('22nd'!U42:U81)+COUNTA('23rd'!U42:U81)+COUNTA('24th'!U42:U81)+COUNTA('25th'!U42:U81)+COUNTA('26th'!U42:U81)+COUNTA('27th'!U42:U81)+COUNTA('28th'!U42:U81)+COUNTA('29th'!U42:U81)+COUNTA('30th'!U42:U81)+COUNTA('31st'!U42:U81)</f>
-        <v/>
-      </c>
-      <c r="W3" s="4" t="n">
+        <f>(COUNTA('1ST'!U42:U81)+COUNTA('2nd'!U42:U81)+COUNTA('3rd'!U42:U81)+COUNTA('4th'!U42:U81)+COUNTA('5th'!U42:U81)+COUNTA('6th'!U42:U81)+COUNTA('7th'!U42:U81)+COUNTA('8th'!U42:U81)+COUNTA('9th'!U42:U81)+COUNTA('10th'!U42:U81)+COUNTA('11th'!U42:U81)+COUNTA('12th'!U42:U81)+COUNTA('13th'!U42:U81)+COUNTA('14th'!U42:U81)+COUNTA('15th'!U42:U81)+COUNTA('16th'!U42:U81)+COUNTA('17th'!U42:U81)+COUNTA('18th'!U42:U81)+COUNTA('19th'!U42:U81)+COUNTA('20th'!U42:U81)+COUNTA('21st'!U42:U81)+COUNTA('22nd'!U42:U81)+COUNTA('23rd'!U42:U81)+COUNTA('24th'!U42:U81)+COUNTA('25th'!U42:U81)+COUNTA('26th'!U42:U81)+COUNTA('27th'!U42:U81)+COUNTA('28th'!U42:U81)+COUNTA('29th'!U42:U81)+COUNTA('30th'!U42:U81)+COUNTA('31st'!U42:U81))+0</f>
+        <v/>
+      </c>
+      <c r="W3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="AB3" s="4" t="n">
+      <c r="AB3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="AG3" s="4" t="n">
+      <c r="AG3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="AL3" s="4" t="n">
+      <c r="AL3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3560,91 +3592,91 @@
         </is>
       </c>
       <c r="C4" s="2">
-        <f>COUNTA('1ST'!C82:C121)+COUNTA('2nd'!C82:C121)+COUNTA('3rd'!C82:C121)+COUNTA('4th'!C82:C121)+COUNTA('5th'!C82:C121)+COUNTA('6th'!C82:C121)+COUNTA('7th'!C82:C121)+COUNTA('8th'!C82:C121)+COUNTA('9th'!C82:C121)+COUNTA('10th'!C82:C121)+COUNTA('11th'!C82:C121)+COUNTA('12th'!C82:C121)+COUNTA('13th'!C82:C121)+COUNTA('14th'!C82:C121)+COUNTA('15th'!C82:C121)+COUNTA('16th'!C82:C121)+COUNTA('17th'!C82:C121)+COUNTA('18th'!C82:C121)+COUNTA('19th'!C82:C121)+COUNTA('20th'!C82:C121)+COUNTA('21st'!C82:C121)+COUNTA('22nd'!C82:C121)+COUNTA('23rd'!C82:C121)+COUNTA('24th'!C82:C121)+COUNTA('25th'!C82:C121)+COUNTA('26th'!C82:C121)+COUNTA('27th'!C82:C121)+COUNTA('28th'!C82:C121)+COUNTA('29th'!C82:C121)+COUNTA('30th'!C82:C121)+COUNTA('31st'!C82:C121)</f>
+        <f>(COUNTA('1ST'!C82:C121)+COUNTA('2nd'!C82:C121)+COUNTA('3rd'!C82:C121)+COUNTA('4th'!C82:C121)+COUNTA('5th'!C82:C121)+COUNTA('6th'!C82:C121)+COUNTA('7th'!C82:C121)+COUNTA('8th'!C82:C121)+COUNTA('9th'!C82:C121)+COUNTA('10th'!C82:C121)+COUNTA('11th'!C82:C121)+COUNTA('12th'!C82:C121)+COUNTA('13th'!C82:C121)+COUNTA('14th'!C82:C121)+COUNTA('15th'!C82:C121)+COUNTA('16th'!C82:C121)+COUNTA('17th'!C82:C121)+COUNTA('18th'!C82:C121)+COUNTA('19th'!C82:C121)+COUNTA('20th'!C82:C121)+COUNTA('21st'!C82:C121)+COUNTA('22nd'!C82:C121)+COUNTA('23rd'!C82:C121)+COUNTA('24th'!C82:C121)+COUNTA('25th'!C82:C121)+COUNTA('26th'!C82:C121)+COUNTA('27th'!C82:C121)+COUNTA('28th'!C82:C121)+COUNTA('29th'!C82:C121)+COUNTA('30th'!C82:C121)+COUNTA('31st'!C82:C121))+0</f>
         <v/>
       </c>
       <c r="D4" s="2">
-        <f>COUNTA('1ST'!D82:D121)+COUNTA('2nd'!D82:D121)+COUNTA('3rd'!D82:D121)+COUNTA('4th'!D82:D121)+COUNTA('5th'!D82:D121)+COUNTA('6th'!D82:D121)+COUNTA('7th'!D82:D121)+COUNTA('8th'!D82:D121)+COUNTA('9th'!D82:D121)+COUNTA('10th'!D82:D121)+COUNTA('11th'!D82:D121)+COUNTA('12th'!D82:D121)+COUNTA('13th'!D82:D121)+COUNTA('14th'!D82:D121)+COUNTA('15th'!D82:D121)+COUNTA('16th'!D82:D121)+COUNTA('17th'!D82:D121)+COUNTA('18th'!D82:D121)+COUNTA('19th'!D82:D121)+COUNTA('20th'!D82:D121)+COUNTA('21st'!D82:D121)+COUNTA('22nd'!D82:D121)+COUNTA('23rd'!D82:D121)+COUNTA('24th'!D82:D121)+COUNTA('25th'!D82:D121)+COUNTA('26th'!D82:D121)+COUNTA('27th'!D82:D121)+COUNTA('28th'!D82:D121)+COUNTA('29th'!D82:D121)+COUNTA('30th'!D82:D121)+COUNTA('31st'!D82:D121)</f>
+        <f>(COUNTA('1ST'!D82:D121)+COUNTA('2nd'!D82:D121)+COUNTA('3rd'!D82:D121)+COUNTA('4th'!D82:D121)+COUNTA('5th'!D82:D121)+COUNTA('6th'!D82:D121)+COUNTA('7th'!D82:D121)+COUNTA('8th'!D82:D121)+COUNTA('9th'!D82:D121)+COUNTA('10th'!D82:D121)+COUNTA('11th'!D82:D121)+COUNTA('12th'!D82:D121)+COUNTA('13th'!D82:D121)+COUNTA('14th'!D82:D121)+COUNTA('15th'!D82:D121)+COUNTA('16th'!D82:D121)+COUNTA('17th'!D82:D121)+COUNTA('18th'!D82:D121)+COUNTA('19th'!D82:D121)+COUNTA('20th'!D82:D121)+COUNTA('21st'!D82:D121)+COUNTA('22nd'!D82:D121)+COUNTA('23rd'!D82:D121)+COUNTA('24th'!D82:D121)+COUNTA('25th'!D82:D121)+COUNTA('26th'!D82:D121)+COUNTA('27th'!D82:D121)+COUNTA('28th'!D82:D121)+COUNTA('29th'!D82:D121)+COUNTA('30th'!D82:D121)+COUNTA('31st'!D82:D121))+0</f>
         <v/>
       </c>
       <c r="E4" s="2">
-        <f>COUNTA('1ST'!E82:E121)+COUNTA('2nd'!E82:E121)+COUNTA('3rd'!E82:E121)+COUNTA('4th'!E82:E121)+COUNTA('5th'!E82:E121)+COUNTA('6th'!E82:E121)+COUNTA('7th'!E82:E121)+COUNTA('8th'!E82:E121)+COUNTA('9th'!E82:E121)+COUNTA('10th'!E82:E121)+COUNTA('11th'!E82:E121)+COUNTA('12th'!E82:E121)+COUNTA('13th'!E82:E121)+COUNTA('14th'!E82:E121)+COUNTA('15th'!E82:E121)+COUNTA('16th'!E82:E121)+COUNTA('17th'!E82:E121)+COUNTA('18th'!E82:E121)+COUNTA('19th'!E82:E121)+COUNTA('20th'!E82:E121)+COUNTA('21st'!E82:E121)+COUNTA('22nd'!E82:E121)+COUNTA('23rd'!E82:E121)+COUNTA('24th'!E82:E121)+COUNTA('25th'!E82:E121)+COUNTA('26th'!E82:E121)+COUNTA('27th'!E82:E121)+COUNTA('28th'!E82:E121)+COUNTA('29th'!E82:E121)+COUNTA('30th'!E82:E121)+COUNTA('31st'!E82:E121)</f>
+        <f>(COUNTA('1ST'!E82:E121)+COUNTA('2nd'!E82:E121)+COUNTA('3rd'!E82:E121)+COUNTA('4th'!E82:E121)+COUNTA('5th'!E82:E121)+COUNTA('6th'!E82:E121)+COUNTA('7th'!E82:E121)+COUNTA('8th'!E82:E121)+COUNTA('9th'!E82:E121)+COUNTA('10th'!E82:E121)+COUNTA('11th'!E82:E121)+COUNTA('12th'!E82:E121)+COUNTA('13th'!E82:E121)+COUNTA('14th'!E82:E121)+COUNTA('15th'!E82:E121)+COUNTA('16th'!E82:E121)+COUNTA('17th'!E82:E121)+COUNTA('18th'!E82:E121)+COUNTA('19th'!E82:E121)+COUNTA('20th'!E82:E121)+COUNTA('21st'!E82:E121)+COUNTA('22nd'!E82:E121)+COUNTA('23rd'!E82:E121)+COUNTA('24th'!E82:E121)+COUNTA('25th'!E82:E121)+COUNTA('26th'!E82:E121)+COUNTA('27th'!E82:E121)+COUNTA('28th'!E82:E121)+COUNTA('29th'!E82:E121)+COUNTA('30th'!E82:E121)+COUNTA('31st'!E82:E121))+0</f>
         <v/>
       </c>
       <c r="F4" s="2">
-        <f>COUNTA('1ST'!F82:F121)+COUNTA('2nd'!F82:F121)+COUNTA('3rd'!F82:F121)+COUNTA('4th'!F82:F121)+COUNTA('5th'!F82:F121)+COUNTA('6th'!F82:F121)+COUNTA('7th'!F82:F121)+COUNTA('8th'!F82:F121)+COUNTA('9th'!F82:F121)+COUNTA('10th'!F82:F121)+COUNTA('11th'!F82:F121)+COUNTA('12th'!F82:F121)+COUNTA('13th'!F82:F121)+COUNTA('14th'!F82:F121)+COUNTA('15th'!F82:F121)+COUNTA('16th'!F82:F121)+COUNTA('17th'!F82:F121)+COUNTA('18th'!F82:F121)+COUNTA('19th'!F82:F121)+COUNTA('20th'!F82:F121)+COUNTA('21st'!F82:F121)+COUNTA('22nd'!F82:F121)+COUNTA('23rd'!F82:F121)+COUNTA('24th'!F82:F121)+COUNTA('25th'!F82:F121)+COUNTA('26th'!F82:F121)+COUNTA('27th'!F82:F121)+COUNTA('28th'!F82:F121)+COUNTA('29th'!F82:F121)+COUNTA('30th'!F82:F121)+COUNTA('31st'!F82:F121)</f>
+        <f>(COUNTA('1ST'!F82:F121)+COUNTA('2nd'!F82:F121)+COUNTA('3rd'!F82:F121)+COUNTA('4th'!F82:F121)+COUNTA('5th'!F82:F121)+COUNTA('6th'!F82:F121)+COUNTA('7th'!F82:F121)+COUNTA('8th'!F82:F121)+COUNTA('9th'!F82:F121)+COUNTA('10th'!F82:F121)+COUNTA('11th'!F82:F121)+COUNTA('12th'!F82:F121)+COUNTA('13th'!F82:F121)+COUNTA('14th'!F82:F121)+COUNTA('15th'!F82:F121)+COUNTA('16th'!F82:F121)+COUNTA('17th'!F82:F121)+COUNTA('18th'!F82:F121)+COUNTA('19th'!F82:F121)+COUNTA('20th'!F82:F121)+COUNTA('21st'!F82:F121)+COUNTA('22nd'!F82:F121)+COUNTA('23rd'!F82:F121)+COUNTA('24th'!F82:F121)+COUNTA('25th'!F82:F121)+COUNTA('26th'!F82:F121)+COUNTA('27th'!F82:F121)+COUNTA('28th'!F82:F121)+COUNTA('29th'!F82:F121)+COUNTA('30th'!F82:F121)+COUNTA('31st'!F82:F121))+0</f>
         <v/>
       </c>
       <c r="G4" s="2">
-        <f>COUNTA('1ST'!G82:G121)+COUNTA('2nd'!G82:G121)+COUNTA('3rd'!G82:G121)+COUNTA('4th'!G82:G121)+COUNTA('5th'!G82:G121)+COUNTA('6th'!G82:G121)+COUNTA('7th'!G82:G121)+COUNTA('8th'!G82:G121)+COUNTA('9th'!G82:G121)+COUNTA('10th'!G82:G121)+COUNTA('11th'!G82:G121)+COUNTA('12th'!G82:G121)+COUNTA('13th'!G82:G121)+COUNTA('14th'!G82:G121)+COUNTA('15th'!G82:G121)+COUNTA('16th'!G82:G121)+COUNTA('17th'!G82:G121)+COUNTA('18th'!G82:G121)+COUNTA('19th'!G82:G121)+COUNTA('20th'!G82:G121)+COUNTA('21st'!G82:G121)+COUNTA('22nd'!G82:G121)+COUNTA('23rd'!G82:G121)+COUNTA('24th'!G82:G121)+COUNTA('25th'!G82:G121)+COUNTA('26th'!G82:G121)+COUNTA('27th'!G82:G121)+COUNTA('28th'!G82:G121)+COUNTA('29th'!G82:G121)+COUNTA('30th'!G82:G121)+COUNTA('31st'!G82:G121)</f>
+        <f>(COUNTA('1ST'!G82:G121)+COUNTA('2nd'!G82:G121)+COUNTA('3rd'!G82:G121)+COUNTA('4th'!G82:G121)+COUNTA('5th'!G82:G121)+COUNTA('6th'!G82:G121)+COUNTA('7th'!G82:G121)+COUNTA('8th'!G82:G121)+COUNTA('9th'!G82:G121)+COUNTA('10th'!G82:G121)+COUNTA('11th'!G82:G121)+COUNTA('12th'!G82:G121)+COUNTA('13th'!G82:G121)+COUNTA('14th'!G82:G121)+COUNTA('15th'!G82:G121)+COUNTA('16th'!G82:G121)+COUNTA('17th'!G82:G121)+COUNTA('18th'!G82:G121)+COUNTA('19th'!G82:G121)+COUNTA('20th'!G82:G121)+COUNTA('21st'!G82:G121)+COUNTA('22nd'!G82:G121)+COUNTA('23rd'!G82:G121)+COUNTA('24th'!G82:G121)+COUNTA('25th'!G82:G121)+COUNTA('26th'!G82:G121)+COUNTA('27th'!G82:G121)+COUNTA('28th'!G82:G121)+COUNTA('29th'!G82:G121)+COUNTA('30th'!G82:G121)+COUNTA('31st'!G82:G121))+0</f>
         <v/>
       </c>
       <c r="H4" s="2">
-        <f>COUNTA('1ST'!H82:H121)+COUNTA('2nd'!H82:H121)+COUNTA('3rd'!H82:H121)+COUNTA('4th'!H82:H121)+COUNTA('5th'!H82:H121)+COUNTA('6th'!H82:H121)+COUNTA('7th'!H82:H121)+COUNTA('8th'!H82:H121)+COUNTA('9th'!H82:H121)+COUNTA('10th'!H82:H121)+COUNTA('11th'!H82:H121)+COUNTA('12th'!H82:H121)+COUNTA('13th'!H82:H121)+COUNTA('14th'!H82:H121)+COUNTA('15th'!H82:H121)+COUNTA('16th'!H82:H121)+COUNTA('17th'!H82:H121)+COUNTA('18th'!H82:H121)+COUNTA('19th'!H82:H121)+COUNTA('20th'!H82:H121)+COUNTA('21st'!H82:H121)+COUNTA('22nd'!H82:H121)+COUNTA('23rd'!H82:H121)+COUNTA('24th'!H82:H121)+COUNTA('25th'!H82:H121)+COUNTA('26th'!H82:H121)+COUNTA('27th'!H82:H121)+COUNTA('28th'!H82:H121)+COUNTA('29th'!H82:H121)+COUNTA('30th'!H82:H121)+COUNTA('31st'!H82:H121)</f>
+        <f>(COUNTA('1ST'!H82:H121)+COUNTA('2nd'!H82:H121)+COUNTA('3rd'!H82:H121)+COUNTA('4th'!H82:H121)+COUNTA('5th'!H82:H121)+COUNTA('6th'!H82:H121)+COUNTA('7th'!H82:H121)+COUNTA('8th'!H82:H121)+COUNTA('9th'!H82:H121)+COUNTA('10th'!H82:H121)+COUNTA('11th'!H82:H121)+COUNTA('12th'!H82:H121)+COUNTA('13th'!H82:H121)+COUNTA('14th'!H82:H121)+COUNTA('15th'!H82:H121)+COUNTA('16th'!H82:H121)+COUNTA('17th'!H82:H121)+COUNTA('18th'!H82:H121)+COUNTA('19th'!H82:H121)+COUNTA('20th'!H82:H121)+COUNTA('21st'!H82:H121)+COUNTA('22nd'!H82:H121)+COUNTA('23rd'!H82:H121)+COUNTA('24th'!H82:H121)+COUNTA('25th'!H82:H121)+COUNTA('26th'!H82:H121)+COUNTA('27th'!H82:H121)+COUNTA('28th'!H82:H121)+COUNTA('29th'!H82:H121)+COUNTA('30th'!H82:H121)+COUNTA('31st'!H82:H121))+0</f>
         <v/>
       </c>
       <c r="I4" s="2">
-        <f>COUNTA('1ST'!I82:I121)+COUNTA('2nd'!I82:I121)+COUNTA('3rd'!I82:I121)+COUNTA('4th'!I82:I121)+COUNTA('5th'!I82:I121)+COUNTA('6th'!I82:I121)+COUNTA('7th'!I82:I121)+COUNTA('8th'!I82:I121)+COUNTA('9th'!I82:I121)+COUNTA('10th'!I82:I121)+COUNTA('11th'!I82:I121)+COUNTA('12th'!I82:I121)+COUNTA('13th'!I82:I121)+COUNTA('14th'!I82:I121)+COUNTA('15th'!I82:I121)+COUNTA('16th'!I82:I121)+COUNTA('17th'!I82:I121)+COUNTA('18th'!I82:I121)+COUNTA('19th'!I82:I121)+COUNTA('20th'!I82:I121)+COUNTA('21st'!I82:I121)+COUNTA('22nd'!I82:I121)+COUNTA('23rd'!I82:I121)+COUNTA('24th'!I82:I121)+COUNTA('25th'!I82:I121)+COUNTA('26th'!I82:I121)+COUNTA('27th'!I82:I121)+COUNTA('28th'!I82:I121)+COUNTA('29th'!I82:I121)+COUNTA('30th'!I82:I121)+COUNTA('31st'!I82:I121)</f>
+        <f>(COUNTA('1ST'!I82:I121)+COUNTA('2nd'!I82:I121)+COUNTA('3rd'!I82:I121)+COUNTA('4th'!I82:I121)+COUNTA('5th'!I82:I121)+COUNTA('6th'!I82:I121)+COUNTA('7th'!I82:I121)+COUNTA('8th'!I82:I121)+COUNTA('9th'!I82:I121)+COUNTA('10th'!I82:I121)+COUNTA('11th'!I82:I121)+COUNTA('12th'!I82:I121)+COUNTA('13th'!I82:I121)+COUNTA('14th'!I82:I121)+COUNTA('15th'!I82:I121)+COUNTA('16th'!I82:I121)+COUNTA('17th'!I82:I121)+COUNTA('18th'!I82:I121)+COUNTA('19th'!I82:I121)+COUNTA('20th'!I82:I121)+COUNTA('21st'!I82:I121)+COUNTA('22nd'!I82:I121)+COUNTA('23rd'!I82:I121)+COUNTA('24th'!I82:I121)+COUNTA('25th'!I82:I121)+COUNTA('26th'!I82:I121)+COUNTA('27th'!I82:I121)+COUNTA('28th'!I82:I121)+COUNTA('29th'!I82:I121)+COUNTA('30th'!I82:I121)+COUNTA('31st'!I82:I121))+0</f>
         <v/>
       </c>
       <c r="J4" s="2">
-        <f>COUNTA('1ST'!J82:J121)+COUNTA('2nd'!J82:J121)+COUNTA('3rd'!J82:J121)+COUNTA('4th'!J82:J121)+COUNTA('5th'!J82:J121)+COUNTA('6th'!J82:J121)+COUNTA('7th'!J82:J121)+COUNTA('8th'!J82:J121)+COUNTA('9th'!J82:J121)+COUNTA('10th'!J82:J121)+COUNTA('11th'!J82:J121)+COUNTA('12th'!J82:J121)+COUNTA('13th'!J82:J121)+COUNTA('14th'!J82:J121)+COUNTA('15th'!J82:J121)+COUNTA('16th'!J82:J121)+COUNTA('17th'!J82:J121)+COUNTA('18th'!J82:J121)+COUNTA('19th'!J82:J121)+COUNTA('20th'!J82:J121)+COUNTA('21st'!J82:J121)+COUNTA('22nd'!J82:J121)+COUNTA('23rd'!J82:J121)+COUNTA('24th'!J82:J121)+COUNTA('25th'!J82:J121)+COUNTA('26th'!J82:J121)+COUNTA('27th'!J82:J121)+COUNTA('28th'!J82:J121)+COUNTA('29th'!J82:J121)+COUNTA('30th'!J82:J121)+COUNTA('31st'!J82:J121)</f>
+        <f>(COUNTA('1ST'!J82:J121)+COUNTA('2nd'!J82:J121)+COUNTA('3rd'!J82:J121)+COUNTA('4th'!J82:J121)+COUNTA('5th'!J82:J121)+COUNTA('6th'!J82:J121)+COUNTA('7th'!J82:J121)+COUNTA('8th'!J82:J121)+COUNTA('9th'!J82:J121)+COUNTA('10th'!J82:J121)+COUNTA('11th'!J82:J121)+COUNTA('12th'!J82:J121)+COUNTA('13th'!J82:J121)+COUNTA('14th'!J82:J121)+COUNTA('15th'!J82:J121)+COUNTA('16th'!J82:J121)+COUNTA('17th'!J82:J121)+COUNTA('18th'!J82:J121)+COUNTA('19th'!J82:J121)+COUNTA('20th'!J82:J121)+COUNTA('21st'!J82:J121)+COUNTA('22nd'!J82:J121)+COUNTA('23rd'!J82:J121)+COUNTA('24th'!J82:J121)+COUNTA('25th'!J82:J121)+COUNTA('26th'!J82:J121)+COUNTA('27th'!J82:J121)+COUNTA('28th'!J82:J121)+COUNTA('29th'!J82:J121)+COUNTA('30th'!J82:J121)+COUNTA('31st'!J82:J121))+0</f>
         <v/>
       </c>
       <c r="K4" s="2">
-        <f>COUNTA('1ST'!K82:K121)+COUNTA('2nd'!K82:K121)+COUNTA('3rd'!K82:K121)+COUNTA('4th'!K82:K121)+COUNTA('5th'!K82:K121)+COUNTA('6th'!K82:K121)+COUNTA('7th'!K82:K121)+COUNTA('8th'!K82:K121)+COUNTA('9th'!K82:K121)+COUNTA('10th'!K82:K121)+COUNTA('11th'!K82:K121)+COUNTA('12th'!K82:K121)+COUNTA('13th'!K82:K121)+COUNTA('14th'!K82:K121)+COUNTA('15th'!K82:K121)+COUNTA('16th'!K82:K121)+COUNTA('17th'!K82:K121)+COUNTA('18th'!K82:K121)+COUNTA('19th'!K82:K121)+COUNTA('20th'!K82:K121)+COUNTA('21st'!K82:K121)+COUNTA('22nd'!K82:K121)+COUNTA('23rd'!K82:K121)+COUNTA('24th'!K82:K121)+COUNTA('25th'!K82:K121)+COUNTA('26th'!K82:K121)+COUNTA('27th'!K82:K121)+COUNTA('28th'!K82:K121)+COUNTA('29th'!K82:K121)+COUNTA('30th'!K82:K121)+COUNTA('31st'!K82:K121)</f>
+        <f>(COUNTA('1ST'!K82:K121)+COUNTA('2nd'!K82:K121)+COUNTA('3rd'!K82:K121)+COUNTA('4th'!K82:K121)+COUNTA('5th'!K82:K121)+COUNTA('6th'!K82:K121)+COUNTA('7th'!K82:K121)+COUNTA('8th'!K82:K121)+COUNTA('9th'!K82:K121)+COUNTA('10th'!K82:K121)+COUNTA('11th'!K82:K121)+COUNTA('12th'!K82:K121)+COUNTA('13th'!K82:K121)+COUNTA('14th'!K82:K121)+COUNTA('15th'!K82:K121)+COUNTA('16th'!K82:K121)+COUNTA('17th'!K82:K121)+COUNTA('18th'!K82:K121)+COUNTA('19th'!K82:K121)+COUNTA('20th'!K82:K121)+COUNTA('21st'!K82:K121)+COUNTA('22nd'!K82:K121)+COUNTA('23rd'!K82:K121)+COUNTA('24th'!K82:K121)+COUNTA('25th'!K82:K121)+COUNTA('26th'!K82:K121)+COUNTA('27th'!K82:K121)+COUNTA('28th'!K82:K121)+COUNTA('29th'!K82:K121)+COUNTA('30th'!K82:K121)+COUNTA('31st'!K82:K121))+0</f>
         <v/>
       </c>
       <c r="L4" s="2">
-        <f>COUNTA('1ST'!L82:L121)+COUNTA('2nd'!L82:L121)+COUNTA('3rd'!L82:L121)+COUNTA('4th'!L82:L121)+COUNTA('5th'!L82:L121)+COUNTA('6th'!L82:L121)+COUNTA('7th'!L82:L121)+COUNTA('8th'!L82:L121)+COUNTA('9th'!L82:L121)+COUNTA('10th'!L82:L121)+COUNTA('11th'!L82:L121)+COUNTA('12th'!L82:L121)+COUNTA('13th'!L82:L121)+COUNTA('14th'!L82:L121)+COUNTA('15th'!L82:L121)+COUNTA('16th'!L82:L121)+COUNTA('17th'!L82:L121)+COUNTA('18th'!L82:L121)+COUNTA('19th'!L82:L121)+COUNTA('20th'!L82:L121)+COUNTA('21st'!L82:L121)+COUNTA('22nd'!L82:L121)+COUNTA('23rd'!L82:L121)+COUNTA('24th'!L82:L121)+COUNTA('25th'!L82:L121)+COUNTA('26th'!L82:L121)+COUNTA('27th'!L82:L121)+COUNTA('28th'!L82:L121)+COUNTA('29th'!L82:L121)+COUNTA('30th'!L82:L121)+COUNTA('31st'!L82:L121)</f>
+        <f>(COUNTA('1ST'!L82:L121)+COUNTA('2nd'!L82:L121)+COUNTA('3rd'!L82:L121)+COUNTA('4th'!L82:L121)+COUNTA('5th'!L82:L121)+COUNTA('6th'!L82:L121)+COUNTA('7th'!L82:L121)+COUNTA('8th'!L82:L121)+COUNTA('9th'!L82:L121)+COUNTA('10th'!L82:L121)+COUNTA('11th'!L82:L121)+COUNTA('12th'!L82:L121)+COUNTA('13th'!L82:L121)+COUNTA('14th'!L82:L121)+COUNTA('15th'!L82:L121)+COUNTA('16th'!L82:L121)+COUNTA('17th'!L82:L121)+COUNTA('18th'!L82:L121)+COUNTA('19th'!L82:L121)+COUNTA('20th'!L82:L121)+COUNTA('21st'!L82:L121)+COUNTA('22nd'!L82:L121)+COUNTA('23rd'!L82:L121)+COUNTA('24th'!L82:L121)+COUNTA('25th'!L82:L121)+COUNTA('26th'!L82:L121)+COUNTA('27th'!L82:L121)+COUNTA('28th'!L82:L121)+COUNTA('29th'!L82:L121)+COUNTA('30th'!L82:L121)+COUNTA('31st'!L82:L121))+0</f>
         <v/>
       </c>
       <c r="M4" s="2">
-        <f>COUNTA('1ST'!M82:M121)+COUNTA('2nd'!M82:M121)+COUNTA('3rd'!M82:M121)+COUNTA('4th'!M82:M121)+COUNTA('5th'!M82:M121)+COUNTA('6th'!M82:M121)+COUNTA('7th'!M82:M121)+COUNTA('8th'!M82:M121)+COUNTA('9th'!M82:M121)+COUNTA('10th'!M82:M121)+COUNTA('11th'!M82:M121)+COUNTA('12th'!M82:M121)+COUNTA('13th'!M82:M121)+COUNTA('14th'!M82:M121)+COUNTA('15th'!M82:M121)+COUNTA('16th'!M82:M121)+COUNTA('17th'!M82:M121)+COUNTA('18th'!M82:M121)+COUNTA('19th'!M82:M121)+COUNTA('20th'!M82:M121)+COUNTA('21st'!M82:M121)+COUNTA('22nd'!M82:M121)+COUNTA('23rd'!M82:M121)+COUNTA('24th'!M82:M121)+COUNTA('25th'!M82:M121)+COUNTA('26th'!M82:M121)+COUNTA('27th'!M82:M121)+COUNTA('28th'!M82:M121)+COUNTA('29th'!M82:M121)+COUNTA('30th'!M82:M121)+COUNTA('31st'!M82:M121)</f>
+        <f>(COUNTA('1ST'!M82:M121)+COUNTA('2nd'!M82:M121)+COUNTA('3rd'!M82:M121)+COUNTA('4th'!M82:M121)+COUNTA('5th'!M82:M121)+COUNTA('6th'!M82:M121)+COUNTA('7th'!M82:M121)+COUNTA('8th'!M82:M121)+COUNTA('9th'!M82:M121)+COUNTA('10th'!M82:M121)+COUNTA('11th'!M82:M121)+COUNTA('12th'!M82:M121)+COUNTA('13th'!M82:M121)+COUNTA('14th'!M82:M121)+COUNTA('15th'!M82:M121)+COUNTA('16th'!M82:M121)+COUNTA('17th'!M82:M121)+COUNTA('18th'!M82:M121)+COUNTA('19th'!M82:M121)+COUNTA('20th'!M82:M121)+COUNTA('21st'!M82:M121)+COUNTA('22nd'!M82:M121)+COUNTA('23rd'!M82:M121)+COUNTA('24th'!M82:M121)+COUNTA('25th'!M82:M121)+COUNTA('26th'!M82:M121)+COUNTA('27th'!M82:M121)+COUNTA('28th'!M82:M121)+COUNTA('29th'!M82:M121)+COUNTA('30th'!M82:M121)+COUNTA('31st'!M82:M121))+0</f>
         <v/>
       </c>
       <c r="N4" s="2">
-        <f>COUNTA('1ST'!N82:N121)+COUNTA('2nd'!N82:N121)+COUNTA('3rd'!N82:N121)+COUNTA('4th'!N82:N121)+COUNTA('5th'!N82:N121)+COUNTA('6th'!N82:N121)+COUNTA('7th'!N82:N121)+COUNTA('8th'!N82:N121)+COUNTA('9th'!N82:N121)+COUNTA('10th'!N82:N121)+COUNTA('11th'!N82:N121)+COUNTA('12th'!N82:N121)+COUNTA('13th'!N82:N121)+COUNTA('14th'!N82:N121)+COUNTA('15th'!N82:N121)+COUNTA('16th'!N82:N121)+COUNTA('17th'!N82:N121)+COUNTA('18th'!N82:N121)+COUNTA('19th'!N82:N121)+COUNTA('20th'!N82:N121)+COUNTA('21st'!N82:N121)+COUNTA('22nd'!N82:N121)+COUNTA('23rd'!N82:N121)+COUNTA('24th'!N82:N121)+COUNTA('25th'!N82:N121)+COUNTA('26th'!N82:N121)+COUNTA('27th'!N82:N121)+COUNTA('28th'!N82:N121)+COUNTA('29th'!N82:N121)+COUNTA('30th'!N82:N121)+COUNTA('31st'!N82:N121)</f>
+        <f>(COUNTA('1ST'!N82:N121)+COUNTA('2nd'!N82:N121)+COUNTA('3rd'!N82:N121)+COUNTA('4th'!N82:N121)+COUNTA('5th'!N82:N121)+COUNTA('6th'!N82:N121)+COUNTA('7th'!N82:N121)+COUNTA('8th'!N82:N121)+COUNTA('9th'!N82:N121)+COUNTA('10th'!N82:N121)+COUNTA('11th'!N82:N121)+COUNTA('12th'!N82:N121)+COUNTA('13th'!N82:N121)+COUNTA('14th'!N82:N121)+COUNTA('15th'!N82:N121)+COUNTA('16th'!N82:N121)+COUNTA('17th'!N82:N121)+COUNTA('18th'!N82:N121)+COUNTA('19th'!N82:N121)+COUNTA('20th'!N82:N121)+COUNTA('21st'!N82:N121)+COUNTA('22nd'!N82:N121)+COUNTA('23rd'!N82:N121)+COUNTA('24th'!N82:N121)+COUNTA('25th'!N82:N121)+COUNTA('26th'!N82:N121)+COUNTA('27th'!N82:N121)+COUNTA('28th'!N82:N121)+COUNTA('29th'!N82:N121)+COUNTA('30th'!N82:N121)+COUNTA('31st'!N82:N121))+0</f>
         <v/>
       </c>
       <c r="O4" s="2">
-        <f>COUNTA('1ST'!O82:O121)+COUNTA('2nd'!O82:O121)+COUNTA('3rd'!O82:O121)+COUNTA('4th'!O82:O121)+COUNTA('5th'!O82:O121)+COUNTA('6th'!O82:O121)+COUNTA('7th'!O82:O121)+COUNTA('8th'!O82:O121)+COUNTA('9th'!O82:O121)+COUNTA('10th'!O82:O121)+COUNTA('11th'!O82:O121)+COUNTA('12th'!O82:O121)+COUNTA('13th'!O82:O121)+COUNTA('14th'!O82:O121)+COUNTA('15th'!O82:O121)+COUNTA('16th'!O82:O121)+COUNTA('17th'!O82:O121)+COUNTA('18th'!O82:O121)+COUNTA('19th'!O82:O121)+COUNTA('20th'!O82:O121)+COUNTA('21st'!O82:O121)+COUNTA('22nd'!O82:O121)+COUNTA('23rd'!O82:O121)+COUNTA('24th'!O82:O121)+COUNTA('25th'!O82:O121)+COUNTA('26th'!O82:O121)+COUNTA('27th'!O82:O121)+COUNTA('28th'!O82:O121)+COUNTA('29th'!O82:O121)+COUNTA('30th'!O82:O121)+COUNTA('31st'!O82:O121)</f>
+        <f>(COUNTA('1ST'!O82:O121)+COUNTA('2nd'!O82:O121)+COUNTA('3rd'!O82:O121)+COUNTA('4th'!O82:O121)+COUNTA('5th'!O82:O121)+COUNTA('6th'!O82:O121)+COUNTA('7th'!O82:O121)+COUNTA('8th'!O82:O121)+COUNTA('9th'!O82:O121)+COUNTA('10th'!O82:O121)+COUNTA('11th'!O82:O121)+COUNTA('12th'!O82:O121)+COUNTA('13th'!O82:O121)+COUNTA('14th'!O82:O121)+COUNTA('15th'!O82:O121)+COUNTA('16th'!O82:O121)+COUNTA('17th'!O82:O121)+COUNTA('18th'!O82:O121)+COUNTA('19th'!O82:O121)+COUNTA('20th'!O82:O121)+COUNTA('21st'!O82:O121)+COUNTA('22nd'!O82:O121)+COUNTA('23rd'!O82:O121)+COUNTA('24th'!O82:O121)+COUNTA('25th'!O82:O121)+COUNTA('26th'!O82:O121)+COUNTA('27th'!O82:O121)+COUNTA('28th'!O82:O121)+COUNTA('29th'!O82:O121)+COUNTA('30th'!O82:O121)+COUNTA('31st'!O82:O121))+0</f>
         <v/>
       </c>
       <c r="P4" s="2">
-        <f>COUNTA('1ST'!P82:P121)+COUNTA('2nd'!P82:P121)+COUNTA('3rd'!P82:P121)+COUNTA('4th'!P82:P121)+COUNTA('5th'!P82:P121)+COUNTA('6th'!P82:P121)+COUNTA('7th'!P82:P121)+COUNTA('8th'!P82:P121)+COUNTA('9th'!P82:P121)+COUNTA('10th'!P82:P121)+COUNTA('11th'!P82:P121)+COUNTA('12th'!P82:P121)+COUNTA('13th'!P82:P121)+COUNTA('14th'!P82:P121)+COUNTA('15th'!P82:P121)+COUNTA('16th'!P82:P121)+COUNTA('17th'!P82:P121)+COUNTA('18th'!P82:P121)+COUNTA('19th'!P82:P121)+COUNTA('20th'!P82:P121)+COUNTA('21st'!P82:P121)+COUNTA('22nd'!P82:P121)+COUNTA('23rd'!P82:P121)+COUNTA('24th'!P82:P121)+COUNTA('25th'!P82:P121)+COUNTA('26th'!P82:P121)+COUNTA('27th'!P82:P121)+COUNTA('28th'!P82:P121)+COUNTA('29th'!P82:P121)+COUNTA('30th'!P82:P121)+COUNTA('31st'!P82:P121)</f>
+        <f>(COUNTA('1ST'!P82:P121)+COUNTA('2nd'!P82:P121)+COUNTA('3rd'!P82:P121)+COUNTA('4th'!P82:P121)+COUNTA('5th'!P82:P121)+COUNTA('6th'!P82:P121)+COUNTA('7th'!P82:P121)+COUNTA('8th'!P82:P121)+COUNTA('9th'!P82:P121)+COUNTA('10th'!P82:P121)+COUNTA('11th'!P82:P121)+COUNTA('12th'!P82:P121)+COUNTA('13th'!P82:P121)+COUNTA('14th'!P82:P121)+COUNTA('15th'!P82:P121)+COUNTA('16th'!P82:P121)+COUNTA('17th'!P82:P121)+COUNTA('18th'!P82:P121)+COUNTA('19th'!P82:P121)+COUNTA('20th'!P82:P121)+COUNTA('21st'!P82:P121)+COUNTA('22nd'!P82:P121)+COUNTA('23rd'!P82:P121)+COUNTA('24th'!P82:P121)+COUNTA('25th'!P82:P121)+COUNTA('26th'!P82:P121)+COUNTA('27th'!P82:P121)+COUNTA('28th'!P82:P121)+COUNTA('29th'!P82:P121)+COUNTA('30th'!P82:P121)+COUNTA('31st'!P82:P121))+0</f>
         <v/>
       </c>
       <c r="Q4" s="2">
-        <f>COUNTA('1ST'!Q82:Q121)+COUNTA('2nd'!Q82:Q121)+COUNTA('3rd'!Q82:Q121)+COUNTA('4th'!Q82:Q121)+COUNTA('5th'!Q82:Q121)+COUNTA('6th'!Q82:Q121)+COUNTA('7th'!Q82:Q121)+COUNTA('8th'!Q82:Q121)+COUNTA('9th'!Q82:Q121)+COUNTA('10th'!Q82:Q121)+COUNTA('11th'!Q82:Q121)+COUNTA('12th'!Q82:Q121)+COUNTA('13th'!Q82:Q121)+COUNTA('14th'!Q82:Q121)+COUNTA('15th'!Q82:Q121)+COUNTA('16th'!Q82:Q121)+COUNTA('17th'!Q82:Q121)+COUNTA('18th'!Q82:Q121)+COUNTA('19th'!Q82:Q121)+COUNTA('20th'!Q82:Q121)+COUNTA('21st'!Q82:Q121)+COUNTA('22nd'!Q82:Q121)+COUNTA('23rd'!Q82:Q121)+COUNTA('24th'!Q82:Q121)+COUNTA('25th'!Q82:Q121)+COUNTA('26th'!Q82:Q121)+COUNTA('27th'!Q82:Q121)+COUNTA('28th'!Q82:Q121)+COUNTA('29th'!Q82:Q121)+COUNTA('30th'!Q82:Q121)+COUNTA('31st'!Q82:Q121)</f>
+        <f>(COUNTA('1ST'!Q82:Q121)+COUNTA('2nd'!Q82:Q121)+COUNTA('3rd'!Q82:Q121)+COUNTA('4th'!Q82:Q121)+COUNTA('5th'!Q82:Q121)+COUNTA('6th'!Q82:Q121)+COUNTA('7th'!Q82:Q121)+COUNTA('8th'!Q82:Q121)+COUNTA('9th'!Q82:Q121)+COUNTA('10th'!Q82:Q121)+COUNTA('11th'!Q82:Q121)+COUNTA('12th'!Q82:Q121)+COUNTA('13th'!Q82:Q121)+COUNTA('14th'!Q82:Q121)+COUNTA('15th'!Q82:Q121)+COUNTA('16th'!Q82:Q121)+COUNTA('17th'!Q82:Q121)+COUNTA('18th'!Q82:Q121)+COUNTA('19th'!Q82:Q121)+COUNTA('20th'!Q82:Q121)+COUNTA('21st'!Q82:Q121)+COUNTA('22nd'!Q82:Q121)+COUNTA('23rd'!Q82:Q121)+COUNTA('24th'!Q82:Q121)+COUNTA('25th'!Q82:Q121)+COUNTA('26th'!Q82:Q121)+COUNTA('27th'!Q82:Q121)+COUNTA('28th'!Q82:Q121)+COUNTA('29th'!Q82:Q121)+COUNTA('30th'!Q82:Q121)+COUNTA('31st'!Q82:Q121))+0</f>
         <v/>
       </c>
       <c r="R4" s="2">
-        <f>COUNTA('1ST'!R82:R121)+COUNTA('2nd'!R82:R121)+COUNTA('3rd'!R82:R121)+COUNTA('4th'!R82:R121)+COUNTA('5th'!R82:R121)+COUNTA('6th'!R82:R121)+COUNTA('7th'!R82:R121)+COUNTA('8th'!R82:R121)+COUNTA('9th'!R82:R121)+COUNTA('10th'!R82:R121)+COUNTA('11th'!R82:R121)+COUNTA('12th'!R82:R121)+COUNTA('13th'!R82:R121)+COUNTA('14th'!R82:R121)+COUNTA('15th'!R82:R121)+COUNTA('16th'!R82:R121)+COUNTA('17th'!R82:R121)+COUNTA('18th'!R82:R121)+COUNTA('19th'!R82:R121)+COUNTA('20th'!R82:R121)+COUNTA('21st'!R82:R121)+COUNTA('22nd'!R82:R121)+COUNTA('23rd'!R82:R121)+COUNTA('24th'!R82:R121)+COUNTA('25th'!R82:R121)+COUNTA('26th'!R82:R121)+COUNTA('27th'!R82:R121)+COUNTA('28th'!R82:R121)+COUNTA('29th'!R82:R121)+COUNTA('30th'!R82:R121)+COUNTA('31st'!R82:R121)</f>
+        <f>(COUNTA('1ST'!R82:R121)+COUNTA('2nd'!R82:R121)+COUNTA('3rd'!R82:R121)+COUNTA('4th'!R82:R121)+COUNTA('5th'!R82:R121)+COUNTA('6th'!R82:R121)+COUNTA('7th'!R82:R121)+COUNTA('8th'!R82:R121)+COUNTA('9th'!R82:R121)+COUNTA('10th'!R82:R121)+COUNTA('11th'!R82:R121)+COUNTA('12th'!R82:R121)+COUNTA('13th'!R82:R121)+COUNTA('14th'!R82:R121)+COUNTA('15th'!R82:R121)+COUNTA('16th'!R82:R121)+COUNTA('17th'!R82:R121)+COUNTA('18th'!R82:R121)+COUNTA('19th'!R82:R121)+COUNTA('20th'!R82:R121)+COUNTA('21st'!R82:R121)+COUNTA('22nd'!R82:R121)+COUNTA('23rd'!R82:R121)+COUNTA('24th'!R82:R121)+COUNTA('25th'!R82:R121)+COUNTA('26th'!R82:R121)+COUNTA('27th'!R82:R121)+COUNTA('28th'!R82:R121)+COUNTA('29th'!R82:R121)+COUNTA('30th'!R82:R121)+COUNTA('31st'!R82:R121))+0</f>
         <v/>
       </c>
       <c r="S4" s="2">
-        <f>COUNTA('1ST'!S82:S121)+COUNTA('2nd'!S82:S121)+COUNTA('3rd'!S82:S121)+COUNTA('4th'!S82:S121)+COUNTA('5th'!S82:S121)+COUNTA('6th'!S82:S121)+COUNTA('7th'!S82:S121)+COUNTA('8th'!S82:S121)+COUNTA('9th'!S82:S121)+COUNTA('10th'!S82:S121)+COUNTA('11th'!S82:S121)+COUNTA('12th'!S82:S121)+COUNTA('13th'!S82:S121)+COUNTA('14th'!S82:S121)+COUNTA('15th'!S82:S121)+COUNTA('16th'!S82:S121)+COUNTA('17th'!S82:S121)+COUNTA('18th'!S82:S121)+COUNTA('19th'!S82:S121)+COUNTA('20th'!S82:S121)+COUNTA('21st'!S82:S121)+COUNTA('22nd'!S82:S121)+COUNTA('23rd'!S82:S121)+COUNTA('24th'!S82:S121)+COUNTA('25th'!S82:S121)+COUNTA('26th'!S82:S121)+COUNTA('27th'!S82:S121)+COUNTA('28th'!S82:S121)+COUNTA('29th'!S82:S121)+COUNTA('30th'!S82:S121)+COUNTA('31st'!S82:S121)</f>
+        <f>(COUNTA('1ST'!S82:S121)+COUNTA('2nd'!S82:S121)+COUNTA('3rd'!S82:S121)+COUNTA('4th'!S82:S121)+COUNTA('5th'!S82:S121)+COUNTA('6th'!S82:S121)+COUNTA('7th'!S82:S121)+COUNTA('8th'!S82:S121)+COUNTA('9th'!S82:S121)+COUNTA('10th'!S82:S121)+COUNTA('11th'!S82:S121)+COUNTA('12th'!S82:S121)+COUNTA('13th'!S82:S121)+COUNTA('14th'!S82:S121)+COUNTA('15th'!S82:S121)+COUNTA('16th'!S82:S121)+COUNTA('17th'!S82:S121)+COUNTA('18th'!S82:S121)+COUNTA('19th'!S82:S121)+COUNTA('20th'!S82:S121)+COUNTA('21st'!S82:S121)+COUNTA('22nd'!S82:S121)+COUNTA('23rd'!S82:S121)+COUNTA('24th'!S82:S121)+COUNTA('25th'!S82:S121)+COUNTA('26th'!S82:S121)+COUNTA('27th'!S82:S121)+COUNTA('28th'!S82:S121)+COUNTA('29th'!S82:S121)+COUNTA('30th'!S82:S121)+COUNTA('31st'!S82:S121))+0</f>
         <v/>
       </c>
       <c r="T4" s="2">
-        <f>COUNTA('1ST'!T82:T121)+COUNTA('2nd'!T82:T121)+COUNTA('3rd'!T82:T121)+COUNTA('4th'!T82:T121)+COUNTA('5th'!T82:T121)+COUNTA('6th'!T82:T121)+COUNTA('7th'!T82:T121)+COUNTA('8th'!T82:T121)+COUNTA('9th'!T82:T121)+COUNTA('10th'!T82:T121)+COUNTA('11th'!T82:T121)+COUNTA('12th'!T82:T121)+COUNTA('13th'!T82:T121)+COUNTA('14th'!T82:T121)+COUNTA('15th'!T82:T121)+COUNTA('16th'!T82:T121)+COUNTA('17th'!T82:T121)+COUNTA('18th'!T82:T121)+COUNTA('19th'!T82:T121)+COUNTA('20th'!T82:T121)+COUNTA('21st'!T82:T121)+COUNTA('22nd'!T82:T121)+COUNTA('23rd'!T82:T121)+COUNTA('24th'!T82:T121)+COUNTA('25th'!T82:T121)+COUNTA('26th'!T82:T121)+COUNTA('27th'!T82:T121)+COUNTA('28th'!T82:T121)+COUNTA('29th'!T82:T121)+COUNTA('30th'!T82:T121)+COUNTA('31st'!T82:T121)</f>
+        <f>(COUNTA('1ST'!T82:T121)+COUNTA('2nd'!T82:T121)+COUNTA('3rd'!T82:T121)+COUNTA('4th'!T82:T121)+COUNTA('5th'!T82:T121)+COUNTA('6th'!T82:T121)+COUNTA('7th'!T82:T121)+COUNTA('8th'!T82:T121)+COUNTA('9th'!T82:T121)+COUNTA('10th'!T82:T121)+COUNTA('11th'!T82:T121)+COUNTA('12th'!T82:T121)+COUNTA('13th'!T82:T121)+COUNTA('14th'!T82:T121)+COUNTA('15th'!T82:T121)+COUNTA('16th'!T82:T121)+COUNTA('17th'!T82:T121)+COUNTA('18th'!T82:T121)+COUNTA('19th'!T82:T121)+COUNTA('20th'!T82:T121)+COUNTA('21st'!T82:T121)+COUNTA('22nd'!T82:T121)+COUNTA('23rd'!T82:T121)+COUNTA('24th'!T82:T121)+COUNTA('25th'!T82:T121)+COUNTA('26th'!T82:T121)+COUNTA('27th'!T82:T121)+COUNTA('28th'!T82:T121)+COUNTA('29th'!T82:T121)+COUNTA('30th'!T82:T121)+COUNTA('31st'!T82:T121))+0</f>
         <v/>
       </c>
       <c r="U4" s="2">
-        <f>COUNTA('1ST'!U82:U121)+COUNTA('2nd'!U82:U121)+COUNTA('3rd'!U82:U121)+COUNTA('4th'!U82:U121)+COUNTA('5th'!U82:U121)+COUNTA('6th'!U82:U121)+COUNTA('7th'!U82:U121)+COUNTA('8th'!U82:U121)+COUNTA('9th'!U82:U121)+COUNTA('10th'!U82:U121)+COUNTA('11th'!U82:U121)+COUNTA('12th'!U82:U121)+COUNTA('13th'!U82:U121)+COUNTA('14th'!U82:U121)+COUNTA('15th'!U82:U121)+COUNTA('16th'!U82:U121)+COUNTA('17th'!U82:U121)+COUNTA('18th'!U82:U121)+COUNTA('19th'!U82:U121)+COUNTA('20th'!U82:U121)+COUNTA('21st'!U82:U121)+COUNTA('22nd'!U82:U121)+COUNTA('23rd'!U82:U121)+COUNTA('24th'!U82:U121)+COUNTA('25th'!U82:U121)+COUNTA('26th'!U82:U121)+COUNTA('27th'!U82:U121)+COUNTA('28th'!U82:U121)+COUNTA('29th'!U82:U121)+COUNTA('30th'!U82:U121)+COUNTA('31st'!U82:U121)</f>
-        <v/>
-      </c>
-      <c r="W4" s="4" t="n">
+        <f>(COUNTA('1ST'!U82:U121)+COUNTA('2nd'!U82:U121)+COUNTA('3rd'!U82:U121)+COUNTA('4th'!U82:U121)+COUNTA('5th'!U82:U121)+COUNTA('6th'!U82:U121)+COUNTA('7th'!U82:U121)+COUNTA('8th'!U82:U121)+COUNTA('9th'!U82:U121)+COUNTA('10th'!U82:U121)+COUNTA('11th'!U82:U121)+COUNTA('12th'!U82:U121)+COUNTA('13th'!U82:U121)+COUNTA('14th'!U82:U121)+COUNTA('15th'!U82:U121)+COUNTA('16th'!U82:U121)+COUNTA('17th'!U82:U121)+COUNTA('18th'!U82:U121)+COUNTA('19th'!U82:U121)+COUNTA('20th'!U82:U121)+COUNTA('21st'!U82:U121)+COUNTA('22nd'!U82:U121)+COUNTA('23rd'!U82:U121)+COUNTA('24th'!U82:U121)+COUNTA('25th'!U82:U121)+COUNTA('26th'!U82:U121)+COUNTA('27th'!U82:U121)+COUNTA('28th'!U82:U121)+COUNTA('29th'!U82:U121)+COUNTA('30th'!U82:U121)+COUNTA('31st'!U82:U121))+0</f>
+        <v/>
+      </c>
+      <c r="W4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="AB4" s="4" t="n">
+      <c r="AB4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="AG4" s="4" t="n">
+      <c r="AG4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="AL4" s="4" t="n">
+      <c r="AL4" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3660,483 +3692,564 @@
         </is>
       </c>
       <c r="C5" s="2">
-        <f>COUNTA('1ST'!C122:C161)+COUNTA('2nd'!C122:C161)+COUNTA('3rd'!C122:C161)+COUNTA('4th'!C122:C161)+COUNTA('5th'!C122:C161)+COUNTA('6th'!C122:C161)+COUNTA('7th'!C122:C161)+COUNTA('8th'!C122:C161)+COUNTA('9th'!C122:C161)+COUNTA('10th'!C122:C161)+COUNTA('11th'!C122:C161)+COUNTA('12th'!C122:C161)+COUNTA('13th'!C122:C161)+COUNTA('14th'!C122:C161)+COUNTA('15th'!C122:C161)+COUNTA('16th'!C122:C161)+COUNTA('17th'!C122:C161)+COUNTA('18th'!C122:C161)+COUNTA('19th'!C122:C161)+COUNTA('20th'!C122:C161)+COUNTA('21st'!C122:C161)+COUNTA('22nd'!C122:C161)+COUNTA('23rd'!C122:C161)+COUNTA('24th'!C122:C161)+COUNTA('25th'!C122:C161)+COUNTA('26th'!C122:C161)+COUNTA('27th'!C122:C161)+COUNTA('28th'!C122:C161)+COUNTA('29th'!C122:C161)+COUNTA('30th'!C122:C161)+COUNTA('31st'!C122:C161)</f>
+        <f>(COUNTA('1ST'!C122:C161)+COUNTA('2nd'!C122:C161)+COUNTA('3rd'!C122:C161)+COUNTA('4th'!C122:C161)+COUNTA('5th'!C122:C161)+COUNTA('6th'!C122:C161)+COUNTA('7th'!C122:C161)+COUNTA('8th'!C122:C161)+COUNTA('9th'!C122:C161)+COUNTA('10th'!C122:C161)+COUNTA('11th'!C122:C161)+COUNTA('12th'!C122:C161)+COUNTA('13th'!C122:C161)+COUNTA('14th'!C122:C161)+COUNTA('15th'!C122:C161)+COUNTA('16th'!C122:C161)+COUNTA('17th'!C122:C161)+COUNTA('18th'!C122:C161)+COUNTA('19th'!C122:C161)+COUNTA('20th'!C122:C161)+COUNTA('21st'!C122:C161)+COUNTA('22nd'!C122:C161)+COUNTA('23rd'!C122:C161)+COUNTA('24th'!C122:C161)+COUNTA('25th'!C122:C161)+COUNTA('26th'!C122:C161)+COUNTA('27th'!C122:C161)+COUNTA('28th'!C122:C161)+COUNTA('29th'!C122:C161)+COUNTA('30th'!C122:C161)+COUNTA('31st'!C122:C161))+0</f>
         <v/>
       </c>
       <c r="D5" s="2">
-        <f>COUNTA('1ST'!D122:D161)+COUNTA('2nd'!D122:D161)+COUNTA('3rd'!D122:D161)+COUNTA('4th'!D122:D161)+COUNTA('5th'!D122:D161)+COUNTA('6th'!D122:D161)+COUNTA('7th'!D122:D161)+COUNTA('8th'!D122:D161)+COUNTA('9th'!D122:D161)+COUNTA('10th'!D122:D161)+COUNTA('11th'!D122:D161)+COUNTA('12th'!D122:D161)+COUNTA('13th'!D122:D161)+COUNTA('14th'!D122:D161)+COUNTA('15th'!D122:D161)+COUNTA('16th'!D122:D161)+COUNTA('17th'!D122:D161)+COUNTA('18th'!D122:D161)+COUNTA('19th'!D122:D161)+COUNTA('20th'!D122:D161)+COUNTA('21st'!D122:D161)+COUNTA('22nd'!D122:D161)+COUNTA('23rd'!D122:D161)+COUNTA('24th'!D122:D161)+COUNTA('25th'!D122:D161)+COUNTA('26th'!D122:D161)+COUNTA('27th'!D122:D161)+COUNTA('28th'!D122:D161)+COUNTA('29th'!D122:D161)+COUNTA('30th'!D122:D161)+COUNTA('31st'!D122:D161)</f>
+        <f>(COUNTA('1ST'!D122:D161)+COUNTA('2nd'!D122:D161)+COUNTA('3rd'!D122:D161)+COUNTA('4th'!D122:D161)+COUNTA('5th'!D122:D161)+COUNTA('6th'!D122:D161)+COUNTA('7th'!D122:D161)+COUNTA('8th'!D122:D161)+COUNTA('9th'!D122:D161)+COUNTA('10th'!D122:D161)+COUNTA('11th'!D122:D161)+COUNTA('12th'!D122:D161)+COUNTA('13th'!D122:D161)+COUNTA('14th'!D122:D161)+COUNTA('15th'!D122:D161)+COUNTA('16th'!D122:D161)+COUNTA('17th'!D122:D161)+COUNTA('18th'!D122:D161)+COUNTA('19th'!D122:D161)+COUNTA('20th'!D122:D161)+COUNTA('21st'!D122:D161)+COUNTA('22nd'!D122:D161)+COUNTA('23rd'!D122:D161)+COUNTA('24th'!D122:D161)+COUNTA('25th'!D122:D161)+COUNTA('26th'!D122:D161)+COUNTA('27th'!D122:D161)+COUNTA('28th'!D122:D161)+COUNTA('29th'!D122:D161)+COUNTA('30th'!D122:D161)+COUNTA('31st'!D122:D161))+0</f>
         <v/>
       </c>
       <c r="E5" s="2">
-        <f>COUNTA('1ST'!E122:E161)+COUNTA('2nd'!E122:E161)+COUNTA('3rd'!E122:E161)+COUNTA('4th'!E122:E161)+COUNTA('5th'!E122:E161)+COUNTA('6th'!E122:E161)+COUNTA('7th'!E122:E161)+COUNTA('8th'!E122:E161)+COUNTA('9th'!E122:E161)+COUNTA('10th'!E122:E161)+COUNTA('11th'!E122:E161)+COUNTA('12th'!E122:E161)+COUNTA('13th'!E122:E161)+COUNTA('14th'!E122:E161)+COUNTA('15th'!E122:E161)+COUNTA('16th'!E122:E161)+COUNTA('17th'!E122:E161)+COUNTA('18th'!E122:E161)+COUNTA('19th'!E122:E161)+COUNTA('20th'!E122:E161)+COUNTA('21st'!E122:E161)+COUNTA('22nd'!E122:E161)+COUNTA('23rd'!E122:E161)+COUNTA('24th'!E122:E161)+COUNTA('25th'!E122:E161)+COUNTA('26th'!E122:E161)+COUNTA('27th'!E122:E161)+COUNTA('28th'!E122:E161)+COUNTA('29th'!E122:E161)+COUNTA('30th'!E122:E161)+COUNTA('31st'!E122:E161)</f>
+        <f>(COUNTA('1ST'!E122:E161)+COUNTA('2nd'!E122:E161)+COUNTA('3rd'!E122:E161)+COUNTA('4th'!E122:E161)+COUNTA('5th'!E122:E161)+COUNTA('6th'!E122:E161)+COUNTA('7th'!E122:E161)+COUNTA('8th'!E122:E161)+COUNTA('9th'!E122:E161)+COUNTA('10th'!E122:E161)+COUNTA('11th'!E122:E161)+COUNTA('12th'!E122:E161)+COUNTA('13th'!E122:E161)+COUNTA('14th'!E122:E161)+COUNTA('15th'!E122:E161)+COUNTA('16th'!E122:E161)+COUNTA('17th'!E122:E161)+COUNTA('18th'!E122:E161)+COUNTA('19th'!E122:E161)+COUNTA('20th'!E122:E161)+COUNTA('21st'!E122:E161)+COUNTA('22nd'!E122:E161)+COUNTA('23rd'!E122:E161)+COUNTA('24th'!E122:E161)+COUNTA('25th'!E122:E161)+COUNTA('26th'!E122:E161)+COUNTA('27th'!E122:E161)+COUNTA('28th'!E122:E161)+COUNTA('29th'!E122:E161)+COUNTA('30th'!E122:E161)+COUNTA('31st'!E122:E161))+0</f>
         <v/>
       </c>
       <c r="F5" s="2">
-        <f>COUNTA('1ST'!F122:F161)+COUNTA('2nd'!F122:F161)+COUNTA('3rd'!F122:F161)+COUNTA('4th'!F122:F161)+COUNTA('5th'!F122:F161)+COUNTA('6th'!F122:F161)+COUNTA('7th'!F122:F161)+COUNTA('8th'!F122:F161)+COUNTA('9th'!F122:F161)+COUNTA('10th'!F122:F161)+COUNTA('11th'!F122:F161)+COUNTA('12th'!F122:F161)+COUNTA('13th'!F122:F161)+COUNTA('14th'!F122:F161)+COUNTA('15th'!F122:F161)+COUNTA('16th'!F122:F161)+COUNTA('17th'!F122:F161)+COUNTA('18th'!F122:F161)+COUNTA('19th'!F122:F161)+COUNTA('20th'!F122:F161)+COUNTA('21st'!F122:F161)+COUNTA('22nd'!F122:F161)+COUNTA('23rd'!F122:F161)+COUNTA('24th'!F122:F161)+COUNTA('25th'!F122:F161)+COUNTA('26th'!F122:F161)+COUNTA('27th'!F122:F161)+COUNTA('28th'!F122:F161)+COUNTA('29th'!F122:F161)+COUNTA('30th'!F122:F161)+COUNTA('31st'!F122:F161)</f>
+        <f>(COUNTA('1ST'!F122:F161)+COUNTA('2nd'!F122:F161)+COUNTA('3rd'!F122:F161)+COUNTA('4th'!F122:F161)+COUNTA('5th'!F122:F161)+COUNTA('6th'!F122:F161)+COUNTA('7th'!F122:F161)+COUNTA('8th'!F122:F161)+COUNTA('9th'!F122:F161)+COUNTA('10th'!F122:F161)+COUNTA('11th'!F122:F161)+COUNTA('12th'!F122:F161)+COUNTA('13th'!F122:F161)+COUNTA('14th'!F122:F161)+COUNTA('15th'!F122:F161)+COUNTA('16th'!F122:F161)+COUNTA('17th'!F122:F161)+COUNTA('18th'!F122:F161)+COUNTA('19th'!F122:F161)+COUNTA('20th'!F122:F161)+COUNTA('21st'!F122:F161)+COUNTA('22nd'!F122:F161)+COUNTA('23rd'!F122:F161)+COUNTA('24th'!F122:F161)+COUNTA('25th'!F122:F161)+COUNTA('26th'!F122:F161)+COUNTA('27th'!F122:F161)+COUNTA('28th'!F122:F161)+COUNTA('29th'!F122:F161)+COUNTA('30th'!F122:F161)+COUNTA('31st'!F122:F161))+0</f>
         <v/>
       </c>
       <c r="G5" s="2">
-        <f>COUNTA('1ST'!G122:G161)+COUNTA('2nd'!G122:G161)+COUNTA('3rd'!G122:G161)+COUNTA('4th'!G122:G161)+COUNTA('5th'!G122:G161)+COUNTA('6th'!G122:G161)+COUNTA('7th'!G122:G161)+COUNTA('8th'!G122:G161)+COUNTA('9th'!G122:G161)+COUNTA('10th'!G122:G161)+COUNTA('11th'!G122:G161)+COUNTA('12th'!G122:G161)+COUNTA('13th'!G122:G161)+COUNTA('14th'!G122:G161)+COUNTA('15th'!G122:G161)+COUNTA('16th'!G122:G161)+COUNTA('17th'!G122:G161)+COUNTA('18th'!G122:G161)+COUNTA('19th'!G122:G161)+COUNTA('20th'!G122:G161)+COUNTA('21st'!G122:G161)+COUNTA('22nd'!G122:G161)+COUNTA('23rd'!G122:G161)+COUNTA('24th'!G122:G161)+COUNTA('25th'!G122:G161)+COUNTA('26th'!G122:G161)+COUNTA('27th'!G122:G161)+COUNTA('28th'!G122:G161)+COUNTA('29th'!G122:G161)+COUNTA('30th'!G122:G161)+COUNTA('31st'!G122:G161)</f>
+        <f>(COUNTA('1ST'!G122:G161)+COUNTA('2nd'!G122:G161)+COUNTA('3rd'!G122:G161)+COUNTA('4th'!G122:G161)+COUNTA('5th'!G122:G161)+COUNTA('6th'!G122:G161)+COUNTA('7th'!G122:G161)+COUNTA('8th'!G122:G161)+COUNTA('9th'!G122:G161)+COUNTA('10th'!G122:G161)+COUNTA('11th'!G122:G161)+COUNTA('12th'!G122:G161)+COUNTA('13th'!G122:G161)+COUNTA('14th'!G122:G161)+COUNTA('15th'!G122:G161)+COUNTA('16th'!G122:G161)+COUNTA('17th'!G122:G161)+COUNTA('18th'!G122:G161)+COUNTA('19th'!G122:G161)+COUNTA('20th'!G122:G161)+COUNTA('21st'!G122:G161)+COUNTA('22nd'!G122:G161)+COUNTA('23rd'!G122:G161)+COUNTA('24th'!G122:G161)+COUNTA('25th'!G122:G161)+COUNTA('26th'!G122:G161)+COUNTA('27th'!G122:G161)+COUNTA('28th'!G122:G161)+COUNTA('29th'!G122:G161)+COUNTA('30th'!G122:G161)+COUNTA('31st'!G122:G161))+0</f>
         <v/>
       </c>
       <c r="H5" s="2">
-        <f>COUNTA('1ST'!H122:H161)+COUNTA('2nd'!H122:H161)+COUNTA('3rd'!H122:H161)+COUNTA('4th'!H122:H161)+COUNTA('5th'!H122:H161)+COUNTA('6th'!H122:H161)+COUNTA('7th'!H122:H161)+COUNTA('8th'!H122:H161)+COUNTA('9th'!H122:H161)+COUNTA('10th'!H122:H161)+COUNTA('11th'!H122:H161)+COUNTA('12th'!H122:H161)+COUNTA('13th'!H122:H161)+COUNTA('14th'!H122:H161)+COUNTA('15th'!H122:H161)+COUNTA('16th'!H122:H161)+COUNTA('17th'!H122:H161)+COUNTA('18th'!H122:H161)+COUNTA('19th'!H122:H161)+COUNTA('20th'!H122:H161)+COUNTA('21st'!H122:H161)+COUNTA('22nd'!H122:H161)+COUNTA('23rd'!H122:H161)+COUNTA('24th'!H122:H161)+COUNTA('25th'!H122:H161)+COUNTA('26th'!H122:H161)+COUNTA('27th'!H122:H161)+COUNTA('28th'!H122:H161)+COUNTA('29th'!H122:H161)+COUNTA('30th'!H122:H161)+COUNTA('31st'!H122:H161)</f>
+        <f>(COUNTA('1ST'!H122:H161)+COUNTA('2nd'!H122:H161)+COUNTA('3rd'!H122:H161)+COUNTA('4th'!H122:H161)+COUNTA('5th'!H122:H161)+COUNTA('6th'!H122:H161)+COUNTA('7th'!H122:H161)+COUNTA('8th'!H122:H161)+COUNTA('9th'!H122:H161)+COUNTA('10th'!H122:H161)+COUNTA('11th'!H122:H161)+COUNTA('12th'!H122:H161)+COUNTA('13th'!H122:H161)+COUNTA('14th'!H122:H161)+COUNTA('15th'!H122:H161)+COUNTA('16th'!H122:H161)+COUNTA('17th'!H122:H161)+COUNTA('18th'!H122:H161)+COUNTA('19th'!H122:H161)+COUNTA('20th'!H122:H161)+COUNTA('21st'!H122:H161)+COUNTA('22nd'!H122:H161)+COUNTA('23rd'!H122:H161)+COUNTA('24th'!H122:H161)+COUNTA('25th'!H122:H161)+COUNTA('26th'!H122:H161)+COUNTA('27th'!H122:H161)+COUNTA('28th'!H122:H161)+COUNTA('29th'!H122:H161)+COUNTA('30th'!H122:H161)+COUNTA('31st'!H122:H161))+0</f>
         <v/>
       </c>
       <c r="I5" s="2">
-        <f>COUNTA('1ST'!I122:I161)+COUNTA('2nd'!I122:I161)+COUNTA('3rd'!I122:I161)+COUNTA('4th'!I122:I161)+COUNTA('5th'!I122:I161)+COUNTA('6th'!I122:I161)+COUNTA('7th'!I122:I161)+COUNTA('8th'!I122:I161)+COUNTA('9th'!I122:I161)+COUNTA('10th'!I122:I161)+COUNTA('11th'!I122:I161)+COUNTA('12th'!I122:I161)+COUNTA('13th'!I122:I161)+COUNTA('14th'!I122:I161)+COUNTA('15th'!I122:I161)+COUNTA('16th'!I122:I161)+COUNTA('17th'!I122:I161)+COUNTA('18th'!I122:I161)+COUNTA('19th'!I122:I161)+COUNTA('20th'!I122:I161)+COUNTA('21st'!I122:I161)+COUNTA('22nd'!I122:I161)+COUNTA('23rd'!I122:I161)+COUNTA('24th'!I122:I161)+COUNTA('25th'!I122:I161)+COUNTA('26th'!I122:I161)+COUNTA('27th'!I122:I161)+COUNTA('28th'!I122:I161)+COUNTA('29th'!I122:I161)+COUNTA('30th'!I122:I161)+COUNTA('31st'!I122:I161)</f>
+        <f>(COUNTA('1ST'!I122:I161)+COUNTA('2nd'!I122:I161)+COUNTA('3rd'!I122:I161)+COUNTA('4th'!I122:I161)+COUNTA('5th'!I122:I161)+COUNTA('6th'!I122:I161)+COUNTA('7th'!I122:I161)+COUNTA('8th'!I122:I161)+COUNTA('9th'!I122:I161)+COUNTA('10th'!I122:I161)+COUNTA('11th'!I122:I161)+COUNTA('12th'!I122:I161)+COUNTA('13th'!I122:I161)+COUNTA('14th'!I122:I161)+COUNTA('15th'!I122:I161)+COUNTA('16th'!I122:I161)+COUNTA('17th'!I122:I161)+COUNTA('18th'!I122:I161)+COUNTA('19th'!I122:I161)+COUNTA('20th'!I122:I161)+COUNTA('21st'!I122:I161)+COUNTA('22nd'!I122:I161)+COUNTA('23rd'!I122:I161)+COUNTA('24th'!I122:I161)+COUNTA('25th'!I122:I161)+COUNTA('26th'!I122:I161)+COUNTA('27th'!I122:I161)+COUNTA('28th'!I122:I161)+COUNTA('29th'!I122:I161)+COUNTA('30th'!I122:I161)+COUNTA('31st'!I122:I161))+0</f>
         <v/>
       </c>
       <c r="J5" s="2">
-        <f>COUNTA('1ST'!J122:J161)+COUNTA('2nd'!J122:J161)+COUNTA('3rd'!J122:J161)+COUNTA('4th'!J122:J161)+COUNTA('5th'!J122:J161)+COUNTA('6th'!J122:J161)+COUNTA('7th'!J122:J161)+COUNTA('8th'!J122:J161)+COUNTA('9th'!J122:J161)+COUNTA('10th'!J122:J161)+COUNTA('11th'!J122:J161)+COUNTA('12th'!J122:J161)+COUNTA('13th'!J122:J161)+COUNTA('14th'!J122:J161)+COUNTA('15th'!J122:J161)+COUNTA('16th'!J122:J161)+COUNTA('17th'!J122:J161)+COUNTA('18th'!J122:J161)+COUNTA('19th'!J122:J161)+COUNTA('20th'!J122:J161)+COUNTA('21st'!J122:J161)+COUNTA('22nd'!J122:J161)+COUNTA('23rd'!J122:J161)+COUNTA('24th'!J122:J161)+COUNTA('25th'!J122:J161)+COUNTA('26th'!J122:J161)+COUNTA('27th'!J122:J161)+COUNTA('28th'!J122:J161)+COUNTA('29th'!J122:J161)+COUNTA('30th'!J122:J161)+COUNTA('31st'!J122:J161)</f>
+        <f>(COUNTA('1ST'!J122:J161)+COUNTA('2nd'!J122:J161)+COUNTA('3rd'!J122:J161)+COUNTA('4th'!J122:J161)+COUNTA('5th'!J122:J161)+COUNTA('6th'!J122:J161)+COUNTA('7th'!J122:J161)+COUNTA('8th'!J122:J161)+COUNTA('9th'!J122:J161)+COUNTA('10th'!J122:J161)+COUNTA('11th'!J122:J161)+COUNTA('12th'!J122:J161)+COUNTA('13th'!J122:J161)+COUNTA('14th'!J122:J161)+COUNTA('15th'!J122:J161)+COUNTA('16th'!J122:J161)+COUNTA('17th'!J122:J161)+COUNTA('18th'!J122:J161)+COUNTA('19th'!J122:J161)+COUNTA('20th'!J122:J161)+COUNTA('21st'!J122:J161)+COUNTA('22nd'!J122:J161)+COUNTA('23rd'!J122:J161)+COUNTA('24th'!J122:J161)+COUNTA('25th'!J122:J161)+COUNTA('26th'!J122:J161)+COUNTA('27th'!J122:J161)+COUNTA('28th'!J122:J161)+COUNTA('29th'!J122:J161)+COUNTA('30th'!J122:J161)+COUNTA('31st'!J122:J161))+0</f>
         <v/>
       </c>
       <c r="K5" s="2">
-        <f>COUNTA('1ST'!K122:K161)+COUNTA('2nd'!K122:K161)+COUNTA('3rd'!K122:K161)+COUNTA('4th'!K122:K161)+COUNTA('5th'!K122:K161)+COUNTA('6th'!K122:K161)+COUNTA('7th'!K122:K161)+COUNTA('8th'!K122:K161)+COUNTA('9th'!K122:K161)+COUNTA('10th'!K122:K161)+COUNTA('11th'!K122:K161)+COUNTA('12th'!K122:K161)+COUNTA('13th'!K122:K161)+COUNTA('14th'!K122:K161)+COUNTA('15th'!K122:K161)+COUNTA('16th'!K122:K161)+COUNTA('17th'!K122:K161)+COUNTA('18th'!K122:K161)+COUNTA('19th'!K122:K161)+COUNTA('20th'!K122:K161)+COUNTA('21st'!K122:K161)+COUNTA('22nd'!K122:K161)+COUNTA('23rd'!K122:K161)+COUNTA('24th'!K122:K161)+COUNTA('25th'!K122:K161)+COUNTA('26th'!K122:K161)+COUNTA('27th'!K122:K161)+COUNTA('28th'!K122:K161)+COUNTA('29th'!K122:K161)+COUNTA('30th'!K122:K161)+COUNTA('31st'!K122:K161)</f>
+        <f>(COUNTA('1ST'!K122:K161)+COUNTA('2nd'!K122:K161)+COUNTA('3rd'!K122:K161)+COUNTA('4th'!K122:K161)+COUNTA('5th'!K122:K161)+COUNTA('6th'!K122:K161)+COUNTA('7th'!K122:K161)+COUNTA('8th'!K122:K161)+COUNTA('9th'!K122:K161)+COUNTA('10th'!K122:K161)+COUNTA('11th'!K122:K161)+COUNTA('12th'!K122:K161)+COUNTA('13th'!K122:K161)+COUNTA('14th'!K122:K161)+COUNTA('15th'!K122:K161)+COUNTA('16th'!K122:K161)+COUNTA('17th'!K122:K161)+COUNTA('18th'!K122:K161)+COUNTA('19th'!K122:K161)+COUNTA('20th'!K122:K161)+COUNTA('21st'!K122:K161)+COUNTA('22nd'!K122:K161)+COUNTA('23rd'!K122:K161)+COUNTA('24th'!K122:K161)+COUNTA('25th'!K122:K161)+COUNTA('26th'!K122:K161)+COUNTA('27th'!K122:K161)+COUNTA('28th'!K122:K161)+COUNTA('29th'!K122:K161)+COUNTA('30th'!K122:K161)+COUNTA('31st'!K122:K161))+0</f>
         <v/>
       </c>
       <c r="L5" s="2">
-        <f>COUNTA('1ST'!L122:L161)+COUNTA('2nd'!L122:L161)+COUNTA('3rd'!L122:L161)+COUNTA('4th'!L122:L161)+COUNTA('5th'!L122:L161)+COUNTA('6th'!L122:L161)+COUNTA('7th'!L122:L161)+COUNTA('8th'!L122:L161)+COUNTA('9th'!L122:L161)+COUNTA('10th'!L122:L161)+COUNTA('11th'!L122:L161)+COUNTA('12th'!L122:L161)+COUNTA('13th'!L122:L161)+COUNTA('14th'!L122:L161)+COUNTA('15th'!L122:L161)+COUNTA('16th'!L122:L161)+COUNTA('17th'!L122:L161)+COUNTA('18th'!L122:L161)+COUNTA('19th'!L122:L161)+COUNTA('20th'!L122:L161)+COUNTA('21st'!L122:L161)+COUNTA('22nd'!L122:L161)+COUNTA('23rd'!L122:L161)+COUNTA('24th'!L122:L161)+COUNTA('25th'!L122:L161)+COUNTA('26th'!L122:L161)+COUNTA('27th'!L122:L161)+COUNTA('28th'!L122:L161)+COUNTA('29th'!L122:L161)+COUNTA('30th'!L122:L161)+COUNTA('31st'!L122:L161)</f>
+        <f>(COUNTA('1ST'!L122:L161)+COUNTA('2nd'!L122:L161)+COUNTA('3rd'!L122:L161)+COUNTA('4th'!L122:L161)+COUNTA('5th'!L122:L161)+COUNTA('6th'!L122:L161)+COUNTA('7th'!L122:L161)+COUNTA('8th'!L122:L161)+COUNTA('9th'!L122:L161)+COUNTA('10th'!L122:L161)+COUNTA('11th'!L122:L161)+COUNTA('12th'!L122:L161)+COUNTA('13th'!L122:L161)+COUNTA('14th'!L122:L161)+COUNTA('15th'!L122:L161)+COUNTA('16th'!L122:L161)+COUNTA('17th'!L122:L161)+COUNTA('18th'!L122:L161)+COUNTA('19th'!L122:L161)+COUNTA('20th'!L122:L161)+COUNTA('21st'!L122:L161)+COUNTA('22nd'!L122:L161)+COUNTA('23rd'!L122:L161)+COUNTA('24th'!L122:L161)+COUNTA('25th'!L122:L161)+COUNTA('26th'!L122:L161)+COUNTA('27th'!L122:L161)+COUNTA('28th'!L122:L161)+COUNTA('29th'!L122:L161)+COUNTA('30th'!L122:L161)+COUNTA('31st'!L122:L161))+0</f>
         <v/>
       </c>
       <c r="M5" s="2">
-        <f>COUNTA('1ST'!M122:M161)+COUNTA('2nd'!M122:M161)+COUNTA('3rd'!M122:M161)+COUNTA('4th'!M122:M161)+COUNTA('5th'!M122:M161)+COUNTA('6th'!M122:M161)+COUNTA('7th'!M122:M161)+COUNTA('8th'!M122:M161)+COUNTA('9th'!M122:M161)+COUNTA('10th'!M122:M161)+COUNTA('11th'!M122:M161)+COUNTA('12th'!M122:M161)+COUNTA('13th'!M122:M161)+COUNTA('14th'!M122:M161)+COUNTA('15th'!M122:M161)+COUNTA('16th'!M122:M161)+COUNTA('17th'!M122:M161)+COUNTA('18th'!M122:M161)+COUNTA('19th'!M122:M161)+COUNTA('20th'!M122:M161)+COUNTA('21st'!M122:M161)+COUNTA('22nd'!M122:M161)+COUNTA('23rd'!M122:M161)+COUNTA('24th'!M122:M161)+COUNTA('25th'!M122:M161)+COUNTA('26th'!M122:M161)+COUNTA('27th'!M122:M161)+COUNTA('28th'!M122:M161)+COUNTA('29th'!M122:M161)+COUNTA('30th'!M122:M161)+COUNTA('31st'!M122:M161)</f>
+        <f>(COUNTA('1ST'!M122:M161)+COUNTA('2nd'!M122:M161)+COUNTA('3rd'!M122:M161)+COUNTA('4th'!M122:M161)+COUNTA('5th'!M122:M161)+COUNTA('6th'!M122:M161)+COUNTA('7th'!M122:M161)+COUNTA('8th'!M122:M161)+COUNTA('9th'!M122:M161)+COUNTA('10th'!M122:M161)+COUNTA('11th'!M122:M161)+COUNTA('12th'!M122:M161)+COUNTA('13th'!M122:M161)+COUNTA('14th'!M122:M161)+COUNTA('15th'!M122:M161)+COUNTA('16th'!M122:M161)+COUNTA('17th'!M122:M161)+COUNTA('18th'!M122:M161)+COUNTA('19th'!M122:M161)+COUNTA('20th'!M122:M161)+COUNTA('21st'!M122:M161)+COUNTA('22nd'!M122:M161)+COUNTA('23rd'!M122:M161)+COUNTA('24th'!M122:M161)+COUNTA('25th'!M122:M161)+COUNTA('26th'!M122:M161)+COUNTA('27th'!M122:M161)+COUNTA('28th'!M122:M161)+COUNTA('29th'!M122:M161)+COUNTA('30th'!M122:M161)+COUNTA('31st'!M122:M161))+0</f>
         <v/>
       </c>
       <c r="N5" s="2">
-        <f>COUNTA('1ST'!N122:N161)+COUNTA('2nd'!N122:N161)+COUNTA('3rd'!N122:N161)+COUNTA('4th'!N122:N161)+COUNTA('5th'!N122:N161)+COUNTA('6th'!N122:N161)+COUNTA('7th'!N122:N161)+COUNTA('8th'!N122:N161)+COUNTA('9th'!N122:N161)+COUNTA('10th'!N122:N161)+COUNTA('11th'!N122:N161)+COUNTA('12th'!N122:N161)+COUNTA('13th'!N122:N161)+COUNTA('14th'!N122:N161)+COUNTA('15th'!N122:N161)+COUNTA('16th'!N122:N161)+COUNTA('17th'!N122:N161)+COUNTA('18th'!N122:N161)+COUNTA('19th'!N122:N161)+COUNTA('20th'!N122:N161)+COUNTA('21st'!N122:N161)+COUNTA('22nd'!N122:N161)+COUNTA('23rd'!N122:N161)+COUNTA('24th'!N122:N161)+COUNTA('25th'!N122:N161)+COUNTA('26th'!N122:N161)+COUNTA('27th'!N122:N161)+COUNTA('28th'!N122:N161)+COUNTA('29th'!N122:N161)+COUNTA('30th'!N122:N161)+COUNTA('31st'!N122:N161)</f>
+        <f>(COUNTA('1ST'!N122:N161)+COUNTA('2nd'!N122:N161)+COUNTA('3rd'!N122:N161)+COUNTA('4th'!N122:N161)+COUNTA('5th'!N122:N161)+COUNTA('6th'!N122:N161)+COUNTA('7th'!N122:N161)+COUNTA('8th'!N122:N161)+COUNTA('9th'!N122:N161)+COUNTA('10th'!N122:N161)+COUNTA('11th'!N122:N161)+COUNTA('12th'!N122:N161)+COUNTA('13th'!N122:N161)+COUNTA('14th'!N122:N161)+COUNTA('15th'!N122:N161)+COUNTA('16th'!N122:N161)+COUNTA('17th'!N122:N161)+COUNTA('18th'!N122:N161)+COUNTA('19th'!N122:N161)+COUNTA('20th'!N122:N161)+COUNTA('21st'!N122:N161)+COUNTA('22nd'!N122:N161)+COUNTA('23rd'!N122:N161)+COUNTA('24th'!N122:N161)+COUNTA('25th'!N122:N161)+COUNTA('26th'!N122:N161)+COUNTA('27th'!N122:N161)+COUNTA('28th'!N122:N161)+COUNTA('29th'!N122:N161)+COUNTA('30th'!N122:N161)+COUNTA('31st'!N122:N161))+0</f>
         <v/>
       </c>
       <c r="O5" s="2">
-        <f>COUNTA('1ST'!O122:O161)+COUNTA('2nd'!O122:O161)+COUNTA('3rd'!O122:O161)+COUNTA('4th'!O122:O161)+COUNTA('5th'!O122:O161)+COUNTA('6th'!O122:O161)+COUNTA('7th'!O122:O161)+COUNTA('8th'!O122:O161)+COUNTA('9th'!O122:O161)+COUNTA('10th'!O122:O161)+COUNTA('11th'!O122:O161)+COUNTA('12th'!O122:O161)+COUNTA('13th'!O122:O161)+COUNTA('14th'!O122:O161)+COUNTA('15th'!O122:O161)+COUNTA('16th'!O122:O161)+COUNTA('17th'!O122:O161)+COUNTA('18th'!O122:O161)+COUNTA('19th'!O122:O161)+COUNTA('20th'!O122:O161)+COUNTA('21st'!O122:O161)+COUNTA('22nd'!O122:O161)+COUNTA('23rd'!O122:O161)+COUNTA('24th'!O122:O161)+COUNTA('25th'!O122:O161)+COUNTA('26th'!O122:O161)+COUNTA('27th'!O122:O161)+COUNTA('28th'!O122:O161)+COUNTA('29th'!O122:O161)+COUNTA('30th'!O122:O161)+COUNTA('31st'!O122:O161)</f>
+        <f>(COUNTA('1ST'!O122:O161)+COUNTA('2nd'!O122:O161)+COUNTA('3rd'!O122:O161)+COUNTA('4th'!O122:O161)+COUNTA('5th'!O122:O161)+COUNTA('6th'!O122:O161)+COUNTA('7th'!O122:O161)+COUNTA('8th'!O122:O161)+COUNTA('9th'!O122:O161)+COUNTA('10th'!O122:O161)+COUNTA('11th'!O122:O161)+COUNTA('12th'!O122:O161)+COUNTA('13th'!O122:O161)+COUNTA('14th'!O122:O161)+COUNTA('15th'!O122:O161)+COUNTA('16th'!O122:O161)+COUNTA('17th'!O122:O161)+COUNTA('18th'!O122:O161)+COUNTA('19th'!O122:O161)+COUNTA('20th'!O122:O161)+COUNTA('21st'!O122:O161)+COUNTA('22nd'!O122:O161)+COUNTA('23rd'!O122:O161)+COUNTA('24th'!O122:O161)+COUNTA('25th'!O122:O161)+COUNTA('26th'!O122:O161)+COUNTA('27th'!O122:O161)+COUNTA('28th'!O122:O161)+COUNTA('29th'!O122:O161)+COUNTA('30th'!O122:O161)+COUNTA('31st'!O122:O161))+0</f>
         <v/>
       </c>
       <c r="P5" s="2">
-        <f>COUNTA('1ST'!P122:P161)+COUNTA('2nd'!P122:P161)+COUNTA('3rd'!P122:P161)+COUNTA('4th'!P122:P161)+COUNTA('5th'!P122:P161)+COUNTA('6th'!P122:P161)+COUNTA('7th'!P122:P161)+COUNTA('8th'!P122:P161)+COUNTA('9th'!P122:P161)+COUNTA('10th'!P122:P161)+COUNTA('11th'!P122:P161)+COUNTA('12th'!P122:P161)+COUNTA('13th'!P122:P161)+COUNTA('14th'!P122:P161)+COUNTA('15th'!P122:P161)+COUNTA('16th'!P122:P161)+COUNTA('17th'!P122:P161)+COUNTA('18th'!P122:P161)+COUNTA('19th'!P122:P161)+COUNTA('20th'!P122:P161)+COUNTA('21st'!P122:P161)+COUNTA('22nd'!P122:P161)+COUNTA('23rd'!P122:P161)+COUNTA('24th'!P122:P161)+COUNTA('25th'!P122:P161)+COUNTA('26th'!P122:P161)+COUNTA('27th'!P122:P161)+COUNTA('28th'!P122:P161)+COUNTA('29th'!P122:P161)+COUNTA('30th'!P122:P161)+COUNTA('31st'!P122:P161)</f>
+        <f>(COUNTA('1ST'!P122:P161)+COUNTA('2nd'!P122:P161)+COUNTA('3rd'!P122:P161)+COUNTA('4th'!P122:P161)+COUNTA('5th'!P122:P161)+COUNTA('6th'!P122:P161)+COUNTA('7th'!P122:P161)+COUNTA('8th'!P122:P161)+COUNTA('9th'!P122:P161)+COUNTA('10th'!P122:P161)+COUNTA('11th'!P122:P161)+COUNTA('12th'!P122:P161)+COUNTA('13th'!P122:P161)+COUNTA('14th'!P122:P161)+COUNTA('15th'!P122:P161)+COUNTA('16th'!P122:P161)+COUNTA('17th'!P122:P161)+COUNTA('18th'!P122:P161)+COUNTA('19th'!P122:P161)+COUNTA('20th'!P122:P161)+COUNTA('21st'!P122:P161)+COUNTA('22nd'!P122:P161)+COUNTA('23rd'!P122:P161)+COUNTA('24th'!P122:P161)+COUNTA('25th'!P122:P161)+COUNTA('26th'!P122:P161)+COUNTA('27th'!P122:P161)+COUNTA('28th'!P122:P161)+COUNTA('29th'!P122:P161)+COUNTA('30th'!P122:P161)+COUNTA('31st'!P122:P161))+0</f>
         <v/>
       </c>
       <c r="Q5" s="2">
-        <f>COUNTA('1ST'!Q122:Q161)+COUNTA('2nd'!Q122:Q161)+COUNTA('3rd'!Q122:Q161)+COUNTA('4th'!Q122:Q161)+COUNTA('5th'!Q122:Q161)+COUNTA('6th'!Q122:Q161)+COUNTA('7th'!Q122:Q161)+COUNTA('8th'!Q122:Q161)+COUNTA('9th'!Q122:Q161)+COUNTA('10th'!Q122:Q161)+COUNTA('11th'!Q122:Q161)+COUNTA('12th'!Q122:Q161)+COUNTA('13th'!Q122:Q161)+COUNTA('14th'!Q122:Q161)+COUNTA('15th'!Q122:Q161)+COUNTA('16th'!Q122:Q161)+COUNTA('17th'!Q122:Q161)+COUNTA('18th'!Q122:Q161)+COUNTA('19th'!Q122:Q161)+COUNTA('20th'!Q122:Q161)+COUNTA('21st'!Q122:Q161)+COUNTA('22nd'!Q122:Q161)+COUNTA('23rd'!Q122:Q161)+COUNTA('24th'!Q122:Q161)+COUNTA('25th'!Q122:Q161)+COUNTA('26th'!Q122:Q161)+COUNTA('27th'!Q122:Q161)+COUNTA('28th'!Q122:Q161)+COUNTA('29th'!Q122:Q161)+COUNTA('30th'!Q122:Q161)+COUNTA('31st'!Q122:Q161)</f>
+        <f>(COUNTA('1ST'!Q122:Q161)+COUNTA('2nd'!Q122:Q161)+COUNTA('3rd'!Q122:Q161)+COUNTA('4th'!Q122:Q161)+COUNTA('5th'!Q122:Q161)+COUNTA('6th'!Q122:Q161)+COUNTA('7th'!Q122:Q161)+COUNTA('8th'!Q122:Q161)+COUNTA('9th'!Q122:Q161)+COUNTA('10th'!Q122:Q161)+COUNTA('11th'!Q122:Q161)+COUNTA('12th'!Q122:Q161)+COUNTA('13th'!Q122:Q161)+COUNTA('14th'!Q122:Q161)+COUNTA('15th'!Q122:Q161)+COUNTA('16th'!Q122:Q161)+COUNTA('17th'!Q122:Q161)+COUNTA('18th'!Q122:Q161)+COUNTA('19th'!Q122:Q161)+COUNTA('20th'!Q122:Q161)+COUNTA('21st'!Q122:Q161)+COUNTA('22nd'!Q122:Q161)+COUNTA('23rd'!Q122:Q161)+COUNTA('24th'!Q122:Q161)+COUNTA('25th'!Q122:Q161)+COUNTA('26th'!Q122:Q161)+COUNTA('27th'!Q122:Q161)+COUNTA('28th'!Q122:Q161)+COUNTA('29th'!Q122:Q161)+COUNTA('30th'!Q122:Q161)+COUNTA('31st'!Q122:Q161))+0</f>
         <v/>
       </c>
       <c r="R5" s="2">
-        <f>COUNTA('1ST'!R122:R161)+COUNTA('2nd'!R122:R161)+COUNTA('3rd'!R122:R161)+COUNTA('4th'!R122:R161)+COUNTA('5th'!R122:R161)+COUNTA('6th'!R122:R161)+COUNTA('7th'!R122:R161)+COUNTA('8th'!R122:R161)+COUNTA('9th'!R122:R161)+COUNTA('10th'!R122:R161)+COUNTA('11th'!R122:R161)+COUNTA('12th'!R122:R161)+COUNTA('13th'!R122:R161)+COUNTA('14th'!R122:R161)+COUNTA('15th'!R122:R161)+COUNTA('16th'!R122:R161)+COUNTA('17th'!R122:R161)+COUNTA('18th'!R122:R161)+COUNTA('19th'!R122:R161)+COUNTA('20th'!R122:R161)+COUNTA('21st'!R122:R161)+COUNTA('22nd'!R122:R161)+COUNTA('23rd'!R122:R161)+COUNTA('24th'!R122:R161)+COUNTA('25th'!R122:R161)+COUNTA('26th'!R122:R161)+COUNTA('27th'!R122:R161)+COUNTA('28th'!R122:R161)+COUNTA('29th'!R122:R161)+COUNTA('30th'!R122:R161)+COUNTA('31st'!R122:R161)</f>
+        <f>(COUNTA('1ST'!R122:R161)+COUNTA('2nd'!R122:R161)+COUNTA('3rd'!R122:R161)+COUNTA('4th'!R122:R161)+COUNTA('5th'!R122:R161)+COUNTA('6th'!R122:R161)+COUNTA('7th'!R122:R161)+COUNTA('8th'!R122:R161)+COUNTA('9th'!R122:R161)+COUNTA('10th'!R122:R161)+COUNTA('11th'!R122:R161)+COUNTA('12th'!R122:R161)+COUNTA('13th'!R122:R161)+COUNTA('14th'!R122:R161)+COUNTA('15th'!R122:R161)+COUNTA('16th'!R122:R161)+COUNTA('17th'!R122:R161)+COUNTA('18th'!R122:R161)+COUNTA('19th'!R122:R161)+COUNTA('20th'!R122:R161)+COUNTA('21st'!R122:R161)+COUNTA('22nd'!R122:R161)+COUNTA('23rd'!R122:R161)+COUNTA('24th'!R122:R161)+COUNTA('25th'!R122:R161)+COUNTA('26th'!R122:R161)+COUNTA('27th'!R122:R161)+COUNTA('28th'!R122:R161)+COUNTA('29th'!R122:R161)+COUNTA('30th'!R122:R161)+COUNTA('31st'!R122:R161))+0</f>
         <v/>
       </c>
       <c r="S5" s="2">
-        <f>COUNTA('1ST'!S122:S161)+COUNTA('2nd'!S122:S161)+COUNTA('3rd'!S122:S161)+COUNTA('4th'!S122:S161)+COUNTA('5th'!S122:S161)+COUNTA('6th'!S122:S161)+COUNTA('7th'!S122:S161)+COUNTA('8th'!S122:S161)+COUNTA('9th'!S122:S161)+COUNTA('10th'!S122:S161)+COUNTA('11th'!S122:S161)+COUNTA('12th'!S122:S161)+COUNTA('13th'!S122:S161)+COUNTA('14th'!S122:S161)+COUNTA('15th'!S122:S161)+COUNTA('16th'!S122:S161)+COUNTA('17th'!S122:S161)+COUNTA('18th'!S122:S161)+COUNTA('19th'!S122:S161)+COUNTA('20th'!S122:S161)+COUNTA('21st'!S122:S161)+COUNTA('22nd'!S122:S161)+COUNTA('23rd'!S122:S161)+COUNTA('24th'!S122:S161)+COUNTA('25th'!S122:S161)+COUNTA('26th'!S122:S161)+COUNTA('27th'!S122:S161)+COUNTA('28th'!S122:S161)+COUNTA('29th'!S122:S161)+COUNTA('30th'!S122:S161)+COUNTA('31st'!S122:S161)</f>
+        <f>(COUNTA('1ST'!S122:S161)+COUNTA('2nd'!S122:S161)+COUNTA('3rd'!S122:S161)+COUNTA('4th'!S122:S161)+COUNTA('5th'!S122:S161)+COUNTA('6th'!S122:S161)+COUNTA('7th'!S122:S161)+COUNTA('8th'!S122:S161)+COUNTA('9th'!S122:S161)+COUNTA('10th'!S122:S161)+COUNTA('11th'!S122:S161)+COUNTA('12th'!S122:S161)+COUNTA('13th'!S122:S161)+COUNTA('14th'!S122:S161)+COUNTA('15th'!S122:S161)+COUNTA('16th'!S122:S161)+COUNTA('17th'!S122:S161)+COUNTA('18th'!S122:S161)+COUNTA('19th'!S122:S161)+COUNTA('20th'!S122:S161)+COUNTA('21st'!S122:S161)+COUNTA('22nd'!S122:S161)+COUNTA('23rd'!S122:S161)+COUNTA('24th'!S122:S161)+COUNTA('25th'!S122:S161)+COUNTA('26th'!S122:S161)+COUNTA('27th'!S122:S161)+COUNTA('28th'!S122:S161)+COUNTA('29th'!S122:S161)+COUNTA('30th'!S122:S161)+COUNTA('31st'!S122:S161))+0</f>
         <v/>
       </c>
       <c r="T5" s="2">
-        <f>COUNTA('1ST'!T122:T161)+COUNTA('2nd'!T122:T161)+COUNTA('3rd'!T122:T161)+COUNTA('4th'!T122:T161)+COUNTA('5th'!T122:T161)+COUNTA('6th'!T122:T161)+COUNTA('7th'!T122:T161)+COUNTA('8th'!T122:T161)+COUNTA('9th'!T122:T161)+COUNTA('10th'!T122:T161)+COUNTA('11th'!T122:T161)+COUNTA('12th'!T122:T161)+COUNTA('13th'!T122:T161)+COUNTA('14th'!T122:T161)+COUNTA('15th'!T122:T161)+COUNTA('16th'!T122:T161)+COUNTA('17th'!T122:T161)+COUNTA('18th'!T122:T161)+COUNTA('19th'!T122:T161)+COUNTA('20th'!T122:T161)+COUNTA('21st'!T122:T161)+COUNTA('22nd'!T122:T161)+COUNTA('23rd'!T122:T161)+COUNTA('24th'!T122:T161)+COUNTA('25th'!T122:T161)+COUNTA('26th'!T122:T161)+COUNTA('27th'!T122:T161)+COUNTA('28th'!T122:T161)+COUNTA('29th'!T122:T161)+COUNTA('30th'!T122:T161)+COUNTA('31st'!T122:T161)</f>
+        <f>(COUNTA('1ST'!T122:T161)+COUNTA('2nd'!T122:T161)+COUNTA('3rd'!T122:T161)+COUNTA('4th'!T122:T161)+COUNTA('5th'!T122:T161)+COUNTA('6th'!T122:T161)+COUNTA('7th'!T122:T161)+COUNTA('8th'!T122:T161)+COUNTA('9th'!T122:T161)+COUNTA('10th'!T122:T161)+COUNTA('11th'!T122:T161)+COUNTA('12th'!T122:T161)+COUNTA('13th'!T122:T161)+COUNTA('14th'!T122:T161)+COUNTA('15th'!T122:T161)+COUNTA('16th'!T122:T161)+COUNTA('17th'!T122:T161)+COUNTA('18th'!T122:T161)+COUNTA('19th'!T122:T161)+COUNTA('20th'!T122:T161)+COUNTA('21st'!T122:T161)+COUNTA('22nd'!T122:T161)+COUNTA('23rd'!T122:T161)+COUNTA('24th'!T122:T161)+COUNTA('25th'!T122:T161)+COUNTA('26th'!T122:T161)+COUNTA('27th'!T122:T161)+COUNTA('28th'!T122:T161)+COUNTA('29th'!T122:T161)+COUNTA('30th'!T122:T161)+COUNTA('31st'!T122:T161))+0</f>
         <v/>
       </c>
       <c r="U5" s="2">
-        <f>COUNTA('1ST'!U122:U161)+COUNTA('2nd'!U122:U161)+COUNTA('3rd'!U122:U161)+COUNTA('4th'!U122:U161)+COUNTA('5th'!U122:U161)+COUNTA('6th'!U122:U161)+COUNTA('7th'!U122:U161)+COUNTA('8th'!U122:U161)+COUNTA('9th'!U122:U161)+COUNTA('10th'!U122:U161)+COUNTA('11th'!U122:U161)+COUNTA('12th'!U122:U161)+COUNTA('13th'!U122:U161)+COUNTA('14th'!U122:U161)+COUNTA('15th'!U122:U161)+COUNTA('16th'!U122:U161)+COUNTA('17th'!U122:U161)+COUNTA('18th'!U122:U161)+COUNTA('19th'!U122:U161)+COUNTA('20th'!U122:U161)+COUNTA('21st'!U122:U161)+COUNTA('22nd'!U122:U161)+COUNTA('23rd'!U122:U161)+COUNTA('24th'!U122:U161)+COUNTA('25th'!U122:U161)+COUNTA('26th'!U122:U161)+COUNTA('27th'!U122:U161)+COUNTA('28th'!U122:U161)+COUNTA('29th'!U122:U161)+COUNTA('30th'!U122:U161)+COUNTA('31st'!U122:U161)</f>
-        <v/>
-      </c>
-      <c r="W5" s="4" t="n">
+        <f>(COUNTA('1ST'!U122:U161)+COUNTA('2nd'!U122:U161)+COUNTA('3rd'!U122:U161)+COUNTA('4th'!U122:U161)+COUNTA('5th'!U122:U161)+COUNTA('6th'!U122:U161)+COUNTA('7th'!U122:U161)+COUNTA('8th'!U122:U161)+COUNTA('9th'!U122:U161)+COUNTA('10th'!U122:U161)+COUNTA('11th'!U122:U161)+COUNTA('12th'!U122:U161)+COUNTA('13th'!U122:U161)+COUNTA('14th'!U122:U161)+COUNTA('15th'!U122:U161)+COUNTA('16th'!U122:U161)+COUNTA('17th'!U122:U161)+COUNTA('18th'!U122:U161)+COUNTA('19th'!U122:U161)+COUNTA('20th'!U122:U161)+COUNTA('21st'!U122:U161)+COUNTA('22nd'!U122:U161)+COUNTA('23rd'!U122:U161)+COUNTA('24th'!U122:U161)+COUNTA('25th'!U122:U161)+COUNTA('26th'!U122:U161)+COUNTA('27th'!U122:U161)+COUNTA('28th'!U122:U161)+COUNTA('29th'!U122:U161)+COUNTA('30th'!U122:U161)+COUNTA('31st'!U122:U161))+0</f>
+        <v/>
+      </c>
+      <c r="W5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="AB5" s="4" t="n">
+      <c r="AB5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="AG5" s="4" t="n">
+      <c r="AG5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="AL5" s="4" t="n">
+      <c r="AL5" s="5" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="6">
-      <c r="W6" s="4" t="n">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <f>SUM(C2:C5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="3">
+        <f>SUM(D2:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="3">
+        <f>SUM(E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="3">
+        <f>SUM(F2:F5)</f>
+        <v/>
+      </c>
+      <c r="G6" s="3">
+        <f>SUM(G2:G5)</f>
+        <v/>
+      </c>
+      <c r="H6" s="3">
+        <f>SUM(H2:H5)</f>
+        <v/>
+      </c>
+      <c r="I6" s="3">
+        <f>SUM(I2:I5)</f>
+        <v/>
+      </c>
+      <c r="J6" s="3">
+        <f>SUM(J2:J5)</f>
+        <v/>
+      </c>
+      <c r="K6" s="3">
+        <f>SUM(K2:K5)</f>
+        <v/>
+      </c>
+      <c r="L6" s="3">
+        <f>SUM(L2:L5)</f>
+        <v/>
+      </c>
+      <c r="M6" s="3">
+        <f>SUM(M2:M5)</f>
+        <v/>
+      </c>
+      <c r="N6" s="3">
+        <f>SUM(N2:N5)</f>
+        <v/>
+      </c>
+      <c r="O6" s="3">
+        <f>SUM(O2:O5)</f>
+        <v/>
+      </c>
+      <c r="P6" s="3">
+        <f>SUM(P2:P5)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="3">
+        <f>SUM(Q2:Q5)</f>
+        <v/>
+      </c>
+      <c r="R6" s="3">
+        <f>SUM(R2:R5)</f>
+        <v/>
+      </c>
+      <c r="S6" s="3">
+        <f>SUM(S2:S5)</f>
+        <v/>
+      </c>
+      <c r="T6" s="3">
+        <f>SUM(T2:T5)</f>
+        <v/>
+      </c>
+      <c r="U6" s="3">
+        <f>SUM(U2:U5)</f>
+        <v/>
+      </c>
+      <c r="W6" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="AB6" s="4" t="n">
+      <c r="AB6" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="AG6" s="4" t="n">
+      <c r="AG6" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="AL6" s="4" t="n">
+      <c r="AL6" s="5" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="7">
-      <c r="W7" s="4" t="n">
+      <c r="W7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="AB7" s="4" t="n">
+      <c r="AB7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="AG7" s="4" t="n">
+      <c r="AG7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="AL7" s="4" t="n">
+      <c r="AL7" s="5" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="8">
-      <c r="W8" s="4" t="n">
+      <c r="W8" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="AB8" s="4" t="n">
+      <c r="AB8" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="AG8" s="4" t="n">
+      <c r="AG8" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="AL8" s="4" t="n">
+      <c r="AL8" s="5" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="9">
-      <c r="W9" s="4" t="n">
+      <c r="W9" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="AB9" s="4" t="n">
+      <c r="AB9" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="AG9" s="4" t="n">
+      <c r="AG9" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="AL9" s="4" t="n">
+      <c r="AL9" s="5" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="10">
-      <c r="W10" s="4" t="n">
+      <c r="W10" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="AB10" s="4" t="n">
+      <c r="AB10" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="AG10" s="4" t="n">
+      <c r="AG10" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="AL10" s="4" t="n">
+      <c r="AL10" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="11">
-      <c r="W11" s="4" t="n">
+      <c r="W11" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="AB11" s="4" t="n">
+      <c r="AB11" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="AG11" s="4" t="n">
+      <c r="AG11" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="AL11" s="4" t="n">
+      <c r="AL11" s="5" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="12">
-      <c r="W12" s="4" t="n">
+      <c r="W12" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="AB12" s="4" t="n">
+      <c r="AB12" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="AG12" s="4" t="n">
+      <c r="AG12" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="AL12" s="4" t="n">
+      <c r="AL12" s="5" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="13">
-      <c r="W13" s="4" t="n">
+      <c r="W13" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="AB13" s="4" t="n">
+      <c r="AB13" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="AG13" s="4" t="n">
+      <c r="AG13" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="AL13" s="4" t="n">
+      <c r="AL13" s="5" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="14">
-      <c r="W14" s="4" t="n">
+      <c r="W14" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="AB14" s="4" t="n">
+      <c r="AB14" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="AG14" s="4" t="n">
+      <c r="AG14" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="AL14" s="4" t="n">
+      <c r="AL14" s="5" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="15">
-      <c r="W15" s="4" t="n">
+      <c r="W15" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="AB15" s="4" t="n">
+      <c r="AB15" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="AG15" s="4" t="n">
+      <c r="AG15" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="AL15" s="4" t="n">
+      <c r="AL15" s="5" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="16">
-      <c r="W16" s="4" t="n">
+      <c r="W16" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="AB16" s="4" t="n">
+      <c r="AB16" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="AG16" s="4" t="n">
+      <c r="AG16" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="AL16" s="4" t="n">
+      <c r="AL16" s="5" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="17">
-      <c r="W17" s="4" t="n">
+      <c r="W17" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="AB17" s="4" t="n">
+      <c r="AB17" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="AG17" s="4" t="n">
+      <c r="AG17" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="AL17" s="4" t="n">
+      <c r="AL17" s="5" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="18">
-      <c r="W18" s="4" t="n">
+      <c r="W18" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="AB18" s="4" t="n">
+      <c r="AB18" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="AG18" s="4" t="n">
+      <c r="AG18" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="AL18" s="4" t="n">
+      <c r="AL18" s="5" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="19">
-      <c r="W19" s="4" t="n">
+      <c r="W19" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="AB19" s="4" t="n">
+      <c r="AB19" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="AG19" s="4" t="n">
+      <c r="AG19" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="AL19" s="4" t="n">
+      <c r="AL19" s="5" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="20">
-      <c r="W20" s="4" t="n">
+      <c r="W20" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="AB20" s="4" t="n">
+      <c r="AB20" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="AG20" s="4" t="n">
+      <c r="AG20" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="AL20" s="4" t="n">
+      <c r="AL20" s="5" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="21">
-      <c r="W21" s="4" t="n">
+      <c r="W21" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="AB21" s="4" t="n">
+      <c r="AB21" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="AG21" s="4" t="n">
+      <c r="AG21" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="AL21" s="4" t="n">
+      <c r="AL21" s="5" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="22">
-      <c r="W22" s="4" t="n">
+      <c r="W22" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="AB22" s="4" t="n">
+      <c r="AB22" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="AG22" s="4" t="n">
+      <c r="AG22" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="AL22" s="4" t="n">
+      <c r="AL22" s="5" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="23">
-      <c r="W23" s="4" t="n">
+      <c r="W23" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="AB23" s="4" t="n">
+      <c r="AB23" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="AG23" s="4" t="n">
+      <c r="AG23" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="AL23" s="4" t="n">
+      <c r="AL23" s="5" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="24">
-      <c r="W24" s="4" t="n">
+      <c r="W24" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="AB24" s="4" t="n">
+      <c r="AB24" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="AG24" s="4" t="n">
+      <c r="AG24" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="AL24" s="4" t="n">
+      <c r="AL24" s="5" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="25">
-      <c r="W25" s="4" t="n">
+      <c r="W25" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="AB25" s="4" t="n">
+      <c r="AB25" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="AG25" s="4" t="n">
+      <c r="AG25" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="AL25" s="4" t="n">
+      <c r="AL25" s="5" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="26">
-      <c r="W26" s="4" t="n">
+      <c r="W26" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="AB26" s="4" t="n">
+      <c r="AB26" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="AG26" s="4" t="n">
+      <c r="AG26" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="AL26" s="4" t="n">
+      <c r="AL26" s="5" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="27">
-      <c r="W27" s="4" t="n">
+      <c r="W27" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="AB27" s="4" t="n">
+      <c r="AB27" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="AG27" s="4" t="n">
+      <c r="AG27" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="AL27" s="4" t="n">
+      <c r="AL27" s="5" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="28">
-      <c r="W28" s="4" t="n">
+      <c r="W28" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="AB28" s="4" t="n">
+      <c r="AB28" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="AG28" s="4" t="n">
+      <c r="AG28" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="AL28" s="4" t="n">
+      <c r="AL28" s="5" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="29">
-      <c r="W29" s="4" t="n">
+      <c r="W29" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="AB29" s="4" t="n">
+      <c r="AB29" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="AG29" s="4" t="n">
+      <c r="AG29" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="AL29" s="4" t="n">
+      <c r="AL29" s="5" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="30">
-      <c r="W30" s="4" t="n">
+      <c r="W30" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="AB30" s="4" t="n">
+      <c r="AB30" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="AG30" s="4" t="n">
+      <c r="AG30" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="AL30" s="4" t="n">
+      <c r="AL30" s="5" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="31">
-      <c r="W31" s="4" t="n">
+      <c r="W31" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="AB31" s="4" t="n">
+      <c r="AB31" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="AG31" s="4" t="n">
+      <c r="AG31" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="AL31" s="4" t="n">
+      <c r="AL31" s="5" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="32">
-      <c r="W32" s="4" t="n">
+      <c r="W32" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="AB32" s="4" t="n">
+      <c r="AB32" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="AG32" s="4" t="n">
+      <c r="AG32" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="AL32" s="4" t="n">
+      <c r="AL32" s="5" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="33">
-      <c r="W33" s="4" t="n">
+      <c r="W33" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="AB33" s="4" t="n">
+      <c r="AB33" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="AG33" s="4" t="n">
+      <c r="AG33" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="AL33" s="4" t="n">
+      <c r="AL33" s="5" t="n">
         <v>31</v>
       </c>
     </row>

</xml_diff>